<commit_message>
Add thick FA|C&E divider and auto highest-possible total on each slip
</commit_message>
<xml_diff>
--- a/grading_rubric_A4.xlsx
+++ b/grading_rubric_A4.xlsx
@@ -99,7 +99,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -132,6 +132,19 @@
       </bottom>
     </border>
     <border>
+      <left style="thick">
+        <color rgb="00404040"/>
+      </left>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00404040"/>
+      </left>
+    </border>
+    <border>
       <bottom style="dashed">
         <color rgb="007F7F7F"/>
       </bottom>
@@ -140,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -171,10 +184,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -183,7 +202,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
@@ -839,7 +858,7 @@
       <c r="D2" s="13" t="n"/>
       <c r="E2" s="13" t="n"/>
       <c r="F2" s="13" t="n"/>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" s="14" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
@@ -857,298 +876,297 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="14" t="n">
+      <c r="A3" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="16">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C3" s="15">
+      <c r="C3" s="16">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="16">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E3" s="15">
+      <c r="E3" s="16">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F3" s="15">
+      <c r="F3" s="16">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G3" s="15">
+      <c r="G3" s="17">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H3" s="15">
+      <c r="H3" s="16">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I3" s="15">
+      <c r="I3" s="16">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J3" s="15">
+      <c r="J3" s="16">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K3" s="15">
+      <c r="K3" s="16">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L3" s="15">
+      <c r="L3" s="16">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M3" s="15">
+      <c r="M3" s="16">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N3" s="7" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="14" t="n">
+      <c r="A4" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="16">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C4" s="15">
+      <c r="C4" s="16">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="16">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="16">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F4" s="15">
+      <c r="F4" s="16">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G4" s="15">
+      <c r="G4" s="17">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H4" s="15">
+      <c r="H4" s="16">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I4" s="15">
+      <c r="I4" s="16">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="16">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K4" s="15">
+      <c r="K4" s="16">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L4" s="15">
+      <c r="L4" s="16">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M4" s="15">
+      <c r="M4" s="16">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N4" s="7" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="14" t="n">
+      <c r="A5" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="16">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C5" s="15">
+      <c r="C5" s="16">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D5" s="15">
+      <c r="D5" s="16">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="16">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="16">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="17">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H5" s="15">
+      <c r="H5" s="16">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I5" s="15">
+      <c r="I5" s="16">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J5" s="15">
+      <c r="J5" s="16">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K5" s="15">
+      <c r="K5" s="16">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L5" s="15">
+      <c r="L5" s="16">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M5" s="15">
+      <c r="M5" s="16">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N5" s="7" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="14" t="n">
+      <c r="A6" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="16">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C6" s="15">
+      <c r="C6" s="16">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="16">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="16">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="16">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="17">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H6" s="15">
+      <c r="H6" s="16">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I6" s="15">
+      <c r="I6" s="16">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="16">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K6" s="15">
+      <c r="K6" s="16">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L6" s="15">
+      <c r="L6" s="16">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M6" s="15">
+      <c r="M6" s="16">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N6" s="7" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="14" t="n">
+      <c r="A7" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="16">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="16">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="16">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="16">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="16">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="17">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H7" s="15">
+      <c r="H7" s="16">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I7" s="15">
+      <c r="I7" s="16">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J7" s="15">
+      <c r="J7" s="16">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K7" s="15">
+      <c r="K7" s="16">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L7" s="15">
+      <c r="L7" s="16">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M7" s="15">
+      <c r="M7" s="16">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N7" s="7" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL SCORE  →</t>
-        </is>
-      </c>
-      <c r="N8" s="17" t="n"/>
+      <c r="A8" s="18">
+        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
+        <v/>
+      </c>
+      <c r="N8" s="19" t="n"/>
     </row>
     <row r="9" ht="9" customHeight="1">
-      <c r="A9" s="18" t="n"/>
-      <c r="B9" s="18" t="n"/>
-      <c r="C9" s="18" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="18" t="n"/>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="18" t="n"/>
-      <c r="J9" s="18" t="n"/>
-      <c r="K9" s="18" t="n"/>
-      <c r="L9" s="18" t="n"/>
-      <c r="M9" s="18" t="n"/>
-      <c r="N9" s="18" t="n"/>
+      <c r="A9" s="20" t="n"/>
+      <c r="B9" s="20" t="n"/>
+      <c r="C9" s="20" t="n"/>
+      <c r="D9" s="20" t="n"/>
+      <c r="E9" s="20" t="n"/>
+      <c r="F9" s="20" t="n"/>
+      <c r="G9" s="20" t="n"/>
+      <c r="H9" s="20" t="n"/>
+      <c r="I9" s="20" t="n"/>
+      <c r="J9" s="20" t="n"/>
+      <c r="K9" s="20" t="n"/>
+      <c r="L9" s="20" t="n"/>
+      <c r="M9" s="20" t="n"/>
+      <c r="N9" s="20" t="n"/>
     </row>
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="10">
@@ -1184,7 +1202,7 @@
       <c r="D11" s="13" t="n"/>
       <c r="E11" s="13" t="n"/>
       <c r="F11" s="13" t="n"/>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="G11" s="14" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
@@ -1202,298 +1220,297 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="14" t="n">
+      <c r="A12" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="16">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="16">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="17">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H12" s="15">
+      <c r="H12" s="16">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I12" s="15">
+      <c r="I12" s="16">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J12" s="15">
+      <c r="J12" s="16">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K12" s="15">
+      <c r="K12" s="16">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L12" s="15">
+      <c r="L12" s="16">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M12" s="15">
+      <c r="M12" s="16">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N12" s="7" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="14" t="n">
+      <c r="A13" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="15">
+      <c r="B13" s="16">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C13" s="15">
+      <c r="C13" s="16">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="16">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="16">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="16">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G13" s="15">
+      <c r="G13" s="17">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H13" s="15">
+      <c r="H13" s="16">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I13" s="15">
+      <c r="I13" s="16">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J13" s="15">
+      <c r="J13" s="16">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K13" s="15">
+      <c r="K13" s="16">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L13" s="15">
+      <c r="L13" s="16">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M13" s="15">
+      <c r="M13" s="16">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N13" s="7" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="14" t="n">
+      <c r="A14" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="15">
+      <c r="B14" s="16">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="16">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="16">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="16">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="16">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G14" s="15">
+      <c r="G14" s="17">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H14" s="15">
+      <c r="H14" s="16">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I14" s="15">
+      <c r="I14" s="16">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J14" s="15">
+      <c r="J14" s="16">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K14" s="15">
+      <c r="K14" s="16">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L14" s="15">
+      <c r="L14" s="16">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M14" s="15">
+      <c r="M14" s="16">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N14" s="7" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="14" t="n">
+      <c r="A15" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="16">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C15" s="15">
+      <c r="C15" s="16">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="16">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="16">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="16">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="17">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="16">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I15" s="15">
+      <c r="I15" s="16">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J15" s="15">
+      <c r="J15" s="16">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K15" s="15">
+      <c r="K15" s="16">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L15" s="15">
+      <c r="L15" s="16">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M15" s="15">
+      <c r="M15" s="16">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N15" s="7" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="14" t="n">
+      <c r="A16" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="16">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="16">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="16">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="16">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="16">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="17">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="16">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I16" s="15">
+      <c r="I16" s="16">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J16" s="15">
+      <c r="J16" s="16">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K16" s="15">
+      <c r="K16" s="16">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L16" s="15">
+      <c r="L16" s="16">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M16" s="15">
+      <c r="M16" s="16">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N16" s="7" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL SCORE  →</t>
-        </is>
-      </c>
-      <c r="N17" s="17" t="n"/>
+      <c r="A17" s="18">
+        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
+        <v/>
+      </c>
+      <c r="N17" s="19" t="n"/>
     </row>
     <row r="18" ht="9" customHeight="1">
-      <c r="A18" s="18" t="n"/>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
-      <c r="F18" s="18" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="18" t="n"/>
-      <c r="I18" s="18" t="n"/>
-      <c r="J18" s="18" t="n"/>
-      <c r="K18" s="18" t="n"/>
-      <c r="L18" s="18" t="n"/>
-      <c r="M18" s="18" t="n"/>
-      <c r="N18" s="18" t="n"/>
+      <c r="A18" s="20" t="n"/>
+      <c r="B18" s="20" t="n"/>
+      <c r="C18" s="20" t="n"/>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="20" t="n"/>
+      <c r="F18" s="20" t="n"/>
+      <c r="G18" s="20" t="n"/>
+      <c r="H18" s="20" t="n"/>
+      <c r="I18" s="20" t="n"/>
+      <c r="J18" s="20" t="n"/>
+      <c r="K18" s="20" t="n"/>
+      <c r="L18" s="20" t="n"/>
+      <c r="M18" s="20" t="n"/>
+      <c r="N18" s="20" t="n"/>
     </row>
     <row r="19" ht="19" customHeight="1">
       <c r="A19" s="10">
@@ -1529,7 +1546,7 @@
       <c r="D20" s="13" t="n"/>
       <c r="E20" s="13" t="n"/>
       <c r="F20" s="13" t="n"/>
-      <c r="G20" s="12" t="inlineStr">
+      <c r="G20" s="14" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
@@ -1547,298 +1564,297 @@
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="14" t="n">
+      <c r="A21" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B21" s="15">
+      <c r="B21" s="16">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C21" s="15">
+      <c r="C21" s="16">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="16">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="16">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F21" s="15">
+      <c r="F21" s="16">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G21" s="15">
+      <c r="G21" s="17">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H21" s="15">
+      <c r="H21" s="16">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I21" s="15">
+      <c r="I21" s="16">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J21" s="15">
+      <c r="J21" s="16">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K21" s="15">
+      <c r="K21" s="16">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L21" s="15">
+      <c r="L21" s="16">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M21" s="15">
+      <c r="M21" s="16">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N21" s="7" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="14" t="n">
+      <c r="A22" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="16">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C22" s="15">
+      <c r="C22" s="16">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="16">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="16">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="16">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G22" s="15">
+      <c r="G22" s="17">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H22" s="15">
+      <c r="H22" s="16">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I22" s="15">
+      <c r="I22" s="16">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J22" s="15">
+      <c r="J22" s="16">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K22" s="15">
+      <c r="K22" s="16">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L22" s="15">
+      <c r="L22" s="16">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M22" s="15">
+      <c r="M22" s="16">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N22" s="7" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="14" t="n">
+      <c r="A23" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="16">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C23" s="15">
+      <c r="C23" s="16">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="16">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="16">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="16">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G23" s="15">
+      <c r="G23" s="17">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H23" s="15">
+      <c r="H23" s="16">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I23" s="15">
+      <c r="I23" s="16">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J23" s="15">
+      <c r="J23" s="16">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K23" s="15">
+      <c r="K23" s="16">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L23" s="15">
+      <c r="L23" s="16">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M23" s="15">
+      <c r="M23" s="16">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N23" s="7" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="14" t="n">
+      <c r="A24" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="16">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C24" s="15">
+      <c r="C24" s="16">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="16">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="16">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F24" s="15">
+      <c r="F24" s="16">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G24" s="15">
+      <c r="G24" s="17">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H24" s="15">
+      <c r="H24" s="16">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I24" s="15">
+      <c r="I24" s="16">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J24" s="15">
+      <c r="J24" s="16">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K24" s="15">
+      <c r="K24" s="16">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L24" s="15">
+      <c r="L24" s="16">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M24" s="15">
+      <c r="M24" s="16">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N24" s="7" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="14" t="n">
+      <c r="A25" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B25" s="15">
+      <c r="B25" s="16">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C25" s="15">
+      <c r="C25" s="16">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D25" s="15">
+      <c r="D25" s="16">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="16">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F25" s="15">
+      <c r="F25" s="16">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G25" s="15">
+      <c r="G25" s="17">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H25" s="15">
+      <c r="H25" s="16">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I25" s="15">
+      <c r="I25" s="16">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J25" s="15">
+      <c r="J25" s="16">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K25" s="15">
+      <c r="K25" s="16">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L25" s="15">
+      <c r="L25" s="16">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M25" s="15">
+      <c r="M25" s="16">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N25" s="7" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL SCORE  →</t>
-        </is>
-      </c>
-      <c r="N26" s="17" t="n"/>
+      <c r="A26" s="18">
+        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
+        <v/>
+      </c>
+      <c r="N26" s="19" t="n"/>
     </row>
     <row r="27" ht="9" customHeight="1">
-      <c r="A27" s="18" t="n"/>
-      <c r="B27" s="18" t="n"/>
-      <c r="C27" s="18" t="n"/>
-      <c r="D27" s="18" t="n"/>
-      <c r="E27" s="18" t="n"/>
-      <c r="F27" s="18" t="n"/>
-      <c r="G27" s="18" t="n"/>
-      <c r="H27" s="18" t="n"/>
-      <c r="I27" s="18" t="n"/>
-      <c r="J27" s="18" t="n"/>
-      <c r="K27" s="18" t="n"/>
-      <c r="L27" s="18" t="n"/>
-      <c r="M27" s="18" t="n"/>
-      <c r="N27" s="18" t="n"/>
+      <c r="A27" s="20" t="n"/>
+      <c r="B27" s="20" t="n"/>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="n"/>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="20" t="n"/>
+      <c r="G27" s="20" t="n"/>
+      <c r="H27" s="20" t="n"/>
+      <c r="I27" s="20" t="n"/>
+      <c r="J27" s="20" t="n"/>
+      <c r="K27" s="20" t="n"/>
+      <c r="L27" s="20" t="n"/>
+      <c r="M27" s="20" t="n"/>
+      <c r="N27" s="20" t="n"/>
     </row>
     <row r="28" ht="19" customHeight="1">
       <c r="A28" s="10">
@@ -1874,7 +1890,7 @@
       <c r="D29" s="13" t="n"/>
       <c r="E29" s="13" t="n"/>
       <c r="F29" s="13" t="n"/>
-      <c r="G29" s="12" t="inlineStr">
+      <c r="G29" s="14" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
@@ -1892,298 +1908,297 @@
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="14" t="n">
+      <c r="A30" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B30" s="15">
+      <c r="B30" s="16">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C30" s="15">
+      <c r="C30" s="16">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="16">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E30" s="15">
+      <c r="E30" s="16">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F30" s="15">
+      <c r="F30" s="16">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G30" s="15">
+      <c r="G30" s="17">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H30" s="15">
+      <c r="H30" s="16">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I30" s="15">
+      <c r="I30" s="16">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J30" s="15">
+      <c r="J30" s="16">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K30" s="15">
+      <c r="K30" s="16">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L30" s="15">
+      <c r="L30" s="16">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M30" s="15">
+      <c r="M30" s="16">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N30" s="7" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="14" t="n">
+      <c r="A31" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B31" s="15">
+      <c r="B31" s="16">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C31" s="15">
+      <c r="C31" s="16">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="16">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E31" s="15">
+      <c r="E31" s="16">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F31" s="15">
+      <c r="F31" s="16">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G31" s="15">
+      <c r="G31" s="17">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H31" s="15">
+      <c r="H31" s="16">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I31" s="15">
+      <c r="I31" s="16">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J31" s="15">
+      <c r="J31" s="16">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K31" s="15">
+      <c r="K31" s="16">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L31" s="15">
+      <c r="L31" s="16">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M31" s="15">
+      <c r="M31" s="16">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N31" s="7" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="14" t="n">
+      <c r="A32" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B32" s="15">
+      <c r="B32" s="16">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C32" s="15">
+      <c r="C32" s="16">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="16">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E32" s="15">
+      <c r="E32" s="16">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F32" s="15">
+      <c r="F32" s="16">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G32" s="15">
+      <c r="G32" s="17">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H32" s="15">
+      <c r="H32" s="16">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I32" s="15">
+      <c r="I32" s="16">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J32" s="15">
+      <c r="J32" s="16">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K32" s="15">
+      <c r="K32" s="16">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L32" s="15">
+      <c r="L32" s="16">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M32" s="15">
+      <c r="M32" s="16">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N32" s="7" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="14" t="n">
+      <c r="A33" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B33" s="15">
+      <c r="B33" s="16">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C33" s="15">
+      <c r="C33" s="16">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D33" s="15">
+      <c r="D33" s="16">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E33" s="15">
+      <c r="E33" s="16">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F33" s="15">
+      <c r="F33" s="16">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G33" s="15">
+      <c r="G33" s="17">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H33" s="15">
+      <c r="H33" s="16">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I33" s="15">
+      <c r="I33" s="16">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J33" s="15">
+      <c r="J33" s="16">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K33" s="15">
+      <c r="K33" s="16">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L33" s="15">
+      <c r="L33" s="16">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M33" s="15">
+      <c r="M33" s="16">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N33" s="7" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="14" t="n">
+      <c r="A34" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B34" s="15">
+      <c r="B34" s="16">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C34" s="15">
+      <c r="C34" s="16">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D34" s="15">
+      <c r="D34" s="16">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E34" s="15">
+      <c r="E34" s="16">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F34" s="15">
+      <c r="F34" s="16">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G34" s="15">
+      <c r="G34" s="17">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H34" s="15">
+      <c r="H34" s="16">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I34" s="15">
+      <c r="I34" s="16">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J34" s="15">
+      <c r="J34" s="16">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K34" s="15">
+      <c r="K34" s="16">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L34" s="15">
+      <c r="L34" s="16">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M34" s="15">
+      <c r="M34" s="16">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N34" s="7" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL SCORE  →</t>
-        </is>
-      </c>
-      <c r="N35" s="17" t="n"/>
+      <c r="A35" s="18">
+        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
+        <v/>
+      </c>
+      <c r="N35" s="19" t="n"/>
     </row>
     <row r="36" ht="9" customHeight="1">
-      <c r="A36" s="18" t="n"/>
-      <c r="B36" s="18" t="n"/>
-      <c r="C36" s="18" t="n"/>
-      <c r="D36" s="18" t="n"/>
-      <c r="E36" s="18" t="n"/>
-      <c r="F36" s="18" t="n"/>
-      <c r="G36" s="18" t="n"/>
-      <c r="H36" s="18" t="n"/>
-      <c r="I36" s="18" t="n"/>
-      <c r="J36" s="18" t="n"/>
-      <c r="K36" s="18" t="n"/>
-      <c r="L36" s="18" t="n"/>
-      <c r="M36" s="18" t="n"/>
-      <c r="N36" s="18" t="n"/>
+      <c r="A36" s="20" t="n"/>
+      <c r="B36" s="20" t="n"/>
+      <c r="C36" s="20" t="n"/>
+      <c r="D36" s="20" t="n"/>
+      <c r="E36" s="20" t="n"/>
+      <c r="F36" s="20" t="n"/>
+      <c r="G36" s="20" t="n"/>
+      <c r="H36" s="20" t="n"/>
+      <c r="I36" s="20" t="n"/>
+      <c r="J36" s="20" t="n"/>
+      <c r="K36" s="20" t="n"/>
+      <c r="L36" s="20" t="n"/>
+      <c r="M36" s="20" t="n"/>
+      <c r="N36" s="20" t="n"/>
     </row>
     <row r="37" ht="19" customHeight="1">
       <c r="A37" s="10">
@@ -2219,7 +2234,7 @@
       <c r="D38" s="13" t="n"/>
       <c r="E38" s="13" t="n"/>
       <c r="F38" s="13" t="n"/>
-      <c r="G38" s="12" t="inlineStr">
+      <c r="G38" s="14" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
@@ -2237,298 +2252,297 @@
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="14" t="n">
+      <c r="A39" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B39" s="15">
+      <c r="B39" s="16">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C39" s="15">
+      <c r="C39" s="16">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D39" s="15">
+      <c r="D39" s="16">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E39" s="15">
+      <c r="E39" s="16">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F39" s="15">
+      <c r="F39" s="16">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G39" s="15">
+      <c r="G39" s="17">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H39" s="15">
+      <c r="H39" s="16">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I39" s="15">
+      <c r="I39" s="16">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J39" s="15">
+      <c r="J39" s="16">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K39" s="15">
+      <c r="K39" s="16">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L39" s="15">
+      <c r="L39" s="16">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M39" s="15">
+      <c r="M39" s="16">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N39" s="7" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="14" t="n">
+      <c r="A40" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B40" s="15">
+      <c r="B40" s="16">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C40" s="15">
+      <c r="C40" s="16">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D40" s="15">
+      <c r="D40" s="16">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E40" s="15">
+      <c r="E40" s="16">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F40" s="15">
+      <c r="F40" s="16">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G40" s="15">
+      <c r="G40" s="17">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H40" s="15">
+      <c r="H40" s="16">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I40" s="15">
+      <c r="I40" s="16">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J40" s="15">
+      <c r="J40" s="16">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K40" s="15">
+      <c r="K40" s="16">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L40" s="15">
+      <c r="L40" s="16">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M40" s="15">
+      <c r="M40" s="16">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N40" s="7" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="14" t="n">
+      <c r="A41" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="15">
+      <c r="B41" s="16">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C41" s="15">
+      <c r="C41" s="16">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D41" s="15">
+      <c r="D41" s="16">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E41" s="15">
+      <c r="E41" s="16">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F41" s="15">
+      <c r="F41" s="16">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G41" s="15">
+      <c r="G41" s="17">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H41" s="15">
+      <c r="H41" s="16">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I41" s="15">
+      <c r="I41" s="16">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J41" s="15">
+      <c r="J41" s="16">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K41" s="15">
+      <c r="K41" s="16">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L41" s="15">
+      <c r="L41" s="16">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M41" s="15">
+      <c r="M41" s="16">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N41" s="7" t="n"/>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="14" t="n">
+      <c r="A42" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B42" s="15">
+      <c r="B42" s="16">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C42" s="15">
+      <c r="C42" s="16">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D42" s="15">
+      <c r="D42" s="16">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E42" s="15">
+      <c r="E42" s="16">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F42" s="15">
+      <c r="F42" s="16">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G42" s="15">
+      <c r="G42" s="17">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H42" s="15">
+      <c r="H42" s="16">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I42" s="15">
+      <c r="I42" s="16">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J42" s="15">
+      <c r="J42" s="16">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K42" s="15">
+      <c r="K42" s="16">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L42" s="15">
+      <c r="L42" s="16">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M42" s="15">
+      <c r="M42" s="16">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N42" s="7" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="14" t="n">
+      <c r="A43" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B43" s="15">
+      <c r="B43" s="16">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C43" s="15">
+      <c r="C43" s="16">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D43" s="15">
+      <c r="D43" s="16">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E43" s="15">
+      <c r="E43" s="16">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F43" s="15">
+      <c r="F43" s="16">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G43" s="15">
+      <c r="G43" s="17">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H43" s="15">
+      <c r="H43" s="16">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I43" s="15">
+      <c r="I43" s="16">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J43" s="15">
+      <c r="J43" s="16">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K43" s="15">
+      <c r="K43" s="16">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L43" s="15">
+      <c r="L43" s="16">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M43" s="15">
+      <c r="M43" s="16">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N43" s="7" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL SCORE  →</t>
-        </is>
-      </c>
-      <c r="N44" s="17" t="n"/>
+      <c r="A44" s="18">
+        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
+        <v/>
+      </c>
+      <c r="N44" s="19" t="n"/>
     </row>
     <row r="45" ht="9" customHeight="1">
-      <c r="A45" s="18" t="n"/>
-      <c r="B45" s="18" t="n"/>
-      <c r="C45" s="18" t="n"/>
-      <c r="D45" s="18" t="n"/>
-      <c r="E45" s="18" t="n"/>
-      <c r="F45" s="18" t="n"/>
-      <c r="G45" s="18" t="n"/>
-      <c r="H45" s="18" t="n"/>
-      <c r="I45" s="18" t="n"/>
-      <c r="J45" s="18" t="n"/>
-      <c r="K45" s="18" t="n"/>
-      <c r="L45" s="18" t="n"/>
-      <c r="M45" s="18" t="n"/>
-      <c r="N45" s="18" t="n"/>
+      <c r="A45" s="20" t="n"/>
+      <c r="B45" s="20" t="n"/>
+      <c r="C45" s="20" t="n"/>
+      <c r="D45" s="20" t="n"/>
+      <c r="E45" s="20" t="n"/>
+      <c r="F45" s="20" t="n"/>
+      <c r="G45" s="20" t="n"/>
+      <c r="H45" s="20" t="n"/>
+      <c r="I45" s="20" t="n"/>
+      <c r="J45" s="20" t="n"/>
+      <c r="K45" s="20" t="n"/>
+      <c r="L45" s="20" t="n"/>
+      <c r="M45" s="20" t="n"/>
+      <c r="N45" s="20" t="n"/>
     </row>
     <row r="46" ht="19" customHeight="1">
       <c r="A46" s="10">
@@ -2564,7 +2578,7 @@
       <c r="D47" s="13" t="n"/>
       <c r="E47" s="13" t="n"/>
       <c r="F47" s="13" t="n"/>
-      <c r="G47" s="12" t="inlineStr">
+      <c r="G47" s="14" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
@@ -2582,282 +2596,281 @@
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="14" t="n">
+      <c r="A48" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B48" s="15">
+      <c r="B48" s="16">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C48" s="15">
+      <c r="C48" s="16">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D48" s="15">
+      <c r="D48" s="16">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E48" s="15">
+      <c r="E48" s="16">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F48" s="15">
+      <c r="F48" s="16">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G48" s="15">
+      <c r="G48" s="17">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H48" s="15">
+      <c r="H48" s="16">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I48" s="15">
+      <c r="I48" s="16">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J48" s="15">
+      <c r="J48" s="16">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K48" s="15">
+      <c r="K48" s="16">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L48" s="15">
+      <c r="L48" s="16">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M48" s="15">
+      <c r="M48" s="16">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N48" s="7" t="n"/>
     </row>
     <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="14" t="n">
+      <c r="A49" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B49" s="15">
+      <c r="B49" s="16">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C49" s="15">
+      <c r="C49" s="16">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D49" s="15">
+      <c r="D49" s="16">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E49" s="15">
+      <c r="E49" s="16">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F49" s="15">
+      <c r="F49" s="16">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G49" s="15">
+      <c r="G49" s="17">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H49" s="15">
+      <c r="H49" s="16">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I49" s="15">
+      <c r="I49" s="16">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J49" s="15">
+      <c r="J49" s="16">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K49" s="15">
+      <c r="K49" s="16">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L49" s="15">
+      <c r="L49" s="16">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M49" s="15">
+      <c r="M49" s="16">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N49" s="7" t="n"/>
     </row>
     <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="14" t="n">
+      <c r="A50" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B50" s="15">
+      <c r="B50" s="16">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C50" s="15">
+      <c r="C50" s="16">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D50" s="15">
+      <c r="D50" s="16">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E50" s="15">
+      <c r="E50" s="16">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F50" s="15">
+      <c r="F50" s="16">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G50" s="15">
+      <c r="G50" s="17">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H50" s="15">
+      <c r="H50" s="16">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I50" s="15">
+      <c r="I50" s="16">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J50" s="15">
+      <c r="J50" s="16">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K50" s="15">
+      <c r="K50" s="16">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L50" s="15">
+      <c r="L50" s="16">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M50" s="15">
+      <c r="M50" s="16">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N50" s="7" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="14" t="n">
+      <c r="A51" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B51" s="15">
+      <c r="B51" s="16">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C51" s="15">
+      <c r="C51" s="16">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D51" s="15">
+      <c r="D51" s="16">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E51" s="15">
+      <c r="E51" s="16">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F51" s="15">
+      <c r="F51" s="16">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G51" s="15">
+      <c r="G51" s="17">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H51" s="15">
+      <c r="H51" s="16">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I51" s="15">
+      <c r="I51" s="16">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J51" s="15">
+      <c r="J51" s="16">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K51" s="15">
+      <c r="K51" s="16">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L51" s="15">
+      <c r="L51" s="16">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M51" s="15">
+      <c r="M51" s="16">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N51" s="7" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="14" t="n">
+      <c r="A52" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B52" s="15">
+      <c r="B52" s="16">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C52" s="15">
+      <c r="C52" s="16">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D52" s="15">
+      <c r="D52" s="16">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E52" s="15">
+      <c r="E52" s="16">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F52" s="15">
+      <c r="F52" s="16">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G52" s="15">
+      <c r="G52" s="17">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H52" s="15">
+      <c r="H52" s="16">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I52" s="15">
+      <c r="I52" s="16">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J52" s="15">
+      <c r="J52" s="16">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K52" s="15">
+      <c r="K52" s="16">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L52" s="15">
+      <c r="L52" s="16">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M52" s="15">
+      <c r="M52" s="16">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N52" s="7" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL SCORE  →</t>
-        </is>
-      </c>
-      <c r="N53" s="17" t="n"/>
+      <c r="A53" s="18">
+        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
+        <v/>
+      </c>
+      <c r="N53" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="24">
@@ -2920,364 +2933,364 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>What each dimension measures</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n"/>
+      <c r="B4" s="22" t="n"/>
     </row>
     <row r="5" ht="33" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>Final Answer  —  Did you land the correct result, properly expressed? Correct value(s), units, and significant figures. This is the ONLY place units and sig figs are judged.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>Concept &amp; Execution  —  Do you understand the physics and can you carry it out? Right principle/equation (concept) + correct substitution, algebra, and method (execution) + clear, ordered, labeled work (communication). Graded on process, using Error-Carried-Forward.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Grading rules (apply before scoring)</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n"/>
+      <c r="B8" s="22" t="n"/>
     </row>
     <row r="9" ht="33" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>1.  Score each column on its own descriptor; never penalize the same flaw twice. Units/sig-fig issues affect only Final Answer.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>2.  Error-Carried-Forward (ECF): judge each step against the student's own prior results, not the answer key.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>3.  Consistency (default): the two columns should tell the same story — strong process usually accompanies a correct answer.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="33" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>4.  ECF override: if the ONLY defect is a single arithmetic/transcription slip and every later step is correct under ECF, score Concept &amp; Execution on process merit (it may reach the top band) even though the final answer is wrong.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>5.  Answer only / no work shown: score Final Answer on merit; Concept &amp; Execution = 0.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>6.  Blank: 0 / 0.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>TYPE A — Single-unknown (Total 5)</t>
         </is>
       </c>
-      <c r="B16" s="20" t="n"/>
+      <c r="B16" s="22" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>Final Answer (0–2)</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
-      <c r="A18" s="24" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B18" s="25" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>Correct value, correct units, appropriate significant figures.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>Correct value but units/sig figs wrong, OR a single arithmetic slip giving a near-correct value.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B20" s="25" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>Incorrect, or blank.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="22" t="inlineStr">
+      <c r="A21" s="24" t="inlineStr">
         <is>
           <t>Concept &amp; Execution (0–3)</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="25" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1">
-      <c r="A22" s="24" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B22" s="25" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>Correct principle/equation; substitution and algebra correct; work clear and complete.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B23" s="25" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>Correct principle; essentially right, with a minor execution slip or sparse-but-followable steps.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="26" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B24" s="25" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>Relevant concept present, but undermined by a wrong equation or a substantive execution error.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B25" s="25" t="inlineStr">
+      <c r="B25" s="27" t="inlineStr">
         <is>
           <t>Wrong concept, or no meaningful work.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>TYPE B — Multi-step / multi-unknown (Total 10)</t>
         </is>
       </c>
-      <c r="B27" s="20" t="n"/>
+      <c r="B27" s="22" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>Final Answer (0–4)</t>
         </is>
       </c>
-      <c r="B28" s="23" t="inlineStr">
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1">
-      <c r="A29" s="24" t="inlineStr">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B29" s="25" t="inlineStr">
+      <c r="B29" s="27" t="inlineStr">
         <is>
           <t>Every required final value correct, with correct units.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="24" t="inlineStr">
+      <c r="A30" s="26" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B30" s="25" t="inlineStr">
+      <c r="B30" s="27" t="inlineStr">
         <is>
           <t>All but one correct; the single miss is minor (units, sig figs, or one small slip).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="19" customHeight="1">
-      <c r="A31" s="24" t="inlineStr">
+      <c r="A31" s="26" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B31" s="25" t="inlineStr">
+      <c r="B31" s="27" t="inlineStr">
         <is>
           <t>Roughly half the values correct.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="24" t="inlineStr">
+      <c r="A32" s="26" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B32" s="25" t="inlineStr">
+      <c r="B32" s="27" t="inlineStr">
         <is>
           <t>One value correct, or most contain significant errors.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="24" t="inlineStr">
+      <c r="A33" s="26" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B33" s="25" t="inlineStr">
+      <c r="B33" s="27" t="inlineStr">
         <is>
           <t>No correct values, or blank.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="22" t="inlineStr">
+      <c r="A34" s="24" t="inlineStr">
         <is>
           <t>Concept &amp; Execution (0–6)</t>
         </is>
       </c>
-      <c r="B34" s="23" t="inlineStr">
+      <c r="B34" s="25" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="35" ht="34" customHeight="1">
-      <c r="A35" s="24" t="inlineStr">
+      <c r="A35" s="26" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B35" s="25" t="inlineStr">
+      <c r="B35" s="27" t="inlineStr">
         <is>
           <t>Correct principle at EVERY step; all substitution, algebra, and units correct (ECF); logically ordered, labeled, easy to follow.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="34" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
+      <c r="A36" s="26" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B36" s="25" t="inlineStr">
+      <c r="B36" s="27" t="inlineStr">
         <is>
           <t>Correct principles and method throughout; at most one trivial slip or slightly sparse justification — physics fully sound.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="34" customHeight="1">
-      <c r="A37" s="24" t="inlineStr">
+      <c r="A37" s="26" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B37" s="25" t="inlineStr">
+      <c r="B37" s="27" t="inlineStr">
         <is>
           <t>Correct approach on the main steps, but ONE real execution error or one wrong/missing equation; work still followable.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="34" customHeight="1">
-      <c r="A38" s="24" t="inlineStr">
+      <c r="A38" s="26" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B38" s="25" t="inlineStr">
+      <c r="B38" s="27" t="inlineStr">
         <is>
           <t>Correct on some steps, but a wrong principle on a major step and/or several execution errors; reasoning has gaps.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="19" customHeight="1">
-      <c r="A39" s="24" t="inlineStr">
+      <c r="A39" s="26" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B39" s="25" t="inlineStr">
+      <c r="B39" s="27" t="inlineStr">
         <is>
           <t>Mostly incorrect method; more than a token of correct physics but hard to follow.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="19" customHeight="1">
-      <c r="A40" s="24" t="inlineStr">
+      <c r="A40" s="26" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B40" s="25" t="inlineStr">
+      <c r="B40" s="27" t="inlineStr">
         <is>
           <t>Little relevant physics; fundamentally the wrong approach with only a token correct fragment.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="19" customHeight="1">
-      <c r="A41" s="24" t="inlineStr">
+      <c r="A41" s="26" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B41" s="25" t="inlineStr">
+      <c r="B41" s="27" t="inlineStr">
         <is>
           <t>No meaningful work, or blank.</t>
         </is>

</xml_diff>

<commit_message>
Add outer table border, slash-format score/total, per-problem max, and vertical signature block
</commit_message>
<xml_diff>
--- a/grading_rubric_A4.xlsx
+++ b/grading_rubric_A4.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +65,10 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
@@ -99,7 +103,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -145,6 +149,146 @@
       </left>
     </border>
     <border>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00404040"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thick">
+        <color rgb="00404040"/>
+      </left>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00404040"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00404040"/>
+      </left>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00404040"/>
+      </right>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00404040"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00404040"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00404040"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00404040"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00404040"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00404040"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="00404040"/>
+      </right>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="00404040"/>
+      </right>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="medium">
+        <color rgb="00404040"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00404040"/>
+      </bottom>
+    </border>
+    <border>
       <bottom style="dashed">
         <color rgb="007F7F7F"/>
       </bottom>
@@ -153,7 +297,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -180,14 +324,20 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,18 +346,27 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -219,7 +378,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -805,7 +964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N53"/>
+  <dimension ref="A1:P53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -821,7 +980,9 @@
     <col width="4.6" customWidth="1" min="11" max="11"/>
     <col width="4.6" customWidth="1" min="12" max="12"/>
     <col width="4.6" customWidth="1" min="13" max="13"/>
-    <col width="7.5" customWidth="1" min="14" max="14"/>
+    <col width="6.5" customWidth="1" min="14" max="14"/>
+    <col width="4.6" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="19" customHeight="1">
@@ -842,6 +1003,8 @@
       <c r="L1" s="11" t="n"/>
       <c r="M1" s="11" t="n"/>
       <c r="N1" s="11" t="n"/>
+      <c r="O1" s="11" t="n"/>
+      <c r="P1" s="11" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
@@ -849,324 +1012,375 @@
           <t>Prob</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C2" s="13" t="n"/>
-      <c r="D2" s="13" t="n"/>
-      <c r="E2" s="13" t="n"/>
-      <c r="F2" s="13" t="n"/>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="14" t="n"/>
+      <c r="E2" s="14" t="n"/>
+      <c r="F2" s="14" t="n"/>
+      <c r="G2" s="15" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H2" s="13" t="n"/>
-      <c r="I2" s="13" t="n"/>
-      <c r="J2" s="13" t="n"/>
-      <c r="K2" s="13" t="n"/>
-      <c r="L2" s="13" t="n"/>
-      <c r="M2" s="13" t="n"/>
-      <c r="N2" s="12" t="inlineStr">
+      <c r="H2" s="14" t="n"/>
+      <c r="I2" s="14" t="n"/>
+      <c r="J2" s="14" t="n"/>
+      <c r="K2" s="14" t="n"/>
+      <c r="L2" s="14" t="n"/>
+      <c r="M2" s="14" t="n"/>
+      <c r="N2" s="13" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
+      <c r="O2" s="14" t="n"/>
+      <c r="P2" s="16" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="15" t="n">
+      <c r="A3" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="16">
+      <c r="B3" s="18">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C3" s="16">
+      <c r="C3" s="18">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="18">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="18">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F3" s="16">
+      <c r="F3" s="18">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G3" s="17">
+      <c r="G3" s="19">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H3" s="16">
+      <c r="H3" s="18">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I3" s="16">
+      <c r="I3" s="18">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J3" s="16">
+      <c r="J3" s="18">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K3" s="16">
+      <c r="K3" s="18">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L3" s="16">
+      <c r="L3" s="18">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M3" s="16">
+      <c r="M3" s="18">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N3" s="7" t="n"/>
+      <c r="O3" s="20">
+        <f>"/ "&amp;Setup!$E$7</f>
+        <v/>
+      </c>
+      <c r="P3" s="21" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="15" t="n">
+      <c r="A4" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="18">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C4" s="16">
+      <c r="C4" s="18">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="18">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="18">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="18">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G4" s="17">
+      <c r="G4" s="19">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H4" s="16">
+      <c r="H4" s="18">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I4" s="16">
+      <c r="I4" s="18">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J4" s="16">
+      <c r="J4" s="18">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K4" s="16">
+      <c r="K4" s="18">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L4" s="16">
+      <c r="L4" s="18">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M4" s="16">
+      <c r="M4" s="18">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N4" s="7" t="n"/>
+      <c r="O4" s="20">
+        <f>"/ "&amp;Setup!$E$8</f>
+        <v/>
+      </c>
+      <c r="P4" s="21" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="15" t="n">
+      <c r="A5" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="18">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="18">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="18">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="18">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="18">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G5" s="17">
+      <c r="G5" s="19">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H5" s="16">
+      <c r="H5" s="18">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I5" s="16">
+      <c r="I5" s="18">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J5" s="16">
+      <c r="J5" s="18">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K5" s="16">
+      <c r="K5" s="18">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L5" s="16">
+      <c r="L5" s="18">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M5" s="16">
+      <c r="M5" s="18">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N5" s="7" t="n"/>
+      <c r="O5" s="20">
+        <f>"/ "&amp;Setup!$E$9</f>
+        <v/>
+      </c>
+      <c r="P5" s="21" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="15" t="n">
+      <c r="A6" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="18">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="18">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="18">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="18">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="18">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G6" s="17">
+      <c r="G6" s="19">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H6" s="16">
+      <c r="H6" s="18">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I6" s="16">
+      <c r="I6" s="18">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J6" s="16">
+      <c r="J6" s="18">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K6" s="16">
+      <c r="K6" s="18">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L6" s="16">
+      <c r="L6" s="18">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M6" s="16">
+      <c r="M6" s="18">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N6" s="7" t="n"/>
+      <c r="O6" s="20">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="P6" s="21" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="15" t="n">
+      <c r="A7" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="18">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="18">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="18">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="18">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="18">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G7" s="17">
+      <c r="G7" s="19">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H7" s="16">
+      <c r="H7" s="18">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I7" s="16">
+      <c r="I7" s="18">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J7" s="16">
+      <c r="J7" s="18">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K7" s="16">
+      <c r="K7" s="18">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L7" s="16">
+      <c r="L7" s="18">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M7" s="16">
+      <c r="M7" s="18">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N7" s="7" t="n"/>
+      <c r="O7" s="20">
+        <f>"/ "&amp;Setup!$E$11</f>
+        <v/>
+      </c>
+      <c r="P7" s="21" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="18">
-        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
-        <v/>
-      </c>
-      <c r="N8" s="19" t="n"/>
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL SCORE  →</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="n"/>
+      <c r="C8" s="23" t="n"/>
+      <c r="D8" s="23" t="n"/>
+      <c r="E8" s="23" t="n"/>
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="23" t="n"/>
+      <c r="H8" s="23" t="n"/>
+      <c r="I8" s="23" t="n"/>
+      <c r="J8" s="23" t="n"/>
+      <c r="K8" s="23" t="n"/>
+      <c r="L8" s="23" t="n"/>
+      <c r="M8" s="23" t="n"/>
+      <c r="N8" s="24" t="n"/>
+      <c r="O8" s="25">
+        <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
+        <v/>
+      </c>
+      <c r="P8" s="26" t="n"/>
     </row>
     <row r="9" ht="9" customHeight="1">
-      <c r="A9" s="20" t="n"/>
-      <c r="B9" s="20" t="n"/>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-      <c r="F9" s="20" t="n"/>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="20" t="n"/>
-      <c r="I9" s="20" t="n"/>
-      <c r="J9" s="20" t="n"/>
-      <c r="K9" s="20" t="n"/>
-      <c r="L9" s="20" t="n"/>
-      <c r="M9" s="20" t="n"/>
-      <c r="N9" s="20" t="n"/>
+      <c r="A9" s="27" t="n"/>
+      <c r="B9" s="27" t="n"/>
+      <c r="C9" s="27" t="n"/>
+      <c r="D9" s="27" t="n"/>
+      <c r="E9" s="27" t="n"/>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="27" t="n"/>
+      <c r="H9" s="27" t="n"/>
+      <c r="I9" s="27" t="n"/>
+      <c r="J9" s="27" t="n"/>
+      <c r="K9" s="27" t="n"/>
+      <c r="L9" s="27" t="n"/>
+      <c r="M9" s="27" t="n"/>
+      <c r="N9" s="27" t="n"/>
+      <c r="O9" s="27" t="n"/>
+      <c r="P9" s="27" t="n"/>
     </row>
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="10">
@@ -1186,6 +1400,8 @@
       <c r="L10" s="11" t="n"/>
       <c r="M10" s="11" t="n"/>
       <c r="N10" s="11" t="n"/>
+      <c r="O10" s="11" t="n"/>
+      <c r="P10" s="11" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
@@ -1193,324 +1409,375 @@
           <t>Prob</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n"/>
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H11" s="13" t="n"/>
-      <c r="I11" s="13" t="n"/>
-      <c r="J11" s="13" t="n"/>
-      <c r="K11" s="13" t="n"/>
-      <c r="L11" s="13" t="n"/>
-      <c r="M11" s="13" t="n"/>
-      <c r="N11" s="12" t="inlineStr">
+      <c r="H11" s="14" t="n"/>
+      <c r="I11" s="14" t="n"/>
+      <c r="J11" s="14" t="n"/>
+      <c r="K11" s="14" t="n"/>
+      <c r="L11" s="14" t="n"/>
+      <c r="M11" s="14" t="n"/>
+      <c r="N11" s="13" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
+      <c r="O11" s="14" t="n"/>
+      <c r="P11" s="16" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="15" t="n">
+      <c r="A12" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="18">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="18">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="18">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="18">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="18">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G12" s="17">
+      <c r="G12" s="19">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H12" s="16">
+      <c r="H12" s="18">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I12" s="16">
+      <c r="I12" s="18">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J12" s="16">
+      <c r="J12" s="18">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K12" s="16">
+      <c r="K12" s="18">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L12" s="16">
+      <c r="L12" s="18">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M12" s="16">
+      <c r="M12" s="18">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N12" s="7" t="n"/>
+      <c r="O12" s="20">
+        <f>"/ "&amp;Setup!$E$7</f>
+        <v/>
+      </c>
+      <c r="P12" s="21" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="15" t="n">
+      <c r="A13" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="18">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C13" s="16">
+      <c r="C13" s="18">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="18">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="18">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="18">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G13" s="17">
+      <c r="G13" s="19">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H13" s="16">
+      <c r="H13" s="18">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I13" s="16">
+      <c r="I13" s="18">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J13" s="16">
+      <c r="J13" s="18">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K13" s="16">
+      <c r="K13" s="18">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L13" s="16">
+      <c r="L13" s="18">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M13" s="16">
+      <c r="M13" s="18">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N13" s="7" t="n"/>
+      <c r="O13" s="20">
+        <f>"/ "&amp;Setup!$E$8</f>
+        <v/>
+      </c>
+      <c r="P13" s="21" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="15" t="n">
+      <c r="A14" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="18">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="18">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="18">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="18">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="18">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G14" s="17">
+      <c r="G14" s="19">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H14" s="16">
+      <c r="H14" s="18">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I14" s="16">
+      <c r="I14" s="18">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J14" s="16">
+      <c r="J14" s="18">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K14" s="16">
+      <c r="K14" s="18">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L14" s="16">
+      <c r="L14" s="18">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M14" s="16">
+      <c r="M14" s="18">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N14" s="7" t="n"/>
+      <c r="O14" s="20">
+        <f>"/ "&amp;Setup!$E$9</f>
+        <v/>
+      </c>
+      <c r="P14" s="21" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="15" t="n">
+      <c r="A15" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="16">
+      <c r="B15" s="18">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C15" s="16">
+      <c r="C15" s="18">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="18">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="18">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="18">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G15" s="17">
+      <c r="G15" s="19">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H15" s="16">
+      <c r="H15" s="18">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I15" s="16">
+      <c r="I15" s="18">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J15" s="16">
+      <c r="J15" s="18">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K15" s="16">
+      <c r="K15" s="18">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L15" s="16">
+      <c r="L15" s="18">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M15" s="16">
+      <c r="M15" s="18">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N15" s="7" t="n"/>
+      <c r="O15" s="20">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="P15" s="21" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="15" t="n">
+      <c r="A16" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="16">
+      <c r="B16" s="18">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="18">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="18">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="18">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="18">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G16" s="17">
+      <c r="G16" s="19">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H16" s="16">
+      <c r="H16" s="18">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="18">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J16" s="16">
+      <c r="J16" s="18">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K16" s="16">
+      <c r="K16" s="18">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L16" s="16">
+      <c r="L16" s="18">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M16" s="16">
+      <c r="M16" s="18">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N16" s="7" t="n"/>
+      <c r="O16" s="20">
+        <f>"/ "&amp;Setup!$E$11</f>
+        <v/>
+      </c>
+      <c r="P16" s="21" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="18">
-        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
-        <v/>
-      </c>
-      <c r="N17" s="19" t="n"/>
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL SCORE  →</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="n"/>
+      <c r="C17" s="23" t="n"/>
+      <c r="D17" s="23" t="n"/>
+      <c r="E17" s="23" t="n"/>
+      <c r="F17" s="23" t="n"/>
+      <c r="G17" s="23" t="n"/>
+      <c r="H17" s="23" t="n"/>
+      <c r="I17" s="23" t="n"/>
+      <c r="J17" s="23" t="n"/>
+      <c r="K17" s="23" t="n"/>
+      <c r="L17" s="23" t="n"/>
+      <c r="M17" s="23" t="n"/>
+      <c r="N17" s="24" t="n"/>
+      <c r="O17" s="25">
+        <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
+        <v/>
+      </c>
+      <c r="P17" s="26" t="n"/>
     </row>
     <row r="18" ht="9" customHeight="1">
-      <c r="A18" s="20" t="n"/>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
-      <c r="F18" s="20" t="n"/>
-      <c r="G18" s="20" t="n"/>
-      <c r="H18" s="20" t="n"/>
-      <c r="I18" s="20" t="n"/>
-      <c r="J18" s="20" t="n"/>
-      <c r="K18" s="20" t="n"/>
-      <c r="L18" s="20" t="n"/>
-      <c r="M18" s="20" t="n"/>
-      <c r="N18" s="20" t="n"/>
+      <c r="A18" s="27" t="n"/>
+      <c r="B18" s="27" t="n"/>
+      <c r="C18" s="27" t="n"/>
+      <c r="D18" s="27" t="n"/>
+      <c r="E18" s="27" t="n"/>
+      <c r="F18" s="27" t="n"/>
+      <c r="G18" s="27" t="n"/>
+      <c r="H18" s="27" t="n"/>
+      <c r="I18" s="27" t="n"/>
+      <c r="J18" s="27" t="n"/>
+      <c r="K18" s="27" t="n"/>
+      <c r="L18" s="27" t="n"/>
+      <c r="M18" s="27" t="n"/>
+      <c r="N18" s="27" t="n"/>
+      <c r="O18" s="27" t="n"/>
+      <c r="P18" s="27" t="n"/>
     </row>
     <row r="19" ht="19" customHeight="1">
       <c r="A19" s="10">
@@ -1530,6 +1797,8 @@
       <c r="L19" s="11" t="n"/>
       <c r="M19" s="11" t="n"/>
       <c r="N19" s="11" t="n"/>
+      <c r="O19" s="11" t="n"/>
+      <c r="P19" s="11" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
@@ -1537,324 +1806,375 @@
           <t>Prob</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n"/>
-      <c r="G20" s="14" t="inlineStr">
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="14" t="n"/>
+      <c r="F20" s="14" t="n"/>
+      <c r="G20" s="15" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H20" s="13" t="n"/>
-      <c r="I20" s="13" t="n"/>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="13" t="n"/>
-      <c r="L20" s="13" t="n"/>
-      <c r="M20" s="13" t="n"/>
-      <c r="N20" s="12" t="inlineStr">
+      <c r="H20" s="14" t="n"/>
+      <c r="I20" s="14" t="n"/>
+      <c r="J20" s="14" t="n"/>
+      <c r="K20" s="14" t="n"/>
+      <c r="L20" s="14" t="n"/>
+      <c r="M20" s="14" t="n"/>
+      <c r="N20" s="13" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
+      <c r="O20" s="14" t="n"/>
+      <c r="P20" s="16" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="15" t="n">
+      <c r="A21" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B21" s="16">
+      <c r="B21" s="18">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C21" s="16">
+      <c r="C21" s="18">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D21" s="16">
+      <c r="D21" s="18">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E21" s="16">
+      <c r="E21" s="18">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F21" s="16">
+      <c r="F21" s="18">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G21" s="17">
+      <c r="G21" s="19">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H21" s="16">
+      <c r="H21" s="18">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I21" s="16">
+      <c r="I21" s="18">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J21" s="16">
+      <c r="J21" s="18">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K21" s="16">
+      <c r="K21" s="18">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L21" s="16">
+      <c r="L21" s="18">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M21" s="16">
+      <c r="M21" s="18">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N21" s="7" t="n"/>
+      <c r="O21" s="20">
+        <f>"/ "&amp;Setup!$E$7</f>
+        <v/>
+      </c>
+      <c r="P21" s="21" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="15" t="n">
+      <c r="A22" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B22" s="16">
+      <c r="B22" s="18">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="18">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="18">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E22" s="16">
+      <c r="E22" s="18">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="18">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G22" s="17">
+      <c r="G22" s="19">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H22" s="16">
+      <c r="H22" s="18">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I22" s="16">
+      <c r="I22" s="18">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J22" s="16">
+      <c r="J22" s="18">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K22" s="16">
+      <c r="K22" s="18">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L22" s="16">
+      <c r="L22" s="18">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M22" s="16">
+      <c r="M22" s="18">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N22" s="7" t="n"/>
+      <c r="O22" s="20">
+        <f>"/ "&amp;Setup!$E$8</f>
+        <v/>
+      </c>
+      <c r="P22" s="21" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="15" t="n">
+      <c r="A23" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B23" s="16">
+      <c r="B23" s="18">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="18">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="18">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E23" s="16">
+      <c r="E23" s="18">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="18">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G23" s="17">
+      <c r="G23" s="19">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H23" s="16">
+      <c r="H23" s="18">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I23" s="16">
+      <c r="I23" s="18">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J23" s="16">
+      <c r="J23" s="18">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K23" s="16">
+      <c r="K23" s="18">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L23" s="16">
+      <c r="L23" s="18">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M23" s="16">
+      <c r="M23" s="18">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N23" s="7" t="n"/>
+      <c r="O23" s="20">
+        <f>"/ "&amp;Setup!$E$9</f>
+        <v/>
+      </c>
+      <c r="P23" s="21" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="15" t="n">
+      <c r="A24" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B24" s="16">
+      <c r="B24" s="18">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="18">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D24" s="16">
+      <c r="D24" s="18">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E24" s="16">
+      <c r="E24" s="18">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F24" s="16">
+      <c r="F24" s="18">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G24" s="17">
+      <c r="G24" s="19">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H24" s="16">
+      <c r="H24" s="18">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I24" s="16">
+      <c r="I24" s="18">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J24" s="16">
+      <c r="J24" s="18">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K24" s="16">
+      <c r="K24" s="18">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L24" s="16">
+      <c r="L24" s="18">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M24" s="16">
+      <c r="M24" s="18">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N24" s="7" t="n"/>
+      <c r="O24" s="20">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="P24" s="21" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="15" t="n">
+      <c r="A25" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B25" s="16">
+      <c r="B25" s="18">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C25" s="16">
+      <c r="C25" s="18">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D25" s="16">
+      <c r="D25" s="18">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E25" s="16">
+      <c r="E25" s="18">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F25" s="16">
+      <c r="F25" s="18">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G25" s="17">
+      <c r="G25" s="19">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H25" s="16">
+      <c r="H25" s="18">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I25" s="16">
+      <c r="I25" s="18">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J25" s="16">
+      <c r="J25" s="18">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K25" s="16">
+      <c r="K25" s="18">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L25" s="16">
+      <c r="L25" s="18">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M25" s="16">
+      <c r="M25" s="18">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N25" s="7" t="n"/>
+      <c r="O25" s="20">
+        <f>"/ "&amp;Setup!$E$11</f>
+        <v/>
+      </c>
+      <c r="P25" s="21" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="18">
-        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
-        <v/>
-      </c>
-      <c r="N26" s="19" t="n"/>
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL SCORE  →</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="n"/>
+      <c r="C26" s="23" t="n"/>
+      <c r="D26" s="23" t="n"/>
+      <c r="E26" s="23" t="n"/>
+      <c r="F26" s="23" t="n"/>
+      <c r="G26" s="23" t="n"/>
+      <c r="H26" s="23" t="n"/>
+      <c r="I26" s="23" t="n"/>
+      <c r="J26" s="23" t="n"/>
+      <c r="K26" s="23" t="n"/>
+      <c r="L26" s="23" t="n"/>
+      <c r="M26" s="23" t="n"/>
+      <c r="N26" s="24" t="n"/>
+      <c r="O26" s="25">
+        <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
+        <v/>
+      </c>
+      <c r="P26" s="26" t="n"/>
     </row>
     <row r="27" ht="9" customHeight="1">
-      <c r="A27" s="20" t="n"/>
-      <c r="B27" s="20" t="n"/>
-      <c r="C27" s="20" t="n"/>
-      <c r="D27" s="20" t="n"/>
-      <c r="E27" s="20" t="n"/>
-      <c r="F27" s="20" t="n"/>
-      <c r="G27" s="20" t="n"/>
-      <c r="H27" s="20" t="n"/>
-      <c r="I27" s="20" t="n"/>
-      <c r="J27" s="20" t="n"/>
-      <c r="K27" s="20" t="n"/>
-      <c r="L27" s="20" t="n"/>
-      <c r="M27" s="20" t="n"/>
-      <c r="N27" s="20" t="n"/>
+      <c r="A27" s="27" t="n"/>
+      <c r="B27" s="27" t="n"/>
+      <c r="C27" s="27" t="n"/>
+      <c r="D27" s="27" t="n"/>
+      <c r="E27" s="27" t="n"/>
+      <c r="F27" s="27" t="n"/>
+      <c r="G27" s="27" t="n"/>
+      <c r="H27" s="27" t="n"/>
+      <c r="I27" s="27" t="n"/>
+      <c r="J27" s="27" t="n"/>
+      <c r="K27" s="27" t="n"/>
+      <c r="L27" s="27" t="n"/>
+      <c r="M27" s="27" t="n"/>
+      <c r="N27" s="27" t="n"/>
+      <c r="O27" s="27" t="n"/>
+      <c r="P27" s="27" t="n"/>
     </row>
     <row r="28" ht="19" customHeight="1">
       <c r="A28" s="10">
@@ -1874,6 +2194,8 @@
       <c r="L28" s="11" t="n"/>
       <c r="M28" s="11" t="n"/>
       <c r="N28" s="11" t="n"/>
+      <c r="O28" s="11" t="n"/>
+      <c r="P28" s="11" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="12" t="inlineStr">
@@ -1881,324 +2203,375 @@
           <t>Prob</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C29" s="13" t="n"/>
-      <c r="D29" s="13" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13" t="n"/>
-      <c r="G29" s="14" t="inlineStr">
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+      <c r="G29" s="15" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H29" s="13" t="n"/>
-      <c r="I29" s="13" t="n"/>
-      <c r="J29" s="13" t="n"/>
-      <c r="K29" s="13" t="n"/>
-      <c r="L29" s="13" t="n"/>
-      <c r="M29" s="13" t="n"/>
-      <c r="N29" s="12" t="inlineStr">
+      <c r="H29" s="14" t="n"/>
+      <c r="I29" s="14" t="n"/>
+      <c r="J29" s="14" t="n"/>
+      <c r="K29" s="14" t="n"/>
+      <c r="L29" s="14" t="n"/>
+      <c r="M29" s="14" t="n"/>
+      <c r="N29" s="13" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
+      <c r="O29" s="14" t="n"/>
+      <c r="P29" s="16" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="15" t="n">
+      <c r="A30" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="18">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="18">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D30" s="16">
+      <c r="D30" s="18">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="18">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F30" s="16">
+      <c r="F30" s="18">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G30" s="17">
+      <c r="G30" s="19">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H30" s="16">
+      <c r="H30" s="18">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I30" s="16">
+      <c r="I30" s="18">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J30" s="16">
+      <c r="J30" s="18">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K30" s="16">
+      <c r="K30" s="18">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L30" s="16">
+      <c r="L30" s="18">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M30" s="16">
+      <c r="M30" s="18">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N30" s="7" t="n"/>
+      <c r="O30" s="20">
+        <f>"/ "&amp;Setup!$E$7</f>
+        <v/>
+      </c>
+      <c r="P30" s="21" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="15" t="n">
+      <c r="A31" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="18">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="18">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="18">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E31" s="16">
+      <c r="E31" s="18">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F31" s="16">
+      <c r="F31" s="18">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G31" s="17">
+      <c r="G31" s="19">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H31" s="16">
+      <c r="H31" s="18">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I31" s="16">
+      <c r="I31" s="18">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J31" s="16">
+      <c r="J31" s="18">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K31" s="16">
+      <c r="K31" s="18">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L31" s="16">
+      <c r="L31" s="18">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M31" s="16">
+      <c r="M31" s="18">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N31" s="7" t="n"/>
+      <c r="O31" s="20">
+        <f>"/ "&amp;Setup!$E$8</f>
+        <v/>
+      </c>
+      <c r="P31" s="21" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="15" t="n">
+      <c r="A32" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B32" s="16">
+      <c r="B32" s="18">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C32" s="16">
+      <c r="C32" s="18">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D32" s="16">
+      <c r="D32" s="18">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E32" s="16">
+      <c r="E32" s="18">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F32" s="16">
+      <c r="F32" s="18">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G32" s="17">
+      <c r="G32" s="19">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H32" s="16">
+      <c r="H32" s="18">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I32" s="16">
+      <c r="I32" s="18">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J32" s="16">
+      <c r="J32" s="18">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K32" s="16">
+      <c r="K32" s="18">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L32" s="16">
+      <c r="L32" s="18">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M32" s="16">
+      <c r="M32" s="18">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N32" s="7" t="n"/>
+      <c r="O32" s="20">
+        <f>"/ "&amp;Setup!$E$9</f>
+        <v/>
+      </c>
+      <c r="P32" s="21" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="15" t="n">
+      <c r="A33" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B33" s="16">
+      <c r="B33" s="18">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C33" s="16">
+      <c r="C33" s="18">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D33" s="16">
+      <c r="D33" s="18">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E33" s="16">
+      <c r="E33" s="18">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F33" s="16">
+      <c r="F33" s="18">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G33" s="17">
+      <c r="G33" s="19">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H33" s="16">
+      <c r="H33" s="18">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I33" s="16">
+      <c r="I33" s="18">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J33" s="16">
+      <c r="J33" s="18">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K33" s="16">
+      <c r="K33" s="18">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L33" s="16">
+      <c r="L33" s="18">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M33" s="16">
+      <c r="M33" s="18">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N33" s="7" t="n"/>
+      <c r="O33" s="20">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="P33" s="21" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="15" t="n">
+      <c r="A34" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B34" s="16">
+      <c r="B34" s="18">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C34" s="16">
+      <c r="C34" s="18">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D34" s="16">
+      <c r="D34" s="18">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E34" s="16">
+      <c r="E34" s="18">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F34" s="16">
+      <c r="F34" s="18">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G34" s="17">
+      <c r="G34" s="19">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H34" s="16">
+      <c r="H34" s="18">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I34" s="16">
+      <c r="I34" s="18">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J34" s="16">
+      <c r="J34" s="18">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K34" s="16">
+      <c r="K34" s="18">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L34" s="16">
+      <c r="L34" s="18">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M34" s="16">
+      <c r="M34" s="18">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N34" s="7" t="n"/>
+      <c r="O34" s="20">
+        <f>"/ "&amp;Setup!$E$11</f>
+        <v/>
+      </c>
+      <c r="P34" s="21" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="18">
-        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
-        <v/>
-      </c>
-      <c r="N35" s="19" t="n"/>
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL SCORE  →</t>
+        </is>
+      </c>
+      <c r="B35" s="23" t="n"/>
+      <c r="C35" s="23" t="n"/>
+      <c r="D35" s="23" t="n"/>
+      <c r="E35" s="23" t="n"/>
+      <c r="F35" s="23" t="n"/>
+      <c r="G35" s="23" t="n"/>
+      <c r="H35" s="23" t="n"/>
+      <c r="I35" s="23" t="n"/>
+      <c r="J35" s="23" t="n"/>
+      <c r="K35" s="23" t="n"/>
+      <c r="L35" s="23" t="n"/>
+      <c r="M35" s="23" t="n"/>
+      <c r="N35" s="24" t="n"/>
+      <c r="O35" s="25">
+        <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
+        <v/>
+      </c>
+      <c r="P35" s="26" t="n"/>
     </row>
     <row r="36" ht="9" customHeight="1">
-      <c r="A36" s="20" t="n"/>
-      <c r="B36" s="20" t="n"/>
-      <c r="C36" s="20" t="n"/>
-      <c r="D36" s="20" t="n"/>
-      <c r="E36" s="20" t="n"/>
-      <c r="F36" s="20" t="n"/>
-      <c r="G36" s="20" t="n"/>
-      <c r="H36" s="20" t="n"/>
-      <c r="I36" s="20" t="n"/>
-      <c r="J36" s="20" t="n"/>
-      <c r="K36" s="20" t="n"/>
-      <c r="L36" s="20" t="n"/>
-      <c r="M36" s="20" t="n"/>
-      <c r="N36" s="20" t="n"/>
+      <c r="A36" s="27" t="n"/>
+      <c r="B36" s="27" t="n"/>
+      <c r="C36" s="27" t="n"/>
+      <c r="D36" s="27" t="n"/>
+      <c r="E36" s="27" t="n"/>
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="27" t="n"/>
+      <c r="H36" s="27" t="n"/>
+      <c r="I36" s="27" t="n"/>
+      <c r="J36" s="27" t="n"/>
+      <c r="K36" s="27" t="n"/>
+      <c r="L36" s="27" t="n"/>
+      <c r="M36" s="27" t="n"/>
+      <c r="N36" s="27" t="n"/>
+      <c r="O36" s="27" t="n"/>
+      <c r="P36" s="27" t="n"/>
     </row>
     <row r="37" ht="19" customHeight="1">
       <c r="A37" s="10">
@@ -2218,6 +2591,8 @@
       <c r="L37" s="11" t="n"/>
       <c r="M37" s="11" t="n"/>
       <c r="N37" s="11" t="n"/>
+      <c r="O37" s="11" t="n"/>
+      <c r="P37" s="11" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
@@ -2225,324 +2600,375 @@
           <t>Prob</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C38" s="13" t="n"/>
-      <c r="D38" s="13" t="n"/>
-      <c r="E38" s="13" t="n"/>
-      <c r="F38" s="13" t="n"/>
-      <c r="G38" s="14" t="inlineStr">
+      <c r="C38" s="14" t="n"/>
+      <c r="D38" s="14" t="n"/>
+      <c r="E38" s="14" t="n"/>
+      <c r="F38" s="14" t="n"/>
+      <c r="G38" s="15" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H38" s="13" t="n"/>
-      <c r="I38" s="13" t="n"/>
-      <c r="J38" s="13" t="n"/>
-      <c r="K38" s="13" t="n"/>
-      <c r="L38" s="13" t="n"/>
-      <c r="M38" s="13" t="n"/>
-      <c r="N38" s="12" t="inlineStr">
+      <c r="H38" s="14" t="n"/>
+      <c r="I38" s="14" t="n"/>
+      <c r="J38" s="14" t="n"/>
+      <c r="K38" s="14" t="n"/>
+      <c r="L38" s="14" t="n"/>
+      <c r="M38" s="14" t="n"/>
+      <c r="N38" s="13" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
+      <c r="O38" s="14" t="n"/>
+      <c r="P38" s="16" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="15" t="n">
+      <c r="A39" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B39" s="16">
+      <c r="B39" s="18">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C39" s="16">
+      <c r="C39" s="18">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D39" s="16">
+      <c r="D39" s="18">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E39" s="16">
+      <c r="E39" s="18">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F39" s="16">
+      <c r="F39" s="18">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G39" s="17">
+      <c r="G39" s="19">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H39" s="16">
+      <c r="H39" s="18">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I39" s="16">
+      <c r="I39" s="18">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J39" s="16">
+      <c r="J39" s="18">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K39" s="16">
+      <c r="K39" s="18">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L39" s="16">
+      <c r="L39" s="18">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M39" s="16">
+      <c r="M39" s="18">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N39" s="7" t="n"/>
+      <c r="O39" s="20">
+        <f>"/ "&amp;Setup!$E$7</f>
+        <v/>
+      </c>
+      <c r="P39" s="21" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="15" t="n">
+      <c r="A40" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B40" s="16">
+      <c r="B40" s="18">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C40" s="16">
+      <c r="C40" s="18">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D40" s="16">
+      <c r="D40" s="18">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E40" s="16">
+      <c r="E40" s="18">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F40" s="16">
+      <c r="F40" s="18">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G40" s="17">
+      <c r="G40" s="19">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H40" s="16">
+      <c r="H40" s="18">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I40" s="16">
+      <c r="I40" s="18">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J40" s="16">
+      <c r="J40" s="18">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K40" s="16">
+      <c r="K40" s="18">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L40" s="16">
+      <c r="L40" s="18">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M40" s="16">
+      <c r="M40" s="18">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N40" s="7" t="n"/>
+      <c r="O40" s="20">
+        <f>"/ "&amp;Setup!$E$8</f>
+        <v/>
+      </c>
+      <c r="P40" s="21" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="15" t="n">
+      <c r="A41" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="16">
+      <c r="B41" s="18">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C41" s="16">
+      <c r="C41" s="18">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D41" s="16">
+      <c r="D41" s="18">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E41" s="16">
+      <c r="E41" s="18">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F41" s="16">
+      <c r="F41" s="18">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G41" s="17">
+      <c r="G41" s="19">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H41" s="16">
+      <c r="H41" s="18">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I41" s="16">
+      <c r="I41" s="18">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J41" s="16">
+      <c r="J41" s="18">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K41" s="16">
+      <c r="K41" s="18">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L41" s="16">
+      <c r="L41" s="18">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M41" s="16">
+      <c r="M41" s="18">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N41" s="7" t="n"/>
+      <c r="O41" s="20">
+        <f>"/ "&amp;Setup!$E$9</f>
+        <v/>
+      </c>
+      <c r="P41" s="21" t="n"/>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="15" t="n">
+      <c r="A42" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B42" s="16">
+      <c r="B42" s="18">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C42" s="16">
+      <c r="C42" s="18">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D42" s="16">
+      <c r="D42" s="18">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E42" s="16">
+      <c r="E42" s="18">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F42" s="16">
+      <c r="F42" s="18">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G42" s="17">
+      <c r="G42" s="19">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H42" s="16">
+      <c r="H42" s="18">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I42" s="16">
+      <c r="I42" s="18">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J42" s="16">
+      <c r="J42" s="18">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K42" s="16">
+      <c r="K42" s="18">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L42" s="16">
+      <c r="L42" s="18">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M42" s="16">
+      <c r="M42" s="18">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N42" s="7" t="n"/>
+      <c r="O42" s="20">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="P42" s="21" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="15" t="n">
+      <c r="A43" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B43" s="16">
+      <c r="B43" s="18">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C43" s="16">
+      <c r="C43" s="18">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D43" s="16">
+      <c r="D43" s="18">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E43" s="16">
+      <c r="E43" s="18">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F43" s="16">
+      <c r="F43" s="18">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G43" s="17">
+      <c r="G43" s="19">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H43" s="16">
+      <c r="H43" s="18">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I43" s="16">
+      <c r="I43" s="18">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J43" s="16">
+      <c r="J43" s="18">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K43" s="16">
+      <c r="K43" s="18">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L43" s="16">
+      <c r="L43" s="18">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M43" s="16">
+      <c r="M43" s="18">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N43" s="7" t="n"/>
+      <c r="O43" s="20">
+        <f>"/ "&amp;Setup!$E$11</f>
+        <v/>
+      </c>
+      <c r="P43" s="21" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="18">
-        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
-        <v/>
-      </c>
-      <c r="N44" s="19" t="n"/>
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL SCORE  →</t>
+        </is>
+      </c>
+      <c r="B44" s="23" t="n"/>
+      <c r="C44" s="23" t="n"/>
+      <c r="D44" s="23" t="n"/>
+      <c r="E44" s="23" t="n"/>
+      <c r="F44" s="23" t="n"/>
+      <c r="G44" s="23" t="n"/>
+      <c r="H44" s="23" t="n"/>
+      <c r="I44" s="23" t="n"/>
+      <c r="J44" s="23" t="n"/>
+      <c r="K44" s="23" t="n"/>
+      <c r="L44" s="23" t="n"/>
+      <c r="M44" s="23" t="n"/>
+      <c r="N44" s="24" t="n"/>
+      <c r="O44" s="25">
+        <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
+        <v/>
+      </c>
+      <c r="P44" s="26" t="n"/>
     </row>
     <row r="45" ht="9" customHeight="1">
-      <c r="A45" s="20" t="n"/>
-      <c r="B45" s="20" t="n"/>
-      <c r="C45" s="20" t="n"/>
-      <c r="D45" s="20" t="n"/>
-      <c r="E45" s="20" t="n"/>
-      <c r="F45" s="20" t="n"/>
-      <c r="G45" s="20" t="n"/>
-      <c r="H45" s="20" t="n"/>
-      <c r="I45" s="20" t="n"/>
-      <c r="J45" s="20" t="n"/>
-      <c r="K45" s="20" t="n"/>
-      <c r="L45" s="20" t="n"/>
-      <c r="M45" s="20" t="n"/>
-      <c r="N45" s="20" t="n"/>
+      <c r="A45" s="27" t="n"/>
+      <c r="B45" s="27" t="n"/>
+      <c r="C45" s="27" t="n"/>
+      <c r="D45" s="27" t="n"/>
+      <c r="E45" s="27" t="n"/>
+      <c r="F45" s="27" t="n"/>
+      <c r="G45" s="27" t="n"/>
+      <c r="H45" s="27" t="n"/>
+      <c r="I45" s="27" t="n"/>
+      <c r="J45" s="27" t="n"/>
+      <c r="K45" s="27" t="n"/>
+      <c r="L45" s="27" t="n"/>
+      <c r="M45" s="27" t="n"/>
+      <c r="N45" s="27" t="n"/>
+      <c r="O45" s="27" t="n"/>
+      <c r="P45" s="27" t="n"/>
     </row>
     <row r="46" ht="19" customHeight="1">
       <c r="A46" s="10">
@@ -2562,6 +2988,8 @@
       <c r="L46" s="11" t="n"/>
       <c r="M46" s="11" t="n"/>
       <c r="N46" s="11" t="n"/>
+      <c r="O46" s="11" t="n"/>
+      <c r="P46" s="11" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="12" t="inlineStr">
@@ -2569,335 +2997,396 @@
           <t>Prob</t>
         </is>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B47" s="13" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C47" s="13" t="n"/>
-      <c r="D47" s="13" t="n"/>
-      <c r="E47" s="13" t="n"/>
-      <c r="F47" s="13" t="n"/>
-      <c r="G47" s="14" t="inlineStr">
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="14" t="n"/>
+      <c r="E47" s="14" t="n"/>
+      <c r="F47" s="14" t="n"/>
+      <c r="G47" s="15" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H47" s="13" t="n"/>
-      <c r="I47" s="13" t="n"/>
-      <c r="J47" s="13" t="n"/>
-      <c r="K47" s="13" t="n"/>
-      <c r="L47" s="13" t="n"/>
-      <c r="M47" s="13" t="n"/>
-      <c r="N47" s="12" t="inlineStr">
+      <c r="H47" s="14" t="n"/>
+      <c r="I47" s="14" t="n"/>
+      <c r="J47" s="14" t="n"/>
+      <c r="K47" s="14" t="n"/>
+      <c r="L47" s="14" t="n"/>
+      <c r="M47" s="14" t="n"/>
+      <c r="N47" s="13" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
+      <c r="O47" s="14" t="n"/>
+      <c r="P47" s="16" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="15" t="n">
+      <c r="A48" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B48" s="16">
+      <c r="B48" s="18">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C48" s="16">
+      <c r="C48" s="18">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D48" s="16">
+      <c r="D48" s="18">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E48" s="16">
+      <c r="E48" s="18">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F48" s="16">
+      <c r="F48" s="18">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G48" s="17">
+      <c r="G48" s="19">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H48" s="16">
+      <c r="H48" s="18">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I48" s="16">
+      <c r="I48" s="18">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J48" s="16">
+      <c r="J48" s="18">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K48" s="16">
+      <c r="K48" s="18">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L48" s="16">
+      <c r="L48" s="18">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M48" s="16">
+      <c r="M48" s="18">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="N48" s="7" t="n"/>
+      <c r="O48" s="20">
+        <f>"/ "&amp;Setup!$E$7</f>
+        <v/>
+      </c>
+      <c r="P48" s="21" t="n"/>
     </row>
     <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="15" t="n">
+      <c r="A49" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B49" s="16">
+      <c r="B49" s="18">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C49" s="16">
+      <c r="C49" s="18">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D49" s="16">
+      <c r="D49" s="18">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E49" s="16">
+      <c r="E49" s="18">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F49" s="16">
+      <c r="F49" s="18">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G49" s="17">
+      <c r="G49" s="19">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H49" s="16">
+      <c r="H49" s="18">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I49" s="16">
+      <c r="I49" s="18">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J49" s="16">
+      <c r="J49" s="18">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K49" s="16">
+      <c r="K49" s="18">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L49" s="16">
+      <c r="L49" s="18">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M49" s="16">
+      <c r="M49" s="18">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="N49" s="7" t="n"/>
+      <c r="O49" s="20">
+        <f>"/ "&amp;Setup!$E$8</f>
+        <v/>
+      </c>
+      <c r="P49" s="21" t="n"/>
     </row>
     <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="15" t="n">
+      <c r="A50" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B50" s="16">
+      <c r="B50" s="18">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C50" s="16">
+      <c r="C50" s="18">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D50" s="16">
+      <c r="D50" s="18">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E50" s="16">
+      <c r="E50" s="18">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F50" s="16">
+      <c r="F50" s="18">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G50" s="17">
+      <c r="G50" s="19">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H50" s="16">
+      <c r="H50" s="18">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I50" s="16">
+      <c r="I50" s="18">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J50" s="16">
+      <c r="J50" s="18">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K50" s="16">
+      <c r="K50" s="18">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L50" s="16">
+      <c r="L50" s="18">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M50" s="16">
+      <c r="M50" s="18">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="N50" s="7" t="n"/>
+      <c r="O50" s="20">
+        <f>"/ "&amp;Setup!$E$9</f>
+        <v/>
+      </c>
+      <c r="P50" s="21" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="15" t="n">
+      <c r="A51" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B51" s="16">
+      <c r="B51" s="18">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C51" s="16">
+      <c r="C51" s="18">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D51" s="16">
+      <c r="D51" s="18">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E51" s="16">
+      <c r="E51" s="18">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F51" s="16">
+      <c r="F51" s="18">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G51" s="17">
+      <c r="G51" s="19">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H51" s="16">
+      <c r="H51" s="18">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I51" s="16">
+      <c r="I51" s="18">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J51" s="16">
+      <c r="J51" s="18">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K51" s="16">
+      <c r="K51" s="18">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L51" s="16">
+      <c r="L51" s="18">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M51" s="16">
+      <c r="M51" s="18">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
       <c r="N51" s="7" t="n"/>
+      <c r="O51" s="20">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="P51" s="21" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="15" t="n">
+      <c r="A52" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B52" s="16">
+      <c r="B52" s="18">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C52" s="16">
+      <c r="C52" s="18">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D52" s="16">
+      <c r="D52" s="18">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E52" s="16">
+      <c r="E52" s="18">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F52" s="16">
+      <c r="F52" s="18">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G52" s="17">
+      <c r="G52" s="19">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H52" s="16">
+      <c r="H52" s="18">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I52" s="16">
+      <c r="I52" s="18">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J52" s="16">
+      <c r="J52" s="18">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K52" s="16">
+      <c r="K52" s="18">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L52" s="16">
+      <c r="L52" s="18">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M52" s="16">
+      <c r="M52" s="18">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
       <c r="N52" s="7" t="n"/>
+      <c r="O52" s="20">
+        <f>"/ "&amp;Setup!$E$11</f>
+        <v/>
+      </c>
+      <c r="P52" s="21" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="18">
-        <f>"TOTAL SCORE  (out of "&amp;SUM(Setup!$E$7:$E$11)&amp;" pts)  →"</f>
-        <v/>
-      </c>
-      <c r="N53" s="19" t="n"/>
+      <c r="A53" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL SCORE  →</t>
+        </is>
+      </c>
+      <c r="B53" s="23" t="n"/>
+      <c r="C53" s="23" t="n"/>
+      <c r="D53" s="23" t="n"/>
+      <c r="E53" s="23" t="n"/>
+      <c r="F53" s="23" t="n"/>
+      <c r="G53" s="23" t="n"/>
+      <c r="H53" s="23" t="n"/>
+      <c r="I53" s="23" t="n"/>
+      <c r="J53" s="23" t="n"/>
+      <c r="K53" s="23" t="n"/>
+      <c r="L53" s="23" t="n"/>
+      <c r="M53" s="23" t="n"/>
+      <c r="N53" s="24" t="n"/>
+      <c r="O53" s="25">
+        <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
+        <v/>
+      </c>
+      <c r="P53" s="26" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="36">
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N20:O20"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="A8:M8"/>
+    <mergeCell ref="N47:O47"/>
     <mergeCell ref="A17:M17"/>
     <mergeCell ref="G29:M29"/>
     <mergeCell ref="A35:M35"/>
     <mergeCell ref="G20:M20"/>
     <mergeCell ref="A53:M53"/>
     <mergeCell ref="G47:M47"/>
-    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A19:P19"/>
+    <mergeCell ref="A10:P10"/>
+    <mergeCell ref="A28:P28"/>
     <mergeCell ref="A44:M44"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B11:F11"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P47:P53"/>
     <mergeCell ref="G2:M2"/>
-    <mergeCell ref="A37:N37"/>
-    <mergeCell ref="A46:N46"/>
     <mergeCell ref="G11:M11"/>
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="B38:F38"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="P20:P26"/>
+    <mergeCell ref="P38:P44"/>
+    <mergeCell ref="P29:P35"/>
     <mergeCell ref="G38:M38"/>
+    <mergeCell ref="A46:P46"/>
     <mergeCell ref="B20:F20"/>
+    <mergeCell ref="A37:P37"/>
     <mergeCell ref="A26:M26"/>
-    <mergeCell ref="A19:N19"/>
-    <mergeCell ref="A10:N10"/>
-    <mergeCell ref="A28:N28"/>
+    <mergeCell ref="P2:P8"/>
+    <mergeCell ref="P11:P17"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
@@ -2933,364 +3422,364 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>What each dimension measures</t>
         </is>
       </c>
-      <c r="B4" s="22" t="n"/>
+      <c r="B4" s="29" t="n"/>
     </row>
     <row r="5" ht="33" customHeight="1">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>Final Answer  —  Did you land the correct result, properly expressed? Correct value(s), units, and significant figures. This is the ONLY place units and sig figs are judged.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Concept &amp; Execution  —  Do you understand the physics and can you carry it out? Right principle/equation (concept) + correct substitution, algebra, and method (execution) + clear, ordered, labeled work (communication). Graded on process, using Error-Carried-Forward.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Grading rules (apply before scoring)</t>
         </is>
       </c>
-      <c r="B8" s="22" t="n"/>
+      <c r="B8" s="29" t="n"/>
     </row>
     <row r="9" ht="33" customHeight="1">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>1.  Score each column on its own descriptor; never penalize the same flaw twice. Units/sig-fig issues affect only Final Answer.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>2.  Error-Carried-Forward (ECF): judge each step against the student's own prior results, not the answer key.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>3.  Consistency (default): the two columns should tell the same story — strong process usually accompanies a correct answer.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="33" customHeight="1">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>4.  ECF override: if the ONLY defect is a single arithmetic/transcription slip and every later step is correct under ECF, score Concept &amp; Execution on process merit (it may reach the top band) even though the final answer is wrong.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>5.  Answer only / no work shown: score Final Answer on merit; Concept &amp; Execution = 0.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>6.  Blank: 0 / 0.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>TYPE A — Single-unknown (Total 5)</t>
         </is>
       </c>
-      <c r="B16" s="22" t="n"/>
+      <c r="B16" s="29" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>Final Answer (0–2)</t>
         </is>
       </c>
-      <c r="B17" s="25" t="inlineStr">
+      <c r="B17" s="32" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
-      <c r="A18" s="26" t="inlineStr">
+      <c r="A18" s="33" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B18" s="27" t="inlineStr">
+      <c r="B18" s="34" t="inlineStr">
         <is>
           <t>Correct value, correct units, appropriate significant figures.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1">
-      <c r="A19" s="26" t="inlineStr">
+      <c r="A19" s="33" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B19" s="27" t="inlineStr">
+      <c r="B19" s="34" t="inlineStr">
         <is>
           <t>Correct value but units/sig figs wrong, OR a single arithmetic slip giving a near-correct value.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1">
-      <c r="A20" s="26" t="inlineStr">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B20" s="27" t="inlineStr">
+      <c r="B20" s="34" t="inlineStr">
         <is>
           <t>Incorrect, or blank.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>Concept &amp; Execution (0–3)</t>
         </is>
       </c>
-      <c r="B21" s="25" t="inlineStr">
+      <c r="B21" s="32" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1">
-      <c r="A22" s="26" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B22" s="27" t="inlineStr">
+      <c r="B22" s="34" t="inlineStr">
         <is>
           <t>Correct principle/equation; substitution and algebra correct; work clear and complete.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="A23" s="26" t="inlineStr">
+      <c r="A23" s="33" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B23" s="27" t="inlineStr">
+      <c r="B23" s="34" t="inlineStr">
         <is>
           <t>Correct principle; essentially right, with a minor execution slip or sparse-but-followable steps.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="33" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B24" s="27" t="inlineStr">
+      <c r="B24" s="34" t="inlineStr">
         <is>
           <t>Relevant concept present, but undermined by a wrong equation or a substantive execution error.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="26" t="inlineStr">
+      <c r="A25" s="33" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B25" s="27" t="inlineStr">
+      <c r="B25" s="34" t="inlineStr">
         <is>
           <t>Wrong concept, or no meaningful work.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="28" t="inlineStr">
         <is>
           <t>TYPE B — Multi-step / multi-unknown (Total 10)</t>
         </is>
       </c>
-      <c r="B27" s="22" t="n"/>
+      <c r="B27" s="29" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="24" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
         <is>
           <t>Final Answer (0–4)</t>
         </is>
       </c>
-      <c r="B28" s="25" t="inlineStr">
+      <c r="B28" s="32" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1">
-      <c r="A29" s="26" t="inlineStr">
+      <c r="A29" s="33" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B29" s="27" t="inlineStr">
+      <c r="B29" s="34" t="inlineStr">
         <is>
           <t>Every required final value correct, with correct units.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="26" t="inlineStr">
+      <c r="A30" s="33" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B30" s="27" t="inlineStr">
+      <c r="B30" s="34" t="inlineStr">
         <is>
           <t>All but one correct; the single miss is minor (units, sig figs, or one small slip).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="19" customHeight="1">
-      <c r="A31" s="26" t="inlineStr">
+      <c r="A31" s="33" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B31" s="27" t="inlineStr">
+      <c r="B31" s="34" t="inlineStr">
         <is>
           <t>Roughly half the values correct.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="26" t="inlineStr">
+      <c r="A32" s="33" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B32" s="27" t="inlineStr">
+      <c r="B32" s="34" t="inlineStr">
         <is>
           <t>One value correct, or most contain significant errors.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="26" t="inlineStr">
+      <c r="A33" s="33" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B33" s="27" t="inlineStr">
+      <c r="B33" s="34" t="inlineStr">
         <is>
           <t>No correct values, or blank.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
+      <c r="A34" s="31" t="inlineStr">
         <is>
           <t>Concept &amp; Execution (0–6)</t>
         </is>
       </c>
-      <c r="B34" s="25" t="inlineStr">
+      <c r="B34" s="32" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="35" ht="34" customHeight="1">
-      <c r="A35" s="26" t="inlineStr">
+      <c r="A35" s="33" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B35" s="27" t="inlineStr">
+      <c r="B35" s="34" t="inlineStr">
         <is>
           <t>Correct principle at EVERY step; all substitution, algebra, and units correct (ECF); logically ordered, labeled, easy to follow.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="34" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
+      <c r="A36" s="33" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B36" s="27" t="inlineStr">
+      <c r="B36" s="34" t="inlineStr">
         <is>
           <t>Correct principles and method throughout; at most one trivial slip or slightly sparse justification — physics fully sound.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="34" customHeight="1">
-      <c r="A37" s="26" t="inlineStr">
+      <c r="A37" s="33" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B37" s="27" t="inlineStr">
+      <c r="B37" s="34" t="inlineStr">
         <is>
           <t>Correct approach on the main steps, but ONE real execution error or one wrong/missing equation; work still followable.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="34" customHeight="1">
-      <c r="A38" s="26" t="inlineStr">
+      <c r="A38" s="33" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B38" s="27" t="inlineStr">
+      <c r="B38" s="34" t="inlineStr">
         <is>
           <t>Correct on some steps, but a wrong principle on a major step and/or several execution errors; reasoning has gaps.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="19" customHeight="1">
-      <c r="A39" s="26" t="inlineStr">
+      <c r="A39" s="33" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B39" s="27" t="inlineStr">
+      <c r="B39" s="34" t="inlineStr">
         <is>
           <t>Mostly incorrect method; more than a token of correct physics but hard to follow.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="19" customHeight="1">
-      <c r="A40" s="26" t="inlineStr">
+      <c r="A40" s="33" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B40" s="27" t="inlineStr">
+      <c r="B40" s="34" t="inlineStr">
         <is>
           <t>Little relevant physics; fundamentally the wrong approach with only a token correct fragment.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="19" customHeight="1">
-      <c r="A41" s="26" t="inlineStr">
+      <c r="A41" s="33" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B41" s="27" t="inlineStr">
+      <c r="B41" s="34" t="inlineStr">
         <is>
           <t>No meaningful work, or blank.</t>
         </is>

</xml_diff>

<commit_message>
Add left Name/Grade&Section vertical block, problem-5 separator rule, wider signing gap
</commit_message>
<xml_diff>
--- a/grading_rubric_A4.xlsx
+++ b/grading_rubric_A4.xlsx
@@ -103,7 +103,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -149,9 +149,9 @@
       </left>
     </border>
     <border>
-      <top style="medium">
-        <color rgb="00404040"/>
-      </top>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="00808080"/>
       </bottom>
@@ -159,9 +159,25 @@
     <border>
       <left/>
       <right/>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top/>
       <bottom style="medium">
         <color rgb="00404040"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
       </bottom>
     </border>
     <border>
@@ -190,23 +206,14 @@
       </bottom>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color rgb="00404040"/>
+      </left>
       <right/>
       <top style="medium">
         <color rgb="00404040"/>
       </top>
       <bottom/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00404040"/>
-      </left>
-      <top style="medium">
-        <color rgb="00404040"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00808080"/>
-      </bottom>
     </border>
     <border>
       <left/>
@@ -258,6 +265,17 @@
       <left style="thin">
         <color rgb="00808080"/>
       </left>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
       <right style="medium">
         <color rgb="00404040"/>
       </right>
@@ -270,11 +288,39 @@
       <left style="thin">
         <color rgb="00808080"/>
       </left>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
       <right style="medium">
         <color rgb="00404040"/>
       </right>
       <top/>
       <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00404040"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -297,7 +343,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -324,20 +370,24 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -349,19 +399,32 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
@@ -964,11 +1027,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="4.6" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
     <col width="4.6" customWidth="1" min="3" max="3"/>
     <col width="4.6" customWidth="1" min="4" max="4"/>
     <col width="4.6" customWidth="1" min="5" max="5"/>
@@ -980,9 +1043,10 @@
     <col width="4.6" customWidth="1" min="11" max="11"/>
     <col width="4.6" customWidth="1" min="12" max="12"/>
     <col width="4.6" customWidth="1" min="13" max="13"/>
-    <col width="6.5" customWidth="1" min="14" max="14"/>
-    <col width="4.6" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="4.6" customWidth="1" min="14" max="14"/>
+    <col width="6.5" customWidth="1" min="15" max="15"/>
+    <col width="4.6" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="19" customHeight="1">
@@ -1005,382 +1069,395 @@
       <c r="N1" s="11" t="n"/>
       <c r="O1" s="11" t="n"/>
       <c r="P1" s="11" t="n"/>
+      <c r="Q1" s="11" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
         <is>
+          <t>Name: _____________________________          Grade &amp; Section: __________________</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
-      <c r="G2" s="15" t="inlineStr">
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
+      <c r="G2" s="15" t="n"/>
+      <c r="H2" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H2" s="14" t="n"/>
-      <c r="I2" s="14" t="n"/>
-      <c r="J2" s="14" t="n"/>
-      <c r="K2" s="14" t="n"/>
-      <c r="L2" s="14" t="n"/>
-      <c r="M2" s="14" t="n"/>
-      <c r="N2" s="13" t="inlineStr">
+      <c r="I2" s="15" t="n"/>
+      <c r="J2" s="15" t="n"/>
+      <c r="K2" s="15" t="n"/>
+      <c r="L2" s="15" t="n"/>
+      <c r="M2" s="15" t="n"/>
+      <c r="N2" s="15" t="n"/>
+      <c r="O2" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="O2" s="14" t="n"/>
-      <c r="P2" s="16" t="inlineStr">
-        <is>
-          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+      <c r="P2" s="15" t="n"/>
+      <c r="Q2" s="17" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="17" t="n">
+      <c r="A3" s="18" t="n"/>
+      <c r="B3" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="18">
+      <c r="C3" s="20">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C3" s="18">
+      <c r="D3" s="20">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D3" s="18">
+      <c r="E3" s="20">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E3" s="18">
+      <c r="F3" s="20">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F3" s="18">
+      <c r="G3" s="20">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G3" s="19">
+      <c r="H3" s="21">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H3" s="18">
+      <c r="I3" s="20">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I3" s="18">
+      <c r="J3" s="20">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J3" s="18">
+      <c r="K3" s="20">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K3" s="18">
+      <c r="L3" s="20">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L3" s="18">
+      <c r="M3" s="20">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M3" s="18">
+      <c r="N3" s="20">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
-      <c r="N3" s="7" t="n"/>
-      <c r="O3" s="20">
+      <c r="O3" s="7" t="n"/>
+      <c r="P3" s="22">
         <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
-      <c r="P3" s="21" t="n"/>
+      <c r="Q3" s="23" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="17" t="n">
+      <c r="A4" s="18" t="n"/>
+      <c r="B4" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="18">
+      <c r="C4" s="20">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C4" s="18">
+      <c r="D4" s="20">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D4" s="18">
+      <c r="E4" s="20">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E4" s="18">
+      <c r="F4" s="20">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F4" s="18">
+      <c r="G4" s="20">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G4" s="19">
+      <c r="H4" s="21">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H4" s="18">
+      <c r="I4" s="20">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I4" s="18">
+      <c r="J4" s="20">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J4" s="18">
+      <c r="K4" s="20">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K4" s="18">
+      <c r="L4" s="20">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L4" s="18">
+      <c r="M4" s="20">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M4" s="18">
+      <c r="N4" s="20">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="20">
+      <c r="O4" s="7" t="n"/>
+      <c r="P4" s="22">
         <f>"/ "&amp;Setup!$E$8</f>
         <v/>
       </c>
-      <c r="P4" s="21" t="n"/>
+      <c r="Q4" s="23" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="18" t="n"/>
+      <c r="B5" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="18">
+      <c r="C5" s="20">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C5" s="18">
+      <c r="D5" s="20">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D5" s="18">
+      <c r="E5" s="20">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E5" s="18">
+      <c r="F5" s="20">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F5" s="18">
+      <c r="G5" s="20">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G5" s="19">
+      <c r="H5" s="21">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H5" s="18">
+      <c r="I5" s="20">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I5" s="18">
+      <c r="J5" s="20">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J5" s="18">
+      <c r="K5" s="20">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K5" s="18">
+      <c r="L5" s="20">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L5" s="18">
+      <c r="M5" s="20">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M5" s="18">
+      <c r="N5" s="20">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
-      <c r="N5" s="7" t="n"/>
-      <c r="O5" s="20">
+      <c r="O5" s="7" t="n"/>
+      <c r="P5" s="22">
         <f>"/ "&amp;Setup!$E$9</f>
         <v/>
       </c>
-      <c r="P5" s="21" t="n"/>
+      <c r="Q5" s="23" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="18" t="n"/>
+      <c r="B6" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="18">
+      <c r="C6" s="20">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C6" s="18">
+      <c r="D6" s="20">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D6" s="18">
+      <c r="E6" s="20">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E6" s="18">
+      <c r="F6" s="20">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F6" s="18">
+      <c r="G6" s="20">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G6" s="19">
+      <c r="H6" s="21">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H6" s="18">
+      <c r="I6" s="20">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I6" s="18">
+      <c r="J6" s="20">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J6" s="18">
+      <c r="K6" s="20">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K6" s="18">
+      <c r="L6" s="20">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L6" s="18">
+      <c r="M6" s="20">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M6" s="18">
+      <c r="N6" s="20">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
-      <c r="N6" s="7" t="n"/>
-      <c r="O6" s="20">
+      <c r="O6" s="7" t="n"/>
+      <c r="P6" s="22">
         <f>"/ "&amp;Setup!$E$10</f>
         <v/>
       </c>
-      <c r="P6" s="21" t="n"/>
+      <c r="Q6" s="23" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="18" t="n"/>
+      <c r="B7" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="18">
+      <c r="C7" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C7" s="18">
+      <c r="D7" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D7" s="18">
+      <c r="E7" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E7" s="18">
+      <c r="F7" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F7" s="18">
+      <c r="G7" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G7" s="19">
+      <c r="H7" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H7" s="18">
+      <c r="I7" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I7" s="18">
+      <c r="J7" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J7" s="18">
+      <c r="K7" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K7" s="18">
+      <c r="L7" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L7" s="18">
+      <c r="M7" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M7" s="18">
+      <c r="N7" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="20">
+      <c r="O7" s="7" t="n"/>
+      <c r="P7" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="P7" s="21" t="n"/>
+      <c r="Q7" s="23" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="28" t="n"/>
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="B8" s="23" t="n"/>
-      <c r="C8" s="23" t="n"/>
-      <c r="D8" s="23" t="n"/>
-      <c r="E8" s="23" t="n"/>
-      <c r="F8" s="23" t="n"/>
-      <c r="G8" s="23" t="n"/>
-      <c r="H8" s="23" t="n"/>
-      <c r="I8" s="23" t="n"/>
-      <c r="J8" s="23" t="n"/>
-      <c r="K8" s="23" t="n"/>
-      <c r="L8" s="23" t="n"/>
-      <c r="M8" s="23" t="n"/>
-      <c r="N8" s="24" t="n"/>
-      <c r="O8" s="25">
+      <c r="C8" s="30" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="30" t="n"/>
+      <c r="F8" s="30" t="n"/>
+      <c r="G8" s="30" t="n"/>
+      <c r="H8" s="30" t="n"/>
+      <c r="I8" s="30" t="n"/>
+      <c r="J8" s="30" t="n"/>
+      <c r="K8" s="30" t="n"/>
+      <c r="L8" s="30" t="n"/>
+      <c r="M8" s="30" t="n"/>
+      <c r="N8" s="30" t="n"/>
+      <c r="O8" s="31" t="n"/>
+      <c r="P8" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="P8" s="26" t="n"/>
+      <c r="Q8" s="33" t="n"/>
     </row>
     <row r="9" ht="9" customHeight="1">
-      <c r="A9" s="27" t="n"/>
-      <c r="B9" s="27" t="n"/>
-      <c r="C9" s="27" t="n"/>
-      <c r="D9" s="27" t="n"/>
-      <c r="E9" s="27" t="n"/>
-      <c r="F9" s="27" t="n"/>
-      <c r="G9" s="27" t="n"/>
-      <c r="H9" s="27" t="n"/>
-      <c r="I9" s="27" t="n"/>
-      <c r="J9" s="27" t="n"/>
-      <c r="K9" s="27" t="n"/>
-      <c r="L9" s="27" t="n"/>
-      <c r="M9" s="27" t="n"/>
-      <c r="N9" s="27" t="n"/>
-      <c r="O9" s="27" t="n"/>
-      <c r="P9" s="27" t="n"/>
+      <c r="A9" s="34" t="n"/>
+      <c r="B9" s="34" t="n"/>
+      <c r="C9" s="34" t="n"/>
+      <c r="D9" s="34" t="n"/>
+      <c r="E9" s="34" t="n"/>
+      <c r="F9" s="34" t="n"/>
+      <c r="G9" s="34" t="n"/>
+      <c r="H9" s="34" t="n"/>
+      <c r="I9" s="34" t="n"/>
+      <c r="J9" s="34" t="n"/>
+      <c r="K9" s="34" t="n"/>
+      <c r="L9" s="34" t="n"/>
+      <c r="M9" s="34" t="n"/>
+      <c r="N9" s="34" t="n"/>
+      <c r="O9" s="34" t="n"/>
+      <c r="P9" s="34" t="n"/>
+      <c r="Q9" s="34" t="n"/>
     </row>
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="10">
@@ -1402,382 +1479,395 @@
       <c r="N10" s="11" t="n"/>
       <c r="O10" s="11" t="n"/>
       <c r="P10" s="11" t="n"/>
+      <c r="Q10" s="11" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
+          <t>Name: _____________________________          Grade &amp; Section: __________________</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="15" t="inlineStr">
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H11" s="14" t="n"/>
-      <c r="I11" s="14" t="n"/>
-      <c r="J11" s="14" t="n"/>
-      <c r="K11" s="14" t="n"/>
-      <c r="L11" s="14" t="n"/>
-      <c r="M11" s="14" t="n"/>
-      <c r="N11" s="13" t="inlineStr">
+      <c r="I11" s="15" t="n"/>
+      <c r="J11" s="15" t="n"/>
+      <c r="K11" s="15" t="n"/>
+      <c r="L11" s="15" t="n"/>
+      <c r="M11" s="15" t="n"/>
+      <c r="N11" s="15" t="n"/>
+      <c r="O11" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="O11" s="14" t="n"/>
-      <c r="P11" s="16" t="inlineStr">
-        <is>
-          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+      <c r="P11" s="15" t="n"/>
+      <c r="Q11" s="17" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="17" t="n">
+      <c r="A12" s="18" t="n"/>
+      <c r="B12" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="18">
+      <c r="C12" s="20">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C12" s="18">
+      <c r="D12" s="20">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D12" s="18">
+      <c r="E12" s="20">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E12" s="18">
+      <c r="F12" s="20">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F12" s="18">
+      <c r="G12" s="20">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G12" s="19">
+      <c r="H12" s="21">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H12" s="18">
+      <c r="I12" s="20">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I12" s="18">
+      <c r="J12" s="20">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J12" s="18">
+      <c r="K12" s="20">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K12" s="18">
+      <c r="L12" s="20">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L12" s="18">
+      <c r="M12" s="20">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M12" s="18">
+      <c r="N12" s="20">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
-      <c r="N12" s="7" t="n"/>
-      <c r="O12" s="20">
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="22">
         <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
-      <c r="P12" s="21" t="n"/>
+      <c r="Q12" s="23" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="17" t="n">
+      <c r="A13" s="18" t="n"/>
+      <c r="B13" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="18">
+      <c r="C13" s="20">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C13" s="18">
+      <c r="D13" s="20">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D13" s="18">
+      <c r="E13" s="20">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E13" s="18">
+      <c r="F13" s="20">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F13" s="18">
+      <c r="G13" s="20">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G13" s="19">
+      <c r="H13" s="21">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H13" s="18">
+      <c r="I13" s="20">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I13" s="18">
+      <c r="J13" s="20">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J13" s="18">
+      <c r="K13" s="20">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K13" s="18">
+      <c r="L13" s="20">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L13" s="18">
+      <c r="M13" s="20">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M13" s="18">
+      <c r="N13" s="20">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="20">
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="22">
         <f>"/ "&amp;Setup!$E$8</f>
         <v/>
       </c>
-      <c r="P13" s="21" t="n"/>
+      <c r="Q13" s="23" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="17" t="n">
+      <c r="A14" s="18" t="n"/>
+      <c r="B14" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="18">
+      <c r="C14" s="20">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C14" s="18">
+      <c r="D14" s="20">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D14" s="18">
+      <c r="E14" s="20">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E14" s="18">
+      <c r="F14" s="20">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F14" s="18">
+      <c r="G14" s="20">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G14" s="19">
+      <c r="H14" s="21">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H14" s="18">
+      <c r="I14" s="20">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I14" s="18">
+      <c r="J14" s="20">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J14" s="18">
+      <c r="K14" s="20">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K14" s="18">
+      <c r="L14" s="20">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L14" s="18">
+      <c r="M14" s="20">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M14" s="18">
+      <c r="N14" s="20">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
-      <c r="N14" s="7" t="n"/>
-      <c r="O14" s="20">
+      <c r="O14" s="7" t="n"/>
+      <c r="P14" s="22">
         <f>"/ "&amp;Setup!$E$9</f>
         <v/>
       </c>
-      <c r="P14" s="21" t="n"/>
+      <c r="Q14" s="23" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="17" t="n">
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="18">
+      <c r="C15" s="20">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C15" s="18">
+      <c r="D15" s="20">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D15" s="18">
+      <c r="E15" s="20">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E15" s="18">
+      <c r="F15" s="20">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F15" s="18">
+      <c r="G15" s="20">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G15" s="19">
+      <c r="H15" s="21">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H15" s="18">
+      <c r="I15" s="20">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I15" s="18">
+      <c r="J15" s="20">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J15" s="18">
+      <c r="K15" s="20">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K15" s="18">
+      <c r="L15" s="20">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L15" s="18">
+      <c r="M15" s="20">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M15" s="18">
+      <c r="N15" s="20">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
-      <c r="N15" s="7" t="n"/>
-      <c r="O15" s="20">
+      <c r="O15" s="7" t="n"/>
+      <c r="P15" s="22">
         <f>"/ "&amp;Setup!$E$10</f>
         <v/>
       </c>
-      <c r="P15" s="21" t="n"/>
+      <c r="Q15" s="23" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="17" t="n">
+      <c r="A16" s="18" t="n"/>
+      <c r="B16" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="18">
+      <c r="C16" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C16" s="18">
+      <c r="D16" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D16" s="18">
+      <c r="E16" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E16" s="18">
+      <c r="F16" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F16" s="18">
+      <c r="G16" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G16" s="19">
+      <c r="H16" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H16" s="18">
+      <c r="I16" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I16" s="18">
+      <c r="J16" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J16" s="18">
+      <c r="K16" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K16" s="18">
+      <c r="L16" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L16" s="18">
+      <c r="M16" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M16" s="18">
+      <c r="N16" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="N16" s="7" t="n"/>
-      <c r="O16" s="20">
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="P16" s="21" t="n"/>
+      <c r="Q16" s="23" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="28" t="n"/>
+      <c r="B17" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="B17" s="23" t="n"/>
-      <c r="C17" s="23" t="n"/>
-      <c r="D17" s="23" t="n"/>
-      <c r="E17" s="23" t="n"/>
-      <c r="F17" s="23" t="n"/>
-      <c r="G17" s="23" t="n"/>
-      <c r="H17" s="23" t="n"/>
-      <c r="I17" s="23" t="n"/>
-      <c r="J17" s="23" t="n"/>
-      <c r="K17" s="23" t="n"/>
-      <c r="L17" s="23" t="n"/>
-      <c r="M17" s="23" t="n"/>
-      <c r="N17" s="24" t="n"/>
-      <c r="O17" s="25">
+      <c r="C17" s="30" t="n"/>
+      <c r="D17" s="30" t="n"/>
+      <c r="E17" s="30" t="n"/>
+      <c r="F17" s="30" t="n"/>
+      <c r="G17" s="30" t="n"/>
+      <c r="H17" s="30" t="n"/>
+      <c r="I17" s="30" t="n"/>
+      <c r="J17" s="30" t="n"/>
+      <c r="K17" s="30" t="n"/>
+      <c r="L17" s="30" t="n"/>
+      <c r="M17" s="30" t="n"/>
+      <c r="N17" s="30" t="n"/>
+      <c r="O17" s="31" t="n"/>
+      <c r="P17" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="P17" s="26" t="n"/>
+      <c r="Q17" s="33" t="n"/>
     </row>
     <row r="18" ht="9" customHeight="1">
-      <c r="A18" s="27" t="n"/>
-      <c r="B18" s="27" t="n"/>
-      <c r="C18" s="27" t="n"/>
-      <c r="D18" s="27" t="n"/>
-      <c r="E18" s="27" t="n"/>
-      <c r="F18" s="27" t="n"/>
-      <c r="G18" s="27" t="n"/>
-      <c r="H18" s="27" t="n"/>
-      <c r="I18" s="27" t="n"/>
-      <c r="J18" s="27" t="n"/>
-      <c r="K18" s="27" t="n"/>
-      <c r="L18" s="27" t="n"/>
-      <c r="M18" s="27" t="n"/>
-      <c r="N18" s="27" t="n"/>
-      <c r="O18" s="27" t="n"/>
-      <c r="P18" s="27" t="n"/>
+      <c r="A18" s="34" t="n"/>
+      <c r="B18" s="34" t="n"/>
+      <c r="C18" s="34" t="n"/>
+      <c r="D18" s="34" t="n"/>
+      <c r="E18" s="34" t="n"/>
+      <c r="F18" s="34" t="n"/>
+      <c r="G18" s="34" t="n"/>
+      <c r="H18" s="34" t="n"/>
+      <c r="I18" s="34" t="n"/>
+      <c r="J18" s="34" t="n"/>
+      <c r="K18" s="34" t="n"/>
+      <c r="L18" s="34" t="n"/>
+      <c r="M18" s="34" t="n"/>
+      <c r="N18" s="34" t="n"/>
+      <c r="O18" s="34" t="n"/>
+      <c r="P18" s="34" t="n"/>
+      <c r="Q18" s="34" t="n"/>
     </row>
     <row r="19" ht="19" customHeight="1">
       <c r="A19" s="10">
@@ -1799,382 +1889,395 @@
       <c r="N19" s="11" t="n"/>
       <c r="O19" s="11" t="n"/>
       <c r="P19" s="11" t="n"/>
+      <c r="Q19" s="11" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
         <is>
+          <t>Name: _____________________________          Grade &amp; Section: __________________</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
-      <c r="E20" s="14" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="15" t="inlineStr">
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="n"/>
+      <c r="G20" s="15" t="n"/>
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H20" s="14" t="n"/>
-      <c r="I20" s="14" t="n"/>
-      <c r="J20" s="14" t="n"/>
-      <c r="K20" s="14" t="n"/>
-      <c r="L20" s="14" t="n"/>
-      <c r="M20" s="14" t="n"/>
-      <c r="N20" s="13" t="inlineStr">
+      <c r="I20" s="15" t="n"/>
+      <c r="J20" s="15" t="n"/>
+      <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="n"/>
+      <c r="N20" s="15" t="n"/>
+      <c r="O20" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="O20" s="14" t="n"/>
-      <c r="P20" s="16" t="inlineStr">
-        <is>
-          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+      <c r="P20" s="15" t="n"/>
+      <c r="Q20" s="17" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="17" t="n">
+      <c r="A21" s="18" t="n"/>
+      <c r="B21" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B21" s="18">
+      <c r="C21" s="20">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C21" s="18">
+      <c r="D21" s="20">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D21" s="18">
+      <c r="E21" s="20">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E21" s="18">
+      <c r="F21" s="20">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F21" s="18">
+      <c r="G21" s="20">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G21" s="19">
+      <c r="H21" s="21">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H21" s="18">
+      <c r="I21" s="20">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I21" s="18">
+      <c r="J21" s="20">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J21" s="18">
+      <c r="K21" s="20">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K21" s="18">
+      <c r="L21" s="20">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L21" s="18">
+      <c r="M21" s="20">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M21" s="18">
+      <c r="N21" s="20">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="20">
+      <c r="O21" s="7" t="n"/>
+      <c r="P21" s="22">
         <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
-      <c r="P21" s="21" t="n"/>
+      <c r="Q21" s="23" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="17" t="n">
+      <c r="A22" s="18" t="n"/>
+      <c r="B22" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B22" s="18">
+      <c r="C22" s="20">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C22" s="18">
+      <c r="D22" s="20">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D22" s="18">
+      <c r="E22" s="20">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E22" s="18">
+      <c r="F22" s="20">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F22" s="18">
+      <c r="G22" s="20">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G22" s="19">
+      <c r="H22" s="21">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H22" s="18">
+      <c r="I22" s="20">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I22" s="18">
+      <c r="J22" s="20">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J22" s="18">
+      <c r="K22" s="20">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K22" s="18">
+      <c r="L22" s="20">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L22" s="18">
+      <c r="M22" s="20">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M22" s="18">
+      <c r="N22" s="20">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
-      <c r="N22" s="7" t="n"/>
-      <c r="O22" s="20">
+      <c r="O22" s="7" t="n"/>
+      <c r="P22" s="22">
         <f>"/ "&amp;Setup!$E$8</f>
         <v/>
       </c>
-      <c r="P22" s="21" t="n"/>
+      <c r="Q22" s="23" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="17" t="n">
+      <c r="A23" s="18" t="n"/>
+      <c r="B23" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B23" s="18">
+      <c r="C23" s="20">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C23" s="18">
+      <c r="D23" s="20">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D23" s="18">
+      <c r="E23" s="20">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E23" s="18">
+      <c r="F23" s="20">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F23" s="18">
+      <c r="G23" s="20">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G23" s="19">
+      <c r="H23" s="21">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H23" s="18">
+      <c r="I23" s="20">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I23" s="18">
+      <c r="J23" s="20">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J23" s="18">
+      <c r="K23" s="20">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K23" s="18">
+      <c r="L23" s="20">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L23" s="18">
+      <c r="M23" s="20">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M23" s="18">
+      <c r="N23" s="20">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
-      <c r="N23" s="7" t="n"/>
-      <c r="O23" s="20">
+      <c r="O23" s="7" t="n"/>
+      <c r="P23" s="22">
         <f>"/ "&amp;Setup!$E$9</f>
         <v/>
       </c>
-      <c r="P23" s="21" t="n"/>
+      <c r="Q23" s="23" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="17" t="n">
+      <c r="A24" s="18" t="n"/>
+      <c r="B24" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B24" s="18">
+      <c r="C24" s="20">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C24" s="18">
+      <c r="D24" s="20">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D24" s="18">
+      <c r="E24" s="20">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E24" s="18">
+      <c r="F24" s="20">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F24" s="18">
+      <c r="G24" s="20">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G24" s="19">
+      <c r="H24" s="21">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H24" s="18">
+      <c r="I24" s="20">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I24" s="18">
+      <c r="J24" s="20">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J24" s="18">
+      <c r="K24" s="20">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K24" s="18">
+      <c r="L24" s="20">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L24" s="18">
+      <c r="M24" s="20">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M24" s="18">
+      <c r="N24" s="20">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
-      <c r="N24" s="7" t="n"/>
-      <c r="O24" s="20">
+      <c r="O24" s="7" t="n"/>
+      <c r="P24" s="22">
         <f>"/ "&amp;Setup!$E$10</f>
         <v/>
       </c>
-      <c r="P24" s="21" t="n"/>
+      <c r="Q24" s="23" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="17" t="n">
+      <c r="A25" s="18" t="n"/>
+      <c r="B25" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B25" s="18">
+      <c r="C25" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C25" s="18">
+      <c r="D25" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D25" s="18">
+      <c r="E25" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E25" s="18">
+      <c r="F25" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F25" s="18">
+      <c r="G25" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G25" s="19">
+      <c r="H25" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H25" s="18">
+      <c r="I25" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I25" s="18">
+      <c r="J25" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J25" s="18">
+      <c r="K25" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K25" s="18">
+      <c r="L25" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L25" s="18">
+      <c r="M25" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M25" s="18">
+      <c r="N25" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="N25" s="7" t="n"/>
-      <c r="O25" s="20">
+      <c r="O25" s="7" t="n"/>
+      <c r="P25" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="P25" s="21" t="n"/>
+      <c r="Q25" s="23" t="n"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="22" t="inlineStr">
+      <c r="A26" s="28" t="n"/>
+      <c r="B26" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="B26" s="23" t="n"/>
-      <c r="C26" s="23" t="n"/>
-      <c r="D26" s="23" t="n"/>
-      <c r="E26" s="23" t="n"/>
-      <c r="F26" s="23" t="n"/>
-      <c r="G26" s="23" t="n"/>
-      <c r="H26" s="23" t="n"/>
-      <c r="I26" s="23" t="n"/>
-      <c r="J26" s="23" t="n"/>
-      <c r="K26" s="23" t="n"/>
-      <c r="L26" s="23" t="n"/>
-      <c r="M26" s="23" t="n"/>
-      <c r="N26" s="24" t="n"/>
-      <c r="O26" s="25">
+      <c r="C26" s="30" t="n"/>
+      <c r="D26" s="30" t="n"/>
+      <c r="E26" s="30" t="n"/>
+      <c r="F26" s="30" t="n"/>
+      <c r="G26" s="30" t="n"/>
+      <c r="H26" s="30" t="n"/>
+      <c r="I26" s="30" t="n"/>
+      <c r="J26" s="30" t="n"/>
+      <c r="K26" s="30" t="n"/>
+      <c r="L26" s="30" t="n"/>
+      <c r="M26" s="30" t="n"/>
+      <c r="N26" s="30" t="n"/>
+      <c r="O26" s="31" t="n"/>
+      <c r="P26" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="P26" s="26" t="n"/>
+      <c r="Q26" s="33" t="n"/>
     </row>
     <row r="27" ht="9" customHeight="1">
-      <c r="A27" s="27" t="n"/>
-      <c r="B27" s="27" t="n"/>
-      <c r="C27" s="27" t="n"/>
-      <c r="D27" s="27" t="n"/>
-      <c r="E27" s="27" t="n"/>
-      <c r="F27" s="27" t="n"/>
-      <c r="G27" s="27" t="n"/>
-      <c r="H27" s="27" t="n"/>
-      <c r="I27" s="27" t="n"/>
-      <c r="J27" s="27" t="n"/>
-      <c r="K27" s="27" t="n"/>
-      <c r="L27" s="27" t="n"/>
-      <c r="M27" s="27" t="n"/>
-      <c r="N27" s="27" t="n"/>
-      <c r="O27" s="27" t="n"/>
-      <c r="P27" s="27" t="n"/>
+      <c r="A27" s="34" t="n"/>
+      <c r="B27" s="34" t="n"/>
+      <c r="C27" s="34" t="n"/>
+      <c r="D27" s="34" t="n"/>
+      <c r="E27" s="34" t="n"/>
+      <c r="F27" s="34" t="n"/>
+      <c r="G27" s="34" t="n"/>
+      <c r="H27" s="34" t="n"/>
+      <c r="I27" s="34" t="n"/>
+      <c r="J27" s="34" t="n"/>
+      <c r="K27" s="34" t="n"/>
+      <c r="L27" s="34" t="n"/>
+      <c r="M27" s="34" t="n"/>
+      <c r="N27" s="34" t="n"/>
+      <c r="O27" s="34" t="n"/>
+      <c r="P27" s="34" t="n"/>
+      <c r="Q27" s="34" t="n"/>
     </row>
     <row r="28" ht="19" customHeight="1">
       <c r="A28" s="10">
@@ -2196,382 +2299,395 @@
       <c r="N28" s="11" t="n"/>
       <c r="O28" s="11" t="n"/>
       <c r="P28" s="11" t="n"/>
+      <c r="Q28" s="11" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="12" t="inlineStr">
         <is>
+          <t>Name: _____________________________          Grade &amp; Section: __________________</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="15" t="inlineStr">
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="15" t="n"/>
+      <c r="G29" s="15" t="n"/>
+      <c r="H29" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H29" s="14" t="n"/>
-      <c r="I29" s="14" t="n"/>
-      <c r="J29" s="14" t="n"/>
-      <c r="K29" s="14" t="n"/>
-      <c r="L29" s="14" t="n"/>
-      <c r="M29" s="14" t="n"/>
-      <c r="N29" s="13" t="inlineStr">
+      <c r="I29" s="15" t="n"/>
+      <c r="J29" s="15" t="n"/>
+      <c r="K29" s="15" t="n"/>
+      <c r="L29" s="15" t="n"/>
+      <c r="M29" s="15" t="n"/>
+      <c r="N29" s="15" t="n"/>
+      <c r="O29" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="O29" s="14" t="n"/>
-      <c r="P29" s="16" t="inlineStr">
-        <is>
-          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+      <c r="P29" s="15" t="n"/>
+      <c r="Q29" s="17" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="17" t="n">
+      <c r="A30" s="18" t="n"/>
+      <c r="B30" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B30" s="18">
+      <c r="C30" s="20">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C30" s="18">
+      <c r="D30" s="20">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D30" s="18">
+      <c r="E30" s="20">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E30" s="18">
+      <c r="F30" s="20">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F30" s="18">
+      <c r="G30" s="20">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G30" s="19">
+      <c r="H30" s="21">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H30" s="18">
+      <c r="I30" s="20">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I30" s="18">
+      <c r="J30" s="20">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J30" s="18">
+      <c r="K30" s="20">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K30" s="18">
+      <c r="L30" s="20">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L30" s="18">
+      <c r="M30" s="20">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M30" s="18">
+      <c r="N30" s="20">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
-      <c r="N30" s="7" t="n"/>
-      <c r="O30" s="20">
+      <c r="O30" s="7" t="n"/>
+      <c r="P30" s="22">
         <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
-      <c r="P30" s="21" t="n"/>
+      <c r="Q30" s="23" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="17" t="n">
+      <c r="A31" s="18" t="n"/>
+      <c r="B31" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B31" s="18">
+      <c r="C31" s="20">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C31" s="18">
+      <c r="D31" s="20">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D31" s="18">
+      <c r="E31" s="20">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E31" s="18">
+      <c r="F31" s="20">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F31" s="18">
+      <c r="G31" s="20">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G31" s="19">
+      <c r="H31" s="21">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H31" s="18">
+      <c r="I31" s="20">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I31" s="18">
+      <c r="J31" s="20">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J31" s="18">
+      <c r="K31" s="20">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K31" s="18">
+      <c r="L31" s="20">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L31" s="18">
+      <c r="M31" s="20">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M31" s="18">
+      <c r="N31" s="20">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
-      <c r="N31" s="7" t="n"/>
-      <c r="O31" s="20">
+      <c r="O31" s="7" t="n"/>
+      <c r="P31" s="22">
         <f>"/ "&amp;Setup!$E$8</f>
         <v/>
       </c>
-      <c r="P31" s="21" t="n"/>
+      <c r="Q31" s="23" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="17" t="n">
+      <c r="A32" s="18" t="n"/>
+      <c r="B32" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B32" s="18">
+      <c r="C32" s="20">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C32" s="18">
+      <c r="D32" s="20">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D32" s="18">
+      <c r="E32" s="20">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E32" s="18">
+      <c r="F32" s="20">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F32" s="18">
+      <c r="G32" s="20">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G32" s="19">
+      <c r="H32" s="21">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H32" s="18">
+      <c r="I32" s="20">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I32" s="18">
+      <c r="J32" s="20">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J32" s="18">
+      <c r="K32" s="20">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K32" s="18">
+      <c r="L32" s="20">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L32" s="18">
+      <c r="M32" s="20">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M32" s="18">
+      <c r="N32" s="20">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
-      <c r="N32" s="7" t="n"/>
-      <c r="O32" s="20">
+      <c r="O32" s="7" t="n"/>
+      <c r="P32" s="22">
         <f>"/ "&amp;Setup!$E$9</f>
         <v/>
       </c>
-      <c r="P32" s="21" t="n"/>
+      <c r="Q32" s="23" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="17" t="n">
+      <c r="A33" s="18" t="n"/>
+      <c r="B33" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B33" s="18">
+      <c r="C33" s="20">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C33" s="18">
+      <c r="D33" s="20">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D33" s="18">
+      <c r="E33" s="20">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E33" s="18">
+      <c r="F33" s="20">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F33" s="18">
+      <c r="G33" s="20">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G33" s="19">
+      <c r="H33" s="21">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H33" s="18">
+      <c r="I33" s="20">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I33" s="18">
+      <c r="J33" s="20">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J33" s="18">
+      <c r="K33" s="20">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K33" s="18">
+      <c r="L33" s="20">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L33" s="18">
+      <c r="M33" s="20">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M33" s="18">
+      <c r="N33" s="20">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
-      <c r="N33" s="7" t="n"/>
-      <c r="O33" s="20">
+      <c r="O33" s="7" t="n"/>
+      <c r="P33" s="22">
         <f>"/ "&amp;Setup!$E$10</f>
         <v/>
       </c>
-      <c r="P33" s="21" t="n"/>
+      <c r="Q33" s="23" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="17" t="n">
+      <c r="A34" s="18" t="n"/>
+      <c r="B34" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B34" s="18">
+      <c r="C34" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C34" s="18">
+      <c r="D34" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D34" s="18">
+      <c r="E34" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E34" s="18">
+      <c r="F34" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F34" s="18">
+      <c r="G34" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G34" s="19">
+      <c r="H34" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H34" s="18">
+      <c r="I34" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I34" s="18">
+      <c r="J34" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J34" s="18">
+      <c r="K34" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K34" s="18">
+      <c r="L34" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L34" s="18">
+      <c r="M34" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M34" s="18">
+      <c r="N34" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="N34" s="7" t="n"/>
-      <c r="O34" s="20">
+      <c r="O34" s="7" t="n"/>
+      <c r="P34" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="P34" s="21" t="n"/>
+      <c r="Q34" s="23" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="22" t="inlineStr">
+      <c r="A35" s="28" t="n"/>
+      <c r="B35" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="B35" s="23" t="n"/>
-      <c r="C35" s="23" t="n"/>
-      <c r="D35" s="23" t="n"/>
-      <c r="E35" s="23" t="n"/>
-      <c r="F35" s="23" t="n"/>
-      <c r="G35" s="23" t="n"/>
-      <c r="H35" s="23" t="n"/>
-      <c r="I35" s="23" t="n"/>
-      <c r="J35" s="23" t="n"/>
-      <c r="K35" s="23" t="n"/>
-      <c r="L35" s="23" t="n"/>
-      <c r="M35" s="23" t="n"/>
-      <c r="N35" s="24" t="n"/>
-      <c r="O35" s="25">
+      <c r="C35" s="30" t="n"/>
+      <c r="D35" s="30" t="n"/>
+      <c r="E35" s="30" t="n"/>
+      <c r="F35" s="30" t="n"/>
+      <c r="G35" s="30" t="n"/>
+      <c r="H35" s="30" t="n"/>
+      <c r="I35" s="30" t="n"/>
+      <c r="J35" s="30" t="n"/>
+      <c r="K35" s="30" t="n"/>
+      <c r="L35" s="30" t="n"/>
+      <c r="M35" s="30" t="n"/>
+      <c r="N35" s="30" t="n"/>
+      <c r="O35" s="31" t="n"/>
+      <c r="P35" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="P35" s="26" t="n"/>
+      <c r="Q35" s="33" t="n"/>
     </row>
     <row r="36" ht="9" customHeight="1">
-      <c r="A36" s="27" t="n"/>
-      <c r="B36" s="27" t="n"/>
-      <c r="C36" s="27" t="n"/>
-      <c r="D36" s="27" t="n"/>
-      <c r="E36" s="27" t="n"/>
-      <c r="F36" s="27" t="n"/>
-      <c r="G36" s="27" t="n"/>
-      <c r="H36" s="27" t="n"/>
-      <c r="I36" s="27" t="n"/>
-      <c r="J36" s="27" t="n"/>
-      <c r="K36" s="27" t="n"/>
-      <c r="L36" s="27" t="n"/>
-      <c r="M36" s="27" t="n"/>
-      <c r="N36" s="27" t="n"/>
-      <c r="O36" s="27" t="n"/>
-      <c r="P36" s="27" t="n"/>
+      <c r="A36" s="34" t="n"/>
+      <c r="B36" s="34" t="n"/>
+      <c r="C36" s="34" t="n"/>
+      <c r="D36" s="34" t="n"/>
+      <c r="E36" s="34" t="n"/>
+      <c r="F36" s="34" t="n"/>
+      <c r="G36" s="34" t="n"/>
+      <c r="H36" s="34" t="n"/>
+      <c r="I36" s="34" t="n"/>
+      <c r="J36" s="34" t="n"/>
+      <c r="K36" s="34" t="n"/>
+      <c r="L36" s="34" t="n"/>
+      <c r="M36" s="34" t="n"/>
+      <c r="N36" s="34" t="n"/>
+      <c r="O36" s="34" t="n"/>
+      <c r="P36" s="34" t="n"/>
+      <c r="Q36" s="34" t="n"/>
     </row>
     <row r="37" ht="19" customHeight="1">
       <c r="A37" s="10">
@@ -2593,382 +2709,395 @@
       <c r="N37" s="11" t="n"/>
       <c r="O37" s="11" t="n"/>
       <c r="P37" s="11" t="n"/>
+      <c r="Q37" s="11" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
+          <t>Name: _____________________________          Grade &amp; Section: __________________</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="C38" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C38" s="14" t="n"/>
-      <c r="D38" s="14" t="n"/>
-      <c r="E38" s="14" t="n"/>
-      <c r="F38" s="14" t="n"/>
-      <c r="G38" s="15" t="inlineStr">
+      <c r="D38" s="15" t="n"/>
+      <c r="E38" s="15" t="n"/>
+      <c r="F38" s="15" t="n"/>
+      <c r="G38" s="15" t="n"/>
+      <c r="H38" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H38" s="14" t="n"/>
-      <c r="I38" s="14" t="n"/>
-      <c r="J38" s="14" t="n"/>
-      <c r="K38" s="14" t="n"/>
-      <c r="L38" s="14" t="n"/>
-      <c r="M38" s="14" t="n"/>
-      <c r="N38" s="13" t="inlineStr">
+      <c r="I38" s="15" t="n"/>
+      <c r="J38" s="15" t="n"/>
+      <c r="K38" s="15" t="n"/>
+      <c r="L38" s="15" t="n"/>
+      <c r="M38" s="15" t="n"/>
+      <c r="N38" s="15" t="n"/>
+      <c r="O38" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="O38" s="14" t="n"/>
-      <c r="P38" s="16" t="inlineStr">
-        <is>
-          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+      <c r="P38" s="15" t="n"/>
+      <c r="Q38" s="17" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="17" t="n">
+      <c r="A39" s="18" t="n"/>
+      <c r="B39" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B39" s="18">
+      <c r="C39" s="20">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C39" s="18">
+      <c r="D39" s="20">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D39" s="18">
+      <c r="E39" s="20">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E39" s="18">
+      <c r="F39" s="20">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F39" s="18">
+      <c r="G39" s="20">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G39" s="19">
+      <c r="H39" s="21">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H39" s="18">
+      <c r="I39" s="20">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I39" s="18">
+      <c r="J39" s="20">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J39" s="18">
+      <c r="K39" s="20">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K39" s="18">
+      <c r="L39" s="20">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L39" s="18">
+      <c r="M39" s="20">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M39" s="18">
+      <c r="N39" s="20">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
-      <c r="N39" s="7" t="n"/>
-      <c r="O39" s="20">
+      <c r="O39" s="7" t="n"/>
+      <c r="P39" s="22">
         <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
-      <c r="P39" s="21" t="n"/>
+      <c r="Q39" s="23" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="17" t="n">
+      <c r="A40" s="18" t="n"/>
+      <c r="B40" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B40" s="18">
+      <c r="C40" s="20">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C40" s="18">
+      <c r="D40" s="20">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D40" s="18">
+      <c r="E40" s="20">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E40" s="18">
+      <c r="F40" s="20">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F40" s="18">
+      <c r="G40" s="20">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G40" s="19">
+      <c r="H40" s="21">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H40" s="18">
+      <c r="I40" s="20">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I40" s="18">
+      <c r="J40" s="20">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J40" s="18">
+      <c r="K40" s="20">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K40" s="18">
+      <c r="L40" s="20">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L40" s="18">
+      <c r="M40" s="20">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M40" s="18">
+      <c r="N40" s="20">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
-      <c r="N40" s="7" t="n"/>
-      <c r="O40" s="20">
+      <c r="O40" s="7" t="n"/>
+      <c r="P40" s="22">
         <f>"/ "&amp;Setup!$E$8</f>
         <v/>
       </c>
-      <c r="P40" s="21" t="n"/>
+      <c r="Q40" s="23" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="17" t="n">
+      <c r="A41" s="18" t="n"/>
+      <c r="B41" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B41" s="18">
+      <c r="C41" s="20">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C41" s="18">
+      <c r="D41" s="20">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D41" s="18">
+      <c r="E41" s="20">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E41" s="18">
+      <c r="F41" s="20">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F41" s="18">
+      <c r="G41" s="20">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G41" s="19">
+      <c r="H41" s="21">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H41" s="18">
+      <c r="I41" s="20">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I41" s="18">
+      <c r="J41" s="20">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J41" s="18">
+      <c r="K41" s="20">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K41" s="18">
+      <c r="L41" s="20">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L41" s="18">
+      <c r="M41" s="20">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M41" s="18">
+      <c r="N41" s="20">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
-      <c r="N41" s="7" t="n"/>
-      <c r="O41" s="20">
+      <c r="O41" s="7" t="n"/>
+      <c r="P41" s="22">
         <f>"/ "&amp;Setup!$E$9</f>
         <v/>
       </c>
-      <c r="P41" s="21" t="n"/>
+      <c r="Q41" s="23" t="n"/>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="17" t="n">
+      <c r="A42" s="18" t="n"/>
+      <c r="B42" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B42" s="18">
+      <c r="C42" s="20">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C42" s="18">
+      <c r="D42" s="20">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D42" s="18">
+      <c r="E42" s="20">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E42" s="18">
+      <c r="F42" s="20">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F42" s="18">
+      <c r="G42" s="20">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G42" s="19">
+      <c r="H42" s="21">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H42" s="18">
+      <c r="I42" s="20">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I42" s="18">
+      <c r="J42" s="20">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J42" s="18">
+      <c r="K42" s="20">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K42" s="18">
+      <c r="L42" s="20">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L42" s="18">
+      <c r="M42" s="20">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M42" s="18">
+      <c r="N42" s="20">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
-      <c r="N42" s="7" t="n"/>
-      <c r="O42" s="20">
+      <c r="O42" s="7" t="n"/>
+      <c r="P42" s="22">
         <f>"/ "&amp;Setup!$E$10</f>
         <v/>
       </c>
-      <c r="P42" s="21" t="n"/>
+      <c r="Q42" s="23" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="17" t="n">
+      <c r="A43" s="18" t="n"/>
+      <c r="B43" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B43" s="18">
+      <c r="C43" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C43" s="18">
+      <c r="D43" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D43" s="18">
+      <c r="E43" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E43" s="18">
+      <c r="F43" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F43" s="18">
+      <c r="G43" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G43" s="19">
+      <c r="H43" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H43" s="18">
+      <c r="I43" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I43" s="18">
+      <c r="J43" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J43" s="18">
+      <c r="K43" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K43" s="18">
+      <c r="L43" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L43" s="18">
+      <c r="M43" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M43" s="18">
+      <c r="N43" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="N43" s="7" t="n"/>
-      <c r="O43" s="20">
+      <c r="O43" s="7" t="n"/>
+      <c r="P43" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="P43" s="21" t="n"/>
+      <c r="Q43" s="23" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="22" t="inlineStr">
+      <c r="A44" s="28" t="n"/>
+      <c r="B44" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="B44" s="23" t="n"/>
-      <c r="C44" s="23" t="n"/>
-      <c r="D44" s="23" t="n"/>
-      <c r="E44" s="23" t="n"/>
-      <c r="F44" s="23" t="n"/>
-      <c r="G44" s="23" t="n"/>
-      <c r="H44" s="23" t="n"/>
-      <c r="I44" s="23" t="n"/>
-      <c r="J44" s="23" t="n"/>
-      <c r="K44" s="23" t="n"/>
-      <c r="L44" s="23" t="n"/>
-      <c r="M44" s="23" t="n"/>
-      <c r="N44" s="24" t="n"/>
-      <c r="O44" s="25">
+      <c r="C44" s="30" t="n"/>
+      <c r="D44" s="30" t="n"/>
+      <c r="E44" s="30" t="n"/>
+      <c r="F44" s="30" t="n"/>
+      <c r="G44" s="30" t="n"/>
+      <c r="H44" s="30" t="n"/>
+      <c r="I44" s="30" t="n"/>
+      <c r="J44" s="30" t="n"/>
+      <c r="K44" s="30" t="n"/>
+      <c r="L44" s="30" t="n"/>
+      <c r="M44" s="30" t="n"/>
+      <c r="N44" s="30" t="n"/>
+      <c r="O44" s="31" t="n"/>
+      <c r="P44" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="P44" s="26" t="n"/>
+      <c r="Q44" s="33" t="n"/>
     </row>
     <row r="45" ht="9" customHeight="1">
-      <c r="A45" s="27" t="n"/>
-      <c r="B45" s="27" t="n"/>
-      <c r="C45" s="27" t="n"/>
-      <c r="D45" s="27" t="n"/>
-      <c r="E45" s="27" t="n"/>
-      <c r="F45" s="27" t="n"/>
-      <c r="G45" s="27" t="n"/>
-      <c r="H45" s="27" t="n"/>
-      <c r="I45" s="27" t="n"/>
-      <c r="J45" s="27" t="n"/>
-      <c r="K45" s="27" t="n"/>
-      <c r="L45" s="27" t="n"/>
-      <c r="M45" s="27" t="n"/>
-      <c r="N45" s="27" t="n"/>
-      <c r="O45" s="27" t="n"/>
-      <c r="P45" s="27" t="n"/>
+      <c r="A45" s="34" t="n"/>
+      <c r="B45" s="34" t="n"/>
+      <c r="C45" s="34" t="n"/>
+      <c r="D45" s="34" t="n"/>
+      <c r="E45" s="34" t="n"/>
+      <c r="F45" s="34" t="n"/>
+      <c r="G45" s="34" t="n"/>
+      <c r="H45" s="34" t="n"/>
+      <c r="I45" s="34" t="n"/>
+      <c r="J45" s="34" t="n"/>
+      <c r="K45" s="34" t="n"/>
+      <c r="L45" s="34" t="n"/>
+      <c r="M45" s="34" t="n"/>
+      <c r="N45" s="34" t="n"/>
+      <c r="O45" s="34" t="n"/>
+      <c r="P45" s="34" t="n"/>
+      <c r="Q45" s="34" t="n"/>
     </row>
     <row r="46" ht="19" customHeight="1">
       <c r="A46" s="10">
@@ -2990,403 +3119,421 @@
       <c r="N46" s="11" t="n"/>
       <c r="O46" s="11" t="n"/>
       <c r="P46" s="11" t="n"/>
+      <c r="Q46" s="11" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="12" t="inlineStr">
         <is>
+          <t>Name: _____________________________          Grade &amp; Section: __________________</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="C47" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="C47" s="14" t="n"/>
-      <c r="D47" s="14" t="n"/>
-      <c r="E47" s="14" t="n"/>
-      <c r="F47" s="14" t="n"/>
-      <c r="G47" s="15" t="inlineStr">
+      <c r="D47" s="15" t="n"/>
+      <c r="E47" s="15" t="n"/>
+      <c r="F47" s="15" t="n"/>
+      <c r="G47" s="15" t="n"/>
+      <c r="H47" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="H47" s="14" t="n"/>
-      <c r="I47" s="14" t="n"/>
-      <c r="J47" s="14" t="n"/>
-      <c r="K47" s="14" t="n"/>
-      <c r="L47" s="14" t="n"/>
-      <c r="M47" s="14" t="n"/>
-      <c r="N47" s="13" t="inlineStr">
+      <c r="I47" s="15" t="n"/>
+      <c r="J47" s="15" t="n"/>
+      <c r="K47" s="15" t="n"/>
+      <c r="L47" s="15" t="n"/>
+      <c r="M47" s="15" t="n"/>
+      <c r="N47" s="15" t="n"/>
+      <c r="O47" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="O47" s="14" t="n"/>
-      <c r="P47" s="16" t="inlineStr">
-        <is>
-          <t>Checked and verified by:                    ENGR. PHILIP JAYSON L. LESTOJAS</t>
+      <c r="P47" s="15" t="n"/>
+      <c r="Q47" s="17" t="inlineStr">
+        <is>
+          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="17" t="n">
+      <c r="A48" s="18" t="n"/>
+      <c r="B48" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B48" s="18">
+      <c r="C48" s="20">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="C48" s="18">
+      <c r="D48" s="20">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="D48" s="18">
+      <c r="E48" s="20">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="E48" s="18">
+      <c r="F48" s="20">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="F48" s="18">
+      <c r="G48" s="20">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="G48" s="19">
+      <c r="H48" s="21">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="H48" s="18">
+      <c r="I48" s="20">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="I48" s="18">
+      <c r="J48" s="20">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="J48" s="18">
+      <c r="K48" s="20">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="K48" s="18">
+      <c r="L48" s="20">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="L48" s="18">
+      <c r="M48" s="20">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="M48" s="18">
+      <c r="N48" s="20">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
-      <c r="N48" s="7" t="n"/>
-      <c r="O48" s="20">
+      <c r="O48" s="7" t="n"/>
+      <c r="P48" s="22">
         <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
-      <c r="P48" s="21" t="n"/>
+      <c r="Q48" s="23" t="n"/>
     </row>
     <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="17" t="n">
+      <c r="A49" s="18" t="n"/>
+      <c r="B49" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B49" s="18">
+      <c r="C49" s="20">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="C49" s="18">
+      <c r="D49" s="20">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="D49" s="18">
+      <c r="E49" s="20">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="E49" s="18">
+      <c r="F49" s="20">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="F49" s="18">
+      <c r="G49" s="20">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="G49" s="19">
+      <c r="H49" s="21">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="H49" s="18">
+      <c r="I49" s="20">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="I49" s="18">
+      <c r="J49" s="20">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="J49" s="18">
+      <c r="K49" s="20">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="K49" s="18">
+      <c r="L49" s="20">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="L49" s="18">
+      <c r="M49" s="20">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="M49" s="18">
+      <c r="N49" s="20">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
-      <c r="N49" s="7" t="n"/>
-      <c r="O49" s="20">
+      <c r="O49" s="7" t="n"/>
+      <c r="P49" s="22">
         <f>"/ "&amp;Setup!$E$8</f>
         <v/>
       </c>
-      <c r="P49" s="21" t="n"/>
+      <c r="Q49" s="23" t="n"/>
     </row>
     <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="17" t="n">
+      <c r="A50" s="18" t="n"/>
+      <c r="B50" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B50" s="18">
+      <c r="C50" s="20">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="C50" s="18">
+      <c r="D50" s="20">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="D50" s="18">
+      <c r="E50" s="20">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="E50" s="18">
+      <c r="F50" s="20">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="F50" s="18">
+      <c r="G50" s="20">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="G50" s="19">
+      <c r="H50" s="21">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="H50" s="18">
+      <c r="I50" s="20">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="I50" s="18">
+      <c r="J50" s="20">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="J50" s="18">
+      <c r="K50" s="20">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="K50" s="18">
+      <c r="L50" s="20">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="L50" s="18">
+      <c r="M50" s="20">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="M50" s="18">
+      <c r="N50" s="20">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
-      <c r="N50" s="7" t="n"/>
-      <c r="O50" s="20">
+      <c r="O50" s="7" t="n"/>
+      <c r="P50" s="22">
         <f>"/ "&amp;Setup!$E$9</f>
         <v/>
       </c>
-      <c r="P50" s="21" t="n"/>
+      <c r="Q50" s="23" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="17" t="n">
+      <c r="A51" s="18" t="n"/>
+      <c r="B51" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B51" s="18">
+      <c r="C51" s="20">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="C51" s="18">
+      <c r="D51" s="20">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="D51" s="18">
+      <c r="E51" s="20">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="E51" s="18">
+      <c r="F51" s="20">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="F51" s="18">
+      <c r="G51" s="20">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="G51" s="19">
+      <c r="H51" s="21">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="H51" s="18">
+      <c r="I51" s="20">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="I51" s="18">
+      <c r="J51" s="20">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="J51" s="18">
+      <c r="K51" s="20">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="K51" s="18">
+      <c r="L51" s="20">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="L51" s="18">
+      <c r="M51" s="20">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="M51" s="18">
+      <c r="N51" s="20">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
-      <c r="N51" s="7" t="n"/>
-      <c r="O51" s="20">
+      <c r="O51" s="7" t="n"/>
+      <c r="P51" s="22">
         <f>"/ "&amp;Setup!$E$10</f>
         <v/>
       </c>
-      <c r="P51" s="21" t="n"/>
+      <c r="Q51" s="23" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="17" t="n">
+      <c r="A52" s="18" t="n"/>
+      <c r="B52" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B52" s="18">
+      <c r="C52" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="C52" s="18">
+      <c r="D52" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="D52" s="18">
+      <c r="E52" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="E52" s="18">
+      <c r="F52" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="F52" s="18">
+      <c r="G52" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="G52" s="19">
+      <c r="H52" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="H52" s="18">
+      <c r="I52" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="I52" s="18">
+      <c r="J52" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="J52" s="18">
+      <c r="K52" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="K52" s="18">
+      <c r="L52" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="L52" s="18">
+      <c r="M52" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="M52" s="18">
+      <c r="N52" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="N52" s="7" t="n"/>
-      <c r="O52" s="20">
+      <c r="O52" s="7" t="n"/>
+      <c r="P52" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="P52" s="21" t="n"/>
+      <c r="Q52" s="23" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="22" t="inlineStr">
+      <c r="A53" s="28" t="n"/>
+      <c r="B53" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="B53" s="23" t="n"/>
-      <c r="C53" s="23" t="n"/>
-      <c r="D53" s="23" t="n"/>
-      <c r="E53" s="23" t="n"/>
-      <c r="F53" s="23" t="n"/>
-      <c r="G53" s="23" t="n"/>
-      <c r="H53" s="23" t="n"/>
-      <c r="I53" s="23" t="n"/>
-      <c r="J53" s="23" t="n"/>
-      <c r="K53" s="23" t="n"/>
-      <c r="L53" s="23" t="n"/>
-      <c r="M53" s="23" t="n"/>
-      <c r="N53" s="24" t="n"/>
-      <c r="O53" s="25">
+      <c r="C53" s="30" t="n"/>
+      <c r="D53" s="30" t="n"/>
+      <c r="E53" s="30" t="n"/>
+      <c r="F53" s="30" t="n"/>
+      <c r="G53" s="30" t="n"/>
+      <c r="H53" s="30" t="n"/>
+      <c r="I53" s="30" t="n"/>
+      <c r="J53" s="30" t="n"/>
+      <c r="K53" s="30" t="n"/>
+      <c r="L53" s="30" t="n"/>
+      <c r="M53" s="30" t="n"/>
+      <c r="N53" s="30" t="n"/>
+      <c r="O53" s="31" t="n"/>
+      <c r="P53" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="P53" s="26" t="n"/>
+      <c r="Q53" s="33" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="A8:M8"/>
-    <mergeCell ref="N47:O47"/>
-    <mergeCell ref="A17:M17"/>
-    <mergeCell ref="G29:M29"/>
-    <mergeCell ref="A35:M35"/>
-    <mergeCell ref="G20:M20"/>
-    <mergeCell ref="A53:M53"/>
-    <mergeCell ref="G47:M47"/>
-    <mergeCell ref="A19:P19"/>
-    <mergeCell ref="A10:P10"/>
-    <mergeCell ref="A28:P28"/>
-    <mergeCell ref="A44:M44"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="P47:P53"/>
-    <mergeCell ref="G2:M2"/>
-    <mergeCell ref="G11:M11"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="P20:P26"/>
-    <mergeCell ref="P38:P44"/>
-    <mergeCell ref="P29:P35"/>
-    <mergeCell ref="G38:M38"/>
-    <mergeCell ref="A46:P46"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="A37:P37"/>
-    <mergeCell ref="A26:M26"/>
-    <mergeCell ref="P2:P8"/>
-    <mergeCell ref="P11:P17"/>
+  <mergeCells count="42">
+    <mergeCell ref="H47:N47"/>
+    <mergeCell ref="Q38:Q44"/>
+    <mergeCell ref="Q29:Q35"/>
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A20:A26"/>
+    <mergeCell ref="Q2:Q8"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="Q11:Q17"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="B35:N35"/>
+    <mergeCell ref="C47:G47"/>
+    <mergeCell ref="B26:N26"/>
+    <mergeCell ref="A29:A35"/>
+    <mergeCell ref="A47:A53"/>
+    <mergeCell ref="H29:N29"/>
+    <mergeCell ref="A38:A44"/>
+    <mergeCell ref="H20:N20"/>
+    <mergeCell ref="H38:N38"/>
+    <mergeCell ref="A37:Q37"/>
+    <mergeCell ref="A46:Q46"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="Q47:Q53"/>
+    <mergeCell ref="O47:P47"/>
+    <mergeCell ref="A11:A17"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="B8:N8"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="H2:N2"/>
+    <mergeCell ref="B17:N17"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="H11:N11"/>
+    <mergeCell ref="B44:N44"/>
+    <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="Q20:Q26"/>
+    <mergeCell ref="B53:N53"/>
+    <mergeCell ref="A19:Q19"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
@@ -3422,364 +3569,364 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="35" t="inlineStr">
         <is>
           <t>What each dimension measures</t>
         </is>
       </c>
-      <c r="B4" s="29" t="n"/>
+      <c r="B4" s="36" t="n"/>
     </row>
     <row r="5" ht="33" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="37" t="inlineStr">
         <is>
           <t>Final Answer  —  Did you land the correct result, properly expressed? Correct value(s), units, and significant figures. This is the ONLY place units and sig figs are judged.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>Concept &amp; Execution  —  Do you understand the physics and can you carry it out? Right principle/equation (concept) + correct substitution, algebra, and method (execution) + clear, ordered, labeled work (communication). Graded on process, using Error-Carried-Forward.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>Grading rules (apply before scoring)</t>
         </is>
       </c>
-      <c r="B8" s="29" t="n"/>
+      <c r="B8" s="36" t="n"/>
     </row>
     <row r="9" ht="33" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>1.  Score each column on its own descriptor; never penalize the same flaw twice. Units/sig-fig issues affect only Final Answer.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>2.  Error-Carried-Forward (ECF): judge each step against the student's own prior results, not the answer key.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="33" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>3.  Consistency (default): the two columns should tell the same story — strong process usually accompanies a correct answer.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="33" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="37" t="inlineStr">
         <is>
           <t>4.  ECF override: if the ONLY defect is a single arithmetic/transcription slip and every later step is correct under ECF, score Concept &amp; Execution on process merit (it may reach the top band) even though the final answer is wrong.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="37" t="inlineStr">
         <is>
           <t>5.  Answer only / no work shown: score Final Answer on merit; Concept &amp; Execution = 0.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t>6.  Blank: 0 / 0.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="35" t="inlineStr">
         <is>
           <t>TYPE A — Single-unknown (Total 5)</t>
         </is>
       </c>
-      <c r="B16" s="29" t="n"/>
+      <c r="B16" s="36" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="38" t="inlineStr">
         <is>
           <t>Final Answer (0–2)</t>
         </is>
       </c>
-      <c r="B17" s="32" t="inlineStr">
+      <c r="B17" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
-      <c r="A18" s="33" t="inlineStr">
+      <c r="A18" s="40" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B18" s="34" t="inlineStr">
+      <c r="B18" s="41" t="inlineStr">
         <is>
           <t>Correct value, correct units, appropriate significant figures.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1">
-      <c r="A19" s="33" t="inlineStr">
+      <c r="A19" s="40" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B19" s="34" t="inlineStr">
+      <c r="B19" s="41" t="inlineStr">
         <is>
           <t>Correct value but units/sig figs wrong, OR a single arithmetic slip giving a near-correct value.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1">
-      <c r="A20" s="33" t="inlineStr">
+      <c r="A20" s="40" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B20" s="34" t="inlineStr">
+      <c r="B20" s="41" t="inlineStr">
         <is>
           <t>Incorrect, or blank.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="38" t="inlineStr">
         <is>
           <t>Concept &amp; Execution (0–3)</t>
         </is>
       </c>
-      <c r="B21" s="32" t="inlineStr">
+      <c r="B21" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1">
-      <c r="A22" s="33" t="inlineStr">
+      <c r="A22" s="40" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B22" s="34" t="inlineStr">
+      <c r="B22" s="41" t="inlineStr">
         <is>
           <t>Correct principle/equation; substitution and algebra correct; work clear and complete.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="A23" s="33" t="inlineStr">
+      <c r="A23" s="40" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B23" s="34" t="inlineStr">
+      <c r="B23" s="41" t="inlineStr">
         <is>
           <t>Correct principle; essentially right, with a minor execution slip or sparse-but-followable steps.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="A24" s="33" t="inlineStr">
+      <c r="A24" s="40" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B24" s="34" t="inlineStr">
+      <c r="B24" s="41" t="inlineStr">
         <is>
           <t>Relevant concept present, but undermined by a wrong equation or a substantive execution error.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="33" t="inlineStr">
+      <c r="A25" s="40" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B25" s="34" t="inlineStr">
+      <c r="B25" s="41" t="inlineStr">
         <is>
           <t>Wrong concept, or no meaningful work.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="35" t="inlineStr">
         <is>
           <t>TYPE B — Multi-step / multi-unknown (Total 10)</t>
         </is>
       </c>
-      <c r="B27" s="29" t="n"/>
+      <c r="B27" s="36" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="38" t="inlineStr">
         <is>
           <t>Final Answer (0–4)</t>
         </is>
       </c>
-      <c r="B28" s="32" t="inlineStr">
+      <c r="B28" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="29" ht="19" customHeight="1">
-      <c r="A29" s="33" t="inlineStr">
+      <c r="A29" s="40" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B29" s="34" t="inlineStr">
+      <c r="B29" s="41" t="inlineStr">
         <is>
           <t>Every required final value correct, with correct units.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="33" t="inlineStr">
+      <c r="A30" s="40" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B30" s="34" t="inlineStr">
+      <c r="B30" s="41" t="inlineStr">
         <is>
           <t>All but one correct; the single miss is minor (units, sig figs, or one small slip).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="19" customHeight="1">
-      <c r="A31" s="33" t="inlineStr">
+      <c r="A31" s="40" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B31" s="34" t="inlineStr">
+      <c r="B31" s="41" t="inlineStr">
         <is>
           <t>Roughly half the values correct.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="33" t="inlineStr">
+      <c r="A32" s="40" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B32" s="34" t="inlineStr">
+      <c r="B32" s="41" t="inlineStr">
         <is>
           <t>One value correct, or most contain significant errors.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="33" t="inlineStr">
+      <c r="A33" s="40" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B33" s="34" t="inlineStr">
+      <c r="B33" s="41" t="inlineStr">
         <is>
           <t>No correct values, or blank.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="31" t="inlineStr">
+      <c r="A34" s="38" t="inlineStr">
         <is>
           <t>Concept &amp; Execution (0–6)</t>
         </is>
       </c>
-      <c r="B34" s="32" t="inlineStr">
+      <c r="B34" s="39" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="35" ht="34" customHeight="1">
-      <c r="A35" s="33" t="inlineStr">
+      <c r="A35" s="40" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B35" s="34" t="inlineStr">
+      <c r="B35" s="41" t="inlineStr">
         <is>
           <t>Correct principle at EVERY step; all substitution, algebra, and units correct (ECF); logically ordered, labeled, easy to follow.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="34" customHeight="1">
-      <c r="A36" s="33" t="inlineStr">
+      <c r="A36" s="40" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B36" s="34" t="inlineStr">
+      <c r="B36" s="41" t="inlineStr">
         <is>
           <t>Correct principles and method throughout; at most one trivial slip or slightly sparse justification — physics fully sound.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="34" customHeight="1">
-      <c r="A37" s="33" t="inlineStr">
+      <c r="A37" s="40" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B37" s="34" t="inlineStr">
+      <c r="B37" s="41" t="inlineStr">
         <is>
           <t>Correct approach on the main steps, but ONE real execution error or one wrong/missing equation; work still followable.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="34" customHeight="1">
-      <c r="A38" s="33" t="inlineStr">
+      <c r="A38" s="40" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B38" s="34" t="inlineStr">
+      <c r="B38" s="41" t="inlineStr">
         <is>
           <t>Correct on some steps, but a wrong principle on a major step and/or several execution errors; reasoning has gaps.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="19" customHeight="1">
-      <c r="A39" s="33" t="inlineStr">
+      <c r="A39" s="40" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B39" s="34" t="inlineStr">
+      <c r="B39" s="41" t="inlineStr">
         <is>
           <t>Mostly incorrect method; more than a token of correct physics but hard to follow.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="19" customHeight="1">
-      <c r="A40" s="33" t="inlineStr">
+      <c r="A40" s="40" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B40" s="34" t="inlineStr">
+      <c r="B40" s="41" t="inlineStr">
         <is>
           <t>Little relevant physics; fundamentally the wrong approach with only a token correct fragment.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="19" customHeight="1">
-      <c r="A41" s="33" t="inlineStr">
+      <c r="A41" s="40" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="B41" s="34" t="inlineStr">
+      <c r="B41" s="41" t="inlineStr">
         <is>
           <t>No meaningful work, or blank.</t>
         </is>

</xml_diff>

<commit_message>
Signature block: label + two blank signing lines + name (explicit breaks, no resize)
</commit_message>
<xml_diff>
--- a/grading_rubric_A4.xlsx
+++ b/grading_rubric_A4.xlsx
@@ -1110,7 +1110,8 @@
       <c r="P2" s="15" t="n"/>
       <c r="Q2" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t>Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1521,8 @@
       <c r="P11" s="15" t="n"/>
       <c r="Q11" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t>Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1932,8 @@
       <c r="P20" s="15" t="n"/>
       <c r="Q20" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t>Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2343,8 @@
       <c r="P29" s="15" t="n"/>
       <c r="Q29" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t>Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2754,8 @@
       <c r="P38" s="15" t="n"/>
       <c r="Q38" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t>Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3165,8 @@
       <c r="P47" s="15" t="n"/>
       <c r="Q47" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:                                        ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t>Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix signature signing gap: force xml:space=preserve so blank lines render in Excel
</commit_message>
<xml_diff>
--- a/grading_rubric_A4.xlsx
+++ b/grading_rubric_A4.xlsx
@@ -1110,8 +1110,8 @@
       <c r="P2" s="15" t="n"/>
       <c r="Q2" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:
-ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t xml:space="preserve">Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
     </row>
@@ -1521,8 +1521,8 @@
       <c r="P11" s="15" t="n"/>
       <c r="Q11" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:
-ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t xml:space="preserve">Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
     </row>
@@ -1932,8 +1932,8 @@
       <c r="P20" s="15" t="n"/>
       <c r="Q20" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:
-ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t xml:space="preserve">Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
     </row>
@@ -2343,8 +2343,8 @@
       <c r="P29" s="15" t="n"/>
       <c r="Q29" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:
-ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t xml:space="preserve">Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
     </row>
@@ -2754,8 +2754,8 @@
       <c r="P38" s="15" t="n"/>
       <c r="Q38" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:
-ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t xml:space="preserve">Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
     </row>
@@ -3165,8 +3165,8 @@
       <c r="P47" s="15" t="n"/>
       <c r="Q47" s="17" t="inlineStr">
         <is>
-          <t>Checked and verified by:
-ENGR. PHILIP JAYSON L. LESTOJAS</t>
+          <t xml:space="preserve">Checked and verified by:
+ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add spacer row between dashed cut line and next slip title
</commit_message>
<xml_diff>
--- a/grading_rubric_A4.xlsx
+++ b/grading_rubric_A4.xlsx
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1441,7 +1441,7 @@
       </c>
       <c r="Q8" s="33" t="n"/>
     </row>
-    <row r="9" ht="9" customHeight="1">
+    <row r="9" ht="7" customHeight="1">
       <c r="A9" s="34" t="n"/>
       <c r="B9" s="34" t="n"/>
       <c r="C9" s="34" t="n"/>
@@ -1460,188 +1460,129 @@
       <c r="P9" s="34" t="n"/>
       <c r="Q9" s="34" t="n"/>
     </row>
-    <row r="10" ht="19" customHeight="1">
-      <c r="A10" s="10">
+    <row r="10" ht="11" customHeight="1"/>
+    <row r="11" ht="19" customHeight="1">
+      <c r="A11" s="10">
         <f>Setup!$B$3&amp;"  •  Rubric: Problem Set "&amp;Setup!$B$4</f>
         <v/>
       </c>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
-      <c r="H10" s="11" t="n"/>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="11" t="n"/>
-      <c r="K10" s="11" t="n"/>
-      <c r="L10" s="11" t="n"/>
-      <c r="M10" s="11" t="n"/>
-      <c r="N10" s="11" t="n"/>
-      <c r="O10" s="11" t="n"/>
-      <c r="P10" s="11" t="n"/>
-      <c r="Q10" s="11" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="11" t="n"/>
+      <c r="K11" s="11" t="n"/>
+      <c r="L11" s="11" t="n"/>
+      <c r="M11" s="11" t="n"/>
+      <c r="N11" s="11" t="n"/>
+      <c r="O11" s="11" t="n"/>
+      <c r="P11" s="11" t="n"/>
+      <c r="Q11" s="11" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Name: _____________________________          Grade &amp; Section: __________________</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="15" t="n"/>
-      <c r="H11" s="16" t="inlineStr">
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="I11" s="15" t="n"/>
-      <c r="J11" s="15" t="n"/>
-      <c r="K11" s="15" t="n"/>
-      <c r="L11" s="15" t="n"/>
-      <c r="M11" s="15" t="n"/>
-      <c r="N11" s="15" t="n"/>
-      <c r="O11" s="14" t="inlineStr">
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="15" t="n"/>
+      <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="15" t="n"/>
+      <c r="N12" s="15" t="n"/>
+      <c r="O12" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="P11" s="15" t="n"/>
-      <c r="Q11" s="17" t="inlineStr">
+      <c r="P12" s="15" t="n"/>
+      <c r="Q12" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Checked and verified by:
 ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="18" t="n"/>
-      <c r="B12" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="20">
-        <f>IF(0&lt;=Setup!$C$7,0,"")</f>
-        <v/>
-      </c>
-      <c r="D12" s="20">
-        <f>IF(1&lt;=Setup!$C$7,1,"")</f>
-        <v/>
-      </c>
-      <c r="E12" s="20">
-        <f>IF(2&lt;=Setup!$C$7,2,"")</f>
-        <v/>
-      </c>
-      <c r="F12" s="20">
-        <f>IF(3&lt;=Setup!$C$7,3,"")</f>
-        <v/>
-      </c>
-      <c r="G12" s="20">
-        <f>IF(4&lt;=Setup!$C$7,4,"")</f>
-        <v/>
-      </c>
-      <c r="H12" s="21">
-        <f>IF(0&lt;=Setup!$D$7,0,"")</f>
-        <v/>
-      </c>
-      <c r="I12" s="20">
-        <f>IF(1&lt;=Setup!$D$7,1,"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="20">
-        <f>IF(2&lt;=Setup!$D$7,2,"")</f>
-        <v/>
-      </c>
-      <c r="K12" s="20">
-        <f>IF(3&lt;=Setup!$D$7,3,"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="20">
-        <f>IF(4&lt;=Setup!$D$7,4,"")</f>
-        <v/>
-      </c>
-      <c r="M12" s="20">
-        <f>IF(5&lt;=Setup!$D$7,5,"")</f>
-        <v/>
-      </c>
-      <c r="N12" s="20">
-        <f>IF(6&lt;=Setup!$D$7,6,"")</f>
-        <v/>
-      </c>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="22">
-        <f>"/ "&amp;Setup!$E$7</f>
-        <v/>
-      </c>
-      <c r="Q12" s="23" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="18" t="n"/>
       <c r="B13" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C13" s="20">
-        <f>IF(0&lt;=Setup!$C$8,0,"")</f>
+        <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
       <c r="D13" s="20">
-        <f>IF(1&lt;=Setup!$C$8,1,"")</f>
+        <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
       <c r="E13" s="20">
-        <f>IF(2&lt;=Setup!$C$8,2,"")</f>
+        <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
       <c r="F13" s="20">
-        <f>IF(3&lt;=Setup!$C$8,3,"")</f>
+        <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
       <c r="G13" s="20">
-        <f>IF(4&lt;=Setup!$C$8,4,"")</f>
+        <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
       <c r="H13" s="21">
-        <f>IF(0&lt;=Setup!$D$8,0,"")</f>
+        <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
       <c r="I13" s="20">
-        <f>IF(1&lt;=Setup!$D$8,1,"")</f>
+        <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
       <c r="J13" s="20">
-        <f>IF(2&lt;=Setup!$D$8,2,"")</f>
+        <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
       <c r="K13" s="20">
-        <f>IF(3&lt;=Setup!$D$8,3,"")</f>
+        <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
       <c r="L13" s="20">
-        <f>IF(4&lt;=Setup!$D$8,4,"")</f>
+        <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
       <c r="M13" s="20">
-        <f>IF(5&lt;=Setup!$D$8,5,"")</f>
+        <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
       <c r="N13" s="20">
-        <f>IF(6&lt;=Setup!$D$8,6,"")</f>
+        <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="O13" s="7" t="n"/>
       <c r="P13" s="22">
-        <f>"/ "&amp;Setup!$E$8</f>
+        <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
       <c r="Q13" s="23" t="n"/>
@@ -1649,59 +1590,59 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="18" t="n"/>
       <c r="B14" s="19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" s="20">
-        <f>IF(0&lt;=Setup!$C$9,0,"")</f>
+        <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
       <c r="D14" s="20">
-        <f>IF(1&lt;=Setup!$C$9,1,"")</f>
+        <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
       <c r="E14" s="20">
-        <f>IF(2&lt;=Setup!$C$9,2,"")</f>
+        <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
       <c r="F14" s="20">
-        <f>IF(3&lt;=Setup!$C$9,3,"")</f>
+        <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
       <c r="G14" s="20">
-        <f>IF(4&lt;=Setup!$C$9,4,"")</f>
+        <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
       <c r="H14" s="21">
-        <f>IF(0&lt;=Setup!$D$9,0,"")</f>
+        <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
       <c r="I14" s="20">
-        <f>IF(1&lt;=Setup!$D$9,1,"")</f>
+        <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
       <c r="J14" s="20">
-        <f>IF(2&lt;=Setup!$D$9,2,"")</f>
+        <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>IF(3&lt;=Setup!$D$9,3,"")</f>
+        <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>IF(4&lt;=Setup!$D$9,4,"")</f>
+        <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
       <c r="M14" s="20">
-        <f>IF(5&lt;=Setup!$D$9,5,"")</f>
+        <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
       <c r="N14" s="20">
-        <f>IF(6&lt;=Setup!$D$9,6,"")</f>
+        <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="O14" s="7" t="n"/>
       <c r="P14" s="22">
-        <f>"/ "&amp;Setup!$E$9</f>
+        <f>"/ "&amp;Setup!$E$8</f>
         <v/>
       </c>
       <c r="Q14" s="23" t="n"/>
@@ -1709,410 +1650,351 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="18" t="n"/>
       <c r="B15" s="19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C15" s="20">
-        <f>IF(0&lt;=Setup!$C$10,0,"")</f>
+        <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
       <c r="D15" s="20">
-        <f>IF(1&lt;=Setup!$C$10,1,"")</f>
+        <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
       <c r="E15" s="20">
-        <f>IF(2&lt;=Setup!$C$10,2,"")</f>
+        <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>IF(3&lt;=Setup!$C$10,3,"")</f>
+        <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
       <c r="G15" s="20">
-        <f>IF(4&lt;=Setup!$C$10,4,"")</f>
+        <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
       <c r="H15" s="21">
-        <f>IF(0&lt;=Setup!$D$10,0,"")</f>
+        <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
       <c r="I15" s="20">
-        <f>IF(1&lt;=Setup!$D$10,1,"")</f>
+        <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
       <c r="J15" s="20">
-        <f>IF(2&lt;=Setup!$D$10,2,"")</f>
+        <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
       <c r="K15" s="20">
-        <f>IF(3&lt;=Setup!$D$10,3,"")</f>
+        <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
       <c r="L15" s="20">
-        <f>IF(4&lt;=Setup!$D$10,4,"")</f>
+        <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
       <c r="M15" s="20">
-        <f>IF(5&lt;=Setup!$D$10,5,"")</f>
+        <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
       <c r="N15" s="20">
-        <f>IF(6&lt;=Setup!$D$10,6,"")</f>
+        <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
       <c r="O15" s="7" t="n"/>
       <c r="P15" s="22">
-        <f>"/ "&amp;Setup!$E$10</f>
+        <f>"/ "&amp;Setup!$E$9</f>
         <v/>
       </c>
       <c r="Q15" s="23" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="18" t="n"/>
-      <c r="B16" s="24" t="n">
+      <c r="B16" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="20">
+        <f>IF(0&lt;=Setup!$C$10,0,"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="20">
+        <f>IF(1&lt;=Setup!$C$10,1,"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="20">
+        <f>IF(2&lt;=Setup!$C$10,2,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="20">
+        <f>IF(3&lt;=Setup!$C$10,3,"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="20">
+        <f>IF(4&lt;=Setup!$C$10,4,"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="21">
+        <f>IF(0&lt;=Setup!$D$10,0,"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="20">
+        <f>IF(1&lt;=Setup!$D$10,1,"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="20">
+        <f>IF(2&lt;=Setup!$D$10,2,"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="20">
+        <f>IF(3&lt;=Setup!$D$10,3,"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="20">
+        <f>IF(4&lt;=Setup!$D$10,4,"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="20">
+        <f>IF(5&lt;=Setup!$D$10,5,"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="20">
+        <f>IF(6&lt;=Setup!$D$10,6,"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" s="22">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="Q16" s="23" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="18" t="n"/>
+      <c r="B17" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="C16" s="25">
+      <c r="C17" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="D16" s="25">
+      <c r="D17" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="E16" s="25">
+      <c r="E17" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="F16" s="25">
+      <c r="F17" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="G16" s="25">
+      <c r="G17" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="H16" s="26">
+      <c r="H17" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="I16" s="25">
+      <c r="I17" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="J16" s="25">
+      <c r="J17" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="K16" s="25">
+      <c r="K17" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="L16" s="25">
+      <c r="L17" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="M16" s="25">
+      <c r="M17" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="N16" s="25">
+      <c r="N17" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="O16" s="7" t="n"/>
-      <c r="P16" s="27">
+      <c r="O17" s="7" t="n"/>
+      <c r="P17" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="Q16" s="23" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="28" t="n"/>
-      <c r="B17" s="29" t="inlineStr">
+      <c r="Q17" s="23" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="28" t="n"/>
+      <c r="B18" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="C17" s="30" t="n"/>
-      <c r="D17" s="30" t="n"/>
-      <c r="E17" s="30" t="n"/>
-      <c r="F17" s="30" t="n"/>
-      <c r="G17" s="30" t="n"/>
-      <c r="H17" s="30" t="n"/>
-      <c r="I17" s="30" t="n"/>
-      <c r="J17" s="30" t="n"/>
-      <c r="K17" s="30" t="n"/>
-      <c r="L17" s="30" t="n"/>
-      <c r="M17" s="30" t="n"/>
-      <c r="N17" s="30" t="n"/>
-      <c r="O17" s="31" t="n"/>
-      <c r="P17" s="32">
+      <c r="C18" s="30" t="n"/>
+      <c r="D18" s="30" t="n"/>
+      <c r="E18" s="30" t="n"/>
+      <c r="F18" s="30" t="n"/>
+      <c r="G18" s="30" t="n"/>
+      <c r="H18" s="30" t="n"/>
+      <c r="I18" s="30" t="n"/>
+      <c r="J18" s="30" t="n"/>
+      <c r="K18" s="30" t="n"/>
+      <c r="L18" s="30" t="n"/>
+      <c r="M18" s="30" t="n"/>
+      <c r="N18" s="30" t="n"/>
+      <c r="O18" s="31" t="n"/>
+      <c r="P18" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="Q17" s="33" t="n"/>
-    </row>
-    <row r="18" ht="9" customHeight="1">
-      <c r="A18" s="34" t="n"/>
-      <c r="B18" s="34" t="n"/>
-      <c r="C18" s="34" t="n"/>
-      <c r="D18" s="34" t="n"/>
-      <c r="E18" s="34" t="n"/>
-      <c r="F18" s="34" t="n"/>
-      <c r="G18" s="34" t="n"/>
-      <c r="H18" s="34" t="n"/>
-      <c r="I18" s="34" t="n"/>
-      <c r="J18" s="34" t="n"/>
-      <c r="K18" s="34" t="n"/>
-      <c r="L18" s="34" t="n"/>
-      <c r="M18" s="34" t="n"/>
-      <c r="N18" s="34" t="n"/>
-      <c r="O18" s="34" t="n"/>
-      <c r="P18" s="34" t="n"/>
-      <c r="Q18" s="34" t="n"/>
-    </row>
-    <row r="19" ht="19" customHeight="1">
-      <c r="A19" s="10">
+      <c r="Q18" s="33" t="n"/>
+    </row>
+    <row r="19" ht="7" customHeight="1">
+      <c r="A19" s="34" t="n"/>
+      <c r="B19" s="34" t="n"/>
+      <c r="C19" s="34" t="n"/>
+      <c r="D19" s="34" t="n"/>
+      <c r="E19" s="34" t="n"/>
+      <c r="F19" s="34" t="n"/>
+      <c r="G19" s="34" t="n"/>
+      <c r="H19" s="34" t="n"/>
+      <c r="I19" s="34" t="n"/>
+      <c r="J19" s="34" t="n"/>
+      <c r="K19" s="34" t="n"/>
+      <c r="L19" s="34" t="n"/>
+      <c r="M19" s="34" t="n"/>
+      <c r="N19" s="34" t="n"/>
+      <c r="O19" s="34" t="n"/>
+      <c r="P19" s="34" t="n"/>
+      <c r="Q19" s="34" t="n"/>
+    </row>
+    <row r="20" ht="11" customHeight="1"/>
+    <row r="21" ht="19" customHeight="1">
+      <c r="A21" s="10">
         <f>Setup!$B$3&amp;"  •  Rubric: Problem Set "&amp;Setup!$B$4</f>
         <v/>
       </c>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
-      <c r="H19" s="11" t="n"/>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="n"/>
-      <c r="K19" s="11" t="n"/>
-      <c r="L19" s="11" t="n"/>
-      <c r="M19" s="11" t="n"/>
-      <c r="N19" s="11" t="n"/>
-      <c r="O19" s="11" t="n"/>
-      <c r="P19" s="11" t="n"/>
-      <c r="Q19" s="11" t="n"/>
-    </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="11" t="n"/>
+      <c r="H21" s="11" t="n"/>
+      <c r="I21" s="11" t="n"/>
+      <c r="J21" s="11" t="n"/>
+      <c r="K21" s="11" t="n"/>
+      <c r="L21" s="11" t="n"/>
+      <c r="M21" s="11" t="n"/>
+      <c r="N21" s="11" t="n"/>
+      <c r="O21" s="11" t="n"/>
+      <c r="P21" s="11" t="n"/>
+      <c r="Q21" s="11" t="n"/>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Name: _____________________________          Grade &amp; Section: __________________</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="D20" s="15" t="n"/>
-      <c r="E20" s="15" t="n"/>
-      <c r="F20" s="15" t="n"/>
-      <c r="G20" s="15" t="n"/>
-      <c r="H20" s="16" t="inlineStr">
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
+      <c r="G22" s="15" t="n"/>
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="I20" s="15" t="n"/>
-      <c r="J20" s="15" t="n"/>
-      <c r="K20" s="15" t="n"/>
-      <c r="L20" s="15" t="n"/>
-      <c r="M20" s="15" t="n"/>
-      <c r="N20" s="15" t="n"/>
-      <c r="O20" s="14" t="inlineStr">
+      <c r="I22" s="15" t="n"/>
+      <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="15" t="n"/>
+      <c r="N22" s="15" t="n"/>
+      <c r="O22" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="P20" s="15" t="n"/>
-      <c r="Q20" s="17" t="inlineStr">
+      <c r="P22" s="15" t="n"/>
+      <c r="Q22" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Checked and verified by:
 ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="18" t="n"/>
-      <c r="B21" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="20">
-        <f>IF(0&lt;=Setup!$C$7,0,"")</f>
-        <v/>
-      </c>
-      <c r="D21" s="20">
-        <f>IF(1&lt;=Setup!$C$7,1,"")</f>
-        <v/>
-      </c>
-      <c r="E21" s="20">
-        <f>IF(2&lt;=Setup!$C$7,2,"")</f>
-        <v/>
-      </c>
-      <c r="F21" s="20">
-        <f>IF(3&lt;=Setup!$C$7,3,"")</f>
-        <v/>
-      </c>
-      <c r="G21" s="20">
-        <f>IF(4&lt;=Setup!$C$7,4,"")</f>
-        <v/>
-      </c>
-      <c r="H21" s="21">
-        <f>IF(0&lt;=Setup!$D$7,0,"")</f>
-        <v/>
-      </c>
-      <c r="I21" s="20">
-        <f>IF(1&lt;=Setup!$D$7,1,"")</f>
-        <v/>
-      </c>
-      <c r="J21" s="20">
-        <f>IF(2&lt;=Setup!$D$7,2,"")</f>
-        <v/>
-      </c>
-      <c r="K21" s="20">
-        <f>IF(3&lt;=Setup!$D$7,3,"")</f>
-        <v/>
-      </c>
-      <c r="L21" s="20">
-        <f>IF(4&lt;=Setup!$D$7,4,"")</f>
-        <v/>
-      </c>
-      <c r="M21" s="20">
-        <f>IF(5&lt;=Setup!$D$7,5,"")</f>
-        <v/>
-      </c>
-      <c r="N21" s="20">
-        <f>IF(6&lt;=Setup!$D$7,6,"")</f>
-        <v/>
-      </c>
-      <c r="O21" s="7" t="n"/>
-      <c r="P21" s="22">
-        <f>"/ "&amp;Setup!$E$7</f>
-        <v/>
-      </c>
-      <c r="Q21" s="23" t="n"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="18" t="n"/>
-      <c r="B22" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C22" s="20">
-        <f>IF(0&lt;=Setup!$C$8,0,"")</f>
-        <v/>
-      </c>
-      <c r="D22" s="20">
-        <f>IF(1&lt;=Setup!$C$8,1,"")</f>
-        <v/>
-      </c>
-      <c r="E22" s="20">
-        <f>IF(2&lt;=Setup!$C$8,2,"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="20">
-        <f>IF(3&lt;=Setup!$C$8,3,"")</f>
-        <v/>
-      </c>
-      <c r="G22" s="20">
-        <f>IF(4&lt;=Setup!$C$8,4,"")</f>
-        <v/>
-      </c>
-      <c r="H22" s="21">
-        <f>IF(0&lt;=Setup!$D$8,0,"")</f>
-        <v/>
-      </c>
-      <c r="I22" s="20">
-        <f>IF(1&lt;=Setup!$D$8,1,"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="20">
-        <f>IF(2&lt;=Setup!$D$8,2,"")</f>
-        <v/>
-      </c>
-      <c r="K22" s="20">
-        <f>IF(3&lt;=Setup!$D$8,3,"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="20">
-        <f>IF(4&lt;=Setup!$D$8,4,"")</f>
-        <v/>
-      </c>
-      <c r="M22" s="20">
-        <f>IF(5&lt;=Setup!$D$8,5,"")</f>
-        <v/>
-      </c>
-      <c r="N22" s="20">
-        <f>IF(6&lt;=Setup!$D$8,6,"")</f>
-        <v/>
-      </c>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="22">
-        <f>"/ "&amp;Setup!$E$8</f>
-        <v/>
-      </c>
-      <c r="Q22" s="23" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="18" t="n"/>
       <c r="B23" s="19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C23" s="20">
-        <f>IF(0&lt;=Setup!$C$9,0,"")</f>
+        <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
       <c r="D23" s="20">
-        <f>IF(1&lt;=Setup!$C$9,1,"")</f>
+        <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
       <c r="E23" s="20">
-        <f>IF(2&lt;=Setup!$C$9,2,"")</f>
+        <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
       <c r="F23" s="20">
-        <f>IF(3&lt;=Setup!$C$9,3,"")</f>
+        <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
       <c r="G23" s="20">
-        <f>IF(4&lt;=Setup!$C$9,4,"")</f>
+        <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
       <c r="H23" s="21">
-        <f>IF(0&lt;=Setup!$D$9,0,"")</f>
+        <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
       <c r="I23" s="20">
-        <f>IF(1&lt;=Setup!$D$9,1,"")</f>
+        <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
       <c r="J23" s="20">
-        <f>IF(2&lt;=Setup!$D$9,2,"")</f>
+        <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
       <c r="K23" s="20">
-        <f>IF(3&lt;=Setup!$D$9,3,"")</f>
+        <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
       <c r="L23" s="20">
-        <f>IF(4&lt;=Setup!$D$9,4,"")</f>
+        <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
       <c r="M23" s="20">
-        <f>IF(5&lt;=Setup!$D$9,5,"")</f>
+        <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
       <c r="N23" s="20">
-        <f>IF(6&lt;=Setup!$D$9,6,"")</f>
+        <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="O23" s="7" t="n"/>
       <c r="P23" s="22">
-        <f>"/ "&amp;Setup!$E$9</f>
+        <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
       <c r="Q23" s="23" t="n"/>
@@ -2120,1426 +2002,1549 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="18" t="n"/>
       <c r="B24" s="19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C24" s="20">
-        <f>IF(0&lt;=Setup!$C$10,0,"")</f>
+        <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
       <c r="D24" s="20">
-        <f>IF(1&lt;=Setup!$C$10,1,"")</f>
+        <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
       <c r="E24" s="20">
-        <f>IF(2&lt;=Setup!$C$10,2,"")</f>
+        <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
       <c r="F24" s="20">
-        <f>IF(3&lt;=Setup!$C$10,3,"")</f>
+        <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
       <c r="G24" s="20">
-        <f>IF(4&lt;=Setup!$C$10,4,"")</f>
+        <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
       <c r="H24" s="21">
-        <f>IF(0&lt;=Setup!$D$10,0,"")</f>
+        <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
       <c r="I24" s="20">
-        <f>IF(1&lt;=Setup!$D$10,1,"")</f>
+        <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
       <c r="J24" s="20">
-        <f>IF(2&lt;=Setup!$D$10,2,"")</f>
+        <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
       <c r="K24" s="20">
-        <f>IF(3&lt;=Setup!$D$10,3,"")</f>
+        <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>IF(4&lt;=Setup!$D$10,4,"")</f>
+        <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
       <c r="M24" s="20">
-        <f>IF(5&lt;=Setup!$D$10,5,"")</f>
+        <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
       <c r="N24" s="20">
-        <f>IF(6&lt;=Setup!$D$10,6,"")</f>
+        <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
       <c r="O24" s="7" t="n"/>
       <c r="P24" s="22">
-        <f>"/ "&amp;Setup!$E$10</f>
+        <f>"/ "&amp;Setup!$E$8</f>
         <v/>
       </c>
       <c r="Q24" s="23" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="18" t="n"/>
-      <c r="B25" s="24" t="n">
+      <c r="B25" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="20">
+        <f>IF(0&lt;=Setup!$C$9,0,"")</f>
+        <v/>
+      </c>
+      <c r="D25" s="20">
+        <f>IF(1&lt;=Setup!$C$9,1,"")</f>
+        <v/>
+      </c>
+      <c r="E25" s="20">
+        <f>IF(2&lt;=Setup!$C$9,2,"")</f>
+        <v/>
+      </c>
+      <c r="F25" s="20">
+        <f>IF(3&lt;=Setup!$C$9,3,"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="20">
+        <f>IF(4&lt;=Setup!$C$9,4,"")</f>
+        <v/>
+      </c>
+      <c r="H25" s="21">
+        <f>IF(0&lt;=Setup!$D$9,0,"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="20">
+        <f>IF(1&lt;=Setup!$D$9,1,"")</f>
+        <v/>
+      </c>
+      <c r="J25" s="20">
+        <f>IF(2&lt;=Setup!$D$9,2,"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="20">
+        <f>IF(3&lt;=Setup!$D$9,3,"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="20">
+        <f>IF(4&lt;=Setup!$D$9,4,"")</f>
+        <v/>
+      </c>
+      <c r="M25" s="20">
+        <f>IF(5&lt;=Setup!$D$9,5,"")</f>
+        <v/>
+      </c>
+      <c r="N25" s="20">
+        <f>IF(6&lt;=Setup!$D$9,6,"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="7" t="n"/>
+      <c r="P25" s="22">
+        <f>"/ "&amp;Setup!$E$9</f>
+        <v/>
+      </c>
+      <c r="Q25" s="23" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="18" t="n"/>
+      <c r="B26" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="20">
+        <f>IF(0&lt;=Setup!$C$10,0,"")</f>
+        <v/>
+      </c>
+      <c r="D26" s="20">
+        <f>IF(1&lt;=Setup!$C$10,1,"")</f>
+        <v/>
+      </c>
+      <c r="E26" s="20">
+        <f>IF(2&lt;=Setup!$C$10,2,"")</f>
+        <v/>
+      </c>
+      <c r="F26" s="20">
+        <f>IF(3&lt;=Setup!$C$10,3,"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="20">
+        <f>IF(4&lt;=Setup!$C$10,4,"")</f>
+        <v/>
+      </c>
+      <c r="H26" s="21">
+        <f>IF(0&lt;=Setup!$D$10,0,"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="20">
+        <f>IF(1&lt;=Setup!$D$10,1,"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="20">
+        <f>IF(2&lt;=Setup!$D$10,2,"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="20">
+        <f>IF(3&lt;=Setup!$D$10,3,"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="20">
+        <f>IF(4&lt;=Setup!$D$10,4,"")</f>
+        <v/>
+      </c>
+      <c r="M26" s="20">
+        <f>IF(5&lt;=Setup!$D$10,5,"")</f>
+        <v/>
+      </c>
+      <c r="N26" s="20">
+        <f>IF(6&lt;=Setup!$D$10,6,"")</f>
+        <v/>
+      </c>
+      <c r="O26" s="7" t="n"/>
+      <c r="P26" s="22">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="Q26" s="23" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="18" t="n"/>
+      <c r="B27" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="C25" s="25">
+      <c r="C27" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="D25" s="25">
+      <c r="D27" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="E25" s="25">
+      <c r="E27" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="F25" s="25">
+      <c r="F27" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="G25" s="25">
+      <c r="G27" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="H25" s="26">
+      <c r="H27" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="I25" s="25">
+      <c r="I27" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="J25" s="25">
+      <c r="J27" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="K25" s="25">
+      <c r="K27" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="L25" s="25">
+      <c r="L27" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="M25" s="25">
+      <c r="M27" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="N25" s="25">
+      <c r="N27" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="O25" s="7" t="n"/>
-      <c r="P25" s="27">
+      <c r="O27" s="7" t="n"/>
+      <c r="P27" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="Q25" s="23" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="28" t="n"/>
-      <c r="B26" s="29" t="inlineStr">
+      <c r="Q27" s="23" t="n"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="28" t="n"/>
+      <c r="B28" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="C26" s="30" t="n"/>
-      <c r="D26" s="30" t="n"/>
-      <c r="E26" s="30" t="n"/>
-      <c r="F26" s="30" t="n"/>
-      <c r="G26" s="30" t="n"/>
-      <c r="H26" s="30" t="n"/>
-      <c r="I26" s="30" t="n"/>
-      <c r="J26" s="30" t="n"/>
-      <c r="K26" s="30" t="n"/>
-      <c r="L26" s="30" t="n"/>
-      <c r="M26" s="30" t="n"/>
-      <c r="N26" s="30" t="n"/>
-      <c r="O26" s="31" t="n"/>
-      <c r="P26" s="32">
+      <c r="C28" s="30" t="n"/>
+      <c r="D28" s="30" t="n"/>
+      <c r="E28" s="30" t="n"/>
+      <c r="F28" s="30" t="n"/>
+      <c r="G28" s="30" t="n"/>
+      <c r="H28" s="30" t="n"/>
+      <c r="I28" s="30" t="n"/>
+      <c r="J28" s="30" t="n"/>
+      <c r="K28" s="30" t="n"/>
+      <c r="L28" s="30" t="n"/>
+      <c r="M28" s="30" t="n"/>
+      <c r="N28" s="30" t="n"/>
+      <c r="O28" s="31" t="n"/>
+      <c r="P28" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="Q26" s="33" t="n"/>
-    </row>
-    <row r="27" ht="9" customHeight="1">
-      <c r="A27" s="34" t="n"/>
-      <c r="B27" s="34" t="n"/>
-      <c r="C27" s="34" t="n"/>
-      <c r="D27" s="34" t="n"/>
-      <c r="E27" s="34" t="n"/>
-      <c r="F27" s="34" t="n"/>
-      <c r="G27" s="34" t="n"/>
-      <c r="H27" s="34" t="n"/>
-      <c r="I27" s="34" t="n"/>
-      <c r="J27" s="34" t="n"/>
-      <c r="K27" s="34" t="n"/>
-      <c r="L27" s="34" t="n"/>
-      <c r="M27" s="34" t="n"/>
-      <c r="N27" s="34" t="n"/>
-      <c r="O27" s="34" t="n"/>
-      <c r="P27" s="34" t="n"/>
-      <c r="Q27" s="34" t="n"/>
-    </row>
-    <row r="28" ht="19" customHeight="1">
-      <c r="A28" s="10">
+      <c r="Q28" s="33" t="n"/>
+    </row>
+    <row r="29" ht="7" customHeight="1">
+      <c r="A29" s="34" t="n"/>
+      <c r="B29" s="34" t="n"/>
+      <c r="C29" s="34" t="n"/>
+      <c r="D29" s="34" t="n"/>
+      <c r="E29" s="34" t="n"/>
+      <c r="F29" s="34" t="n"/>
+      <c r="G29" s="34" t="n"/>
+      <c r="H29" s="34" t="n"/>
+      <c r="I29" s="34" t="n"/>
+      <c r="J29" s="34" t="n"/>
+      <c r="K29" s="34" t="n"/>
+      <c r="L29" s="34" t="n"/>
+      <c r="M29" s="34" t="n"/>
+      <c r="N29" s="34" t="n"/>
+      <c r="O29" s="34" t="n"/>
+      <c r="P29" s="34" t="n"/>
+      <c r="Q29" s="34" t="n"/>
+    </row>
+    <row r="30" ht="11" customHeight="1"/>
+    <row r="31" ht="19" customHeight="1">
+      <c r="A31" s="10">
         <f>Setup!$B$3&amp;"  •  Rubric: Problem Set "&amp;Setup!$B$4</f>
         <v/>
       </c>
-      <c r="B28" s="11" t="n"/>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="11" t="n"/>
-      <c r="E28" s="11" t="n"/>
-      <c r="F28" s="11" t="n"/>
-      <c r="G28" s="11" t="n"/>
-      <c r="H28" s="11" t="n"/>
-      <c r="I28" s="11" t="n"/>
-      <c r="J28" s="11" t="n"/>
-      <c r="K28" s="11" t="n"/>
-      <c r="L28" s="11" t="n"/>
-      <c r="M28" s="11" t="n"/>
-      <c r="N28" s="11" t="n"/>
-      <c r="O28" s="11" t="n"/>
-      <c r="P28" s="11" t="n"/>
-      <c r="Q28" s="11" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="11" t="n"/>
+      <c r="I31" s="11" t="n"/>
+      <c r="J31" s="11" t="n"/>
+      <c r="K31" s="11" t="n"/>
+      <c r="L31" s="11" t="n"/>
+      <c r="M31" s="11" t="n"/>
+      <c r="N31" s="11" t="n"/>
+      <c r="O31" s="11" t="n"/>
+      <c r="P31" s="11" t="n"/>
+      <c r="Q31" s="11" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>Name: _____________________________          Grade &amp; Section: __________________</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B32" s="13" t="inlineStr">
         <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C32" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="n"/>
-      <c r="F29" s="15" t="n"/>
-      <c r="G29" s="15" t="n"/>
-      <c r="H29" s="16" t="inlineStr">
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="I29" s="15" t="n"/>
-      <c r="J29" s="15" t="n"/>
-      <c r="K29" s="15" t="n"/>
-      <c r="L29" s="15" t="n"/>
-      <c r="M29" s="15" t="n"/>
-      <c r="N29" s="15" t="n"/>
-      <c r="O29" s="14" t="inlineStr">
+      <c r="I32" s="15" t="n"/>
+      <c r="J32" s="15" t="n"/>
+      <c r="K32" s="15" t="n"/>
+      <c r="L32" s="15" t="n"/>
+      <c r="M32" s="15" t="n"/>
+      <c r="N32" s="15" t="n"/>
+      <c r="O32" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="P29" s="15" t="n"/>
-      <c r="Q29" s="17" t="inlineStr">
+      <c r="P32" s="15" t="n"/>
+      <c r="Q32" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Checked and verified by:
 ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="18" t="n"/>
-      <c r="B30" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" s="20">
-        <f>IF(0&lt;=Setup!$C$7,0,"")</f>
-        <v/>
-      </c>
-      <c r="D30" s="20">
-        <f>IF(1&lt;=Setup!$C$7,1,"")</f>
-        <v/>
-      </c>
-      <c r="E30" s="20">
-        <f>IF(2&lt;=Setup!$C$7,2,"")</f>
-        <v/>
-      </c>
-      <c r="F30" s="20">
-        <f>IF(3&lt;=Setup!$C$7,3,"")</f>
-        <v/>
-      </c>
-      <c r="G30" s="20">
-        <f>IF(4&lt;=Setup!$C$7,4,"")</f>
-        <v/>
-      </c>
-      <c r="H30" s="21">
-        <f>IF(0&lt;=Setup!$D$7,0,"")</f>
-        <v/>
-      </c>
-      <c r="I30" s="20">
-        <f>IF(1&lt;=Setup!$D$7,1,"")</f>
-        <v/>
-      </c>
-      <c r="J30" s="20">
-        <f>IF(2&lt;=Setup!$D$7,2,"")</f>
-        <v/>
-      </c>
-      <c r="K30" s="20">
-        <f>IF(3&lt;=Setup!$D$7,3,"")</f>
-        <v/>
-      </c>
-      <c r="L30" s="20">
-        <f>IF(4&lt;=Setup!$D$7,4,"")</f>
-        <v/>
-      </c>
-      <c r="M30" s="20">
-        <f>IF(5&lt;=Setup!$D$7,5,"")</f>
-        <v/>
-      </c>
-      <c r="N30" s="20">
-        <f>IF(6&lt;=Setup!$D$7,6,"")</f>
-        <v/>
-      </c>
-      <c r="O30" s="7" t="n"/>
-      <c r="P30" s="22">
-        <f>"/ "&amp;Setup!$E$7</f>
-        <v/>
-      </c>
-      <c r="Q30" s="23" t="n"/>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="18" t="n"/>
-      <c r="B31" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C31" s="20">
-        <f>IF(0&lt;=Setup!$C$8,0,"")</f>
-        <v/>
-      </c>
-      <c r="D31" s="20">
-        <f>IF(1&lt;=Setup!$C$8,1,"")</f>
-        <v/>
-      </c>
-      <c r="E31" s="20">
-        <f>IF(2&lt;=Setup!$C$8,2,"")</f>
-        <v/>
-      </c>
-      <c r="F31" s="20">
-        <f>IF(3&lt;=Setup!$C$8,3,"")</f>
-        <v/>
-      </c>
-      <c r="G31" s="20">
-        <f>IF(4&lt;=Setup!$C$8,4,"")</f>
-        <v/>
-      </c>
-      <c r="H31" s="21">
-        <f>IF(0&lt;=Setup!$D$8,0,"")</f>
-        <v/>
-      </c>
-      <c r="I31" s="20">
-        <f>IF(1&lt;=Setup!$D$8,1,"")</f>
-        <v/>
-      </c>
-      <c r="J31" s="20">
-        <f>IF(2&lt;=Setup!$D$8,2,"")</f>
-        <v/>
-      </c>
-      <c r="K31" s="20">
-        <f>IF(3&lt;=Setup!$D$8,3,"")</f>
-        <v/>
-      </c>
-      <c r="L31" s="20">
-        <f>IF(4&lt;=Setup!$D$8,4,"")</f>
-        <v/>
-      </c>
-      <c r="M31" s="20">
-        <f>IF(5&lt;=Setup!$D$8,5,"")</f>
-        <v/>
-      </c>
-      <c r="N31" s="20">
-        <f>IF(6&lt;=Setup!$D$8,6,"")</f>
-        <v/>
-      </c>
-      <c r="O31" s="7" t="n"/>
-      <c r="P31" s="22">
-        <f>"/ "&amp;Setup!$E$8</f>
-        <v/>
-      </c>
-      <c r="Q31" s="23" t="n"/>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="18" t="n"/>
-      <c r="B32" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="C32" s="20">
-        <f>IF(0&lt;=Setup!$C$9,0,"")</f>
-        <v/>
-      </c>
-      <c r="D32" s="20">
-        <f>IF(1&lt;=Setup!$C$9,1,"")</f>
-        <v/>
-      </c>
-      <c r="E32" s="20">
-        <f>IF(2&lt;=Setup!$C$9,2,"")</f>
-        <v/>
-      </c>
-      <c r="F32" s="20">
-        <f>IF(3&lt;=Setup!$C$9,3,"")</f>
-        <v/>
-      </c>
-      <c r="G32" s="20">
-        <f>IF(4&lt;=Setup!$C$9,4,"")</f>
-        <v/>
-      </c>
-      <c r="H32" s="21">
-        <f>IF(0&lt;=Setup!$D$9,0,"")</f>
-        <v/>
-      </c>
-      <c r="I32" s="20">
-        <f>IF(1&lt;=Setup!$D$9,1,"")</f>
-        <v/>
-      </c>
-      <c r="J32" s="20">
-        <f>IF(2&lt;=Setup!$D$9,2,"")</f>
-        <v/>
-      </c>
-      <c r="K32" s="20">
-        <f>IF(3&lt;=Setup!$D$9,3,"")</f>
-        <v/>
-      </c>
-      <c r="L32" s="20">
-        <f>IF(4&lt;=Setup!$D$9,4,"")</f>
-        <v/>
-      </c>
-      <c r="M32" s="20">
-        <f>IF(5&lt;=Setup!$D$9,5,"")</f>
-        <v/>
-      </c>
-      <c r="N32" s="20">
-        <f>IF(6&lt;=Setup!$D$9,6,"")</f>
-        <v/>
-      </c>
-      <c r="O32" s="7" t="n"/>
-      <c r="P32" s="22">
-        <f>"/ "&amp;Setup!$E$9</f>
-        <v/>
-      </c>
-      <c r="Q32" s="23" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="18" t="n"/>
       <c r="B33" s="19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C33" s="20">
-        <f>IF(0&lt;=Setup!$C$10,0,"")</f>
+        <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
       <c r="D33" s="20">
-        <f>IF(1&lt;=Setup!$C$10,1,"")</f>
+        <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
       <c r="E33" s="20">
-        <f>IF(2&lt;=Setup!$C$10,2,"")</f>
+        <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
       <c r="F33" s="20">
-        <f>IF(3&lt;=Setup!$C$10,3,"")</f>
+        <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
       <c r="G33" s="20">
-        <f>IF(4&lt;=Setup!$C$10,4,"")</f>
+        <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
       <c r="H33" s="21">
-        <f>IF(0&lt;=Setup!$D$10,0,"")</f>
+        <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
       <c r="I33" s="20">
-        <f>IF(1&lt;=Setup!$D$10,1,"")</f>
+        <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
       <c r="J33" s="20">
-        <f>IF(2&lt;=Setup!$D$10,2,"")</f>
+        <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
       <c r="K33" s="20">
-        <f>IF(3&lt;=Setup!$D$10,3,"")</f>
+        <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
       <c r="L33" s="20">
-        <f>IF(4&lt;=Setup!$D$10,4,"")</f>
+        <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
       <c r="M33" s="20">
-        <f>IF(5&lt;=Setup!$D$10,5,"")</f>
+        <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
       <c r="N33" s="20">
-        <f>IF(6&lt;=Setup!$D$10,6,"")</f>
+        <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
       <c r="O33" s="7" t="n"/>
       <c r="P33" s="22">
-        <f>"/ "&amp;Setup!$E$10</f>
+        <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
       <c r="Q33" s="23" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="18" t="n"/>
-      <c r="B34" s="24" t="n">
+      <c r="B34" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="20">
+        <f>IF(0&lt;=Setup!$C$8,0,"")</f>
+        <v/>
+      </c>
+      <c r="D34" s="20">
+        <f>IF(1&lt;=Setup!$C$8,1,"")</f>
+        <v/>
+      </c>
+      <c r="E34" s="20">
+        <f>IF(2&lt;=Setup!$C$8,2,"")</f>
+        <v/>
+      </c>
+      <c r="F34" s="20">
+        <f>IF(3&lt;=Setup!$C$8,3,"")</f>
+        <v/>
+      </c>
+      <c r="G34" s="20">
+        <f>IF(4&lt;=Setup!$C$8,4,"")</f>
+        <v/>
+      </c>
+      <c r="H34" s="21">
+        <f>IF(0&lt;=Setup!$D$8,0,"")</f>
+        <v/>
+      </c>
+      <c r="I34" s="20">
+        <f>IF(1&lt;=Setup!$D$8,1,"")</f>
+        <v/>
+      </c>
+      <c r="J34" s="20">
+        <f>IF(2&lt;=Setup!$D$8,2,"")</f>
+        <v/>
+      </c>
+      <c r="K34" s="20">
+        <f>IF(3&lt;=Setup!$D$8,3,"")</f>
+        <v/>
+      </c>
+      <c r="L34" s="20">
+        <f>IF(4&lt;=Setup!$D$8,4,"")</f>
+        <v/>
+      </c>
+      <c r="M34" s="20">
+        <f>IF(5&lt;=Setup!$D$8,5,"")</f>
+        <v/>
+      </c>
+      <c r="N34" s="20">
+        <f>IF(6&lt;=Setup!$D$8,6,"")</f>
+        <v/>
+      </c>
+      <c r="O34" s="7" t="n"/>
+      <c r="P34" s="22">
+        <f>"/ "&amp;Setup!$E$8</f>
+        <v/>
+      </c>
+      <c r="Q34" s="23" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="18" t="n"/>
+      <c r="B35" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" s="20">
+        <f>IF(0&lt;=Setup!$C$9,0,"")</f>
+        <v/>
+      </c>
+      <c r="D35" s="20">
+        <f>IF(1&lt;=Setup!$C$9,1,"")</f>
+        <v/>
+      </c>
+      <c r="E35" s="20">
+        <f>IF(2&lt;=Setup!$C$9,2,"")</f>
+        <v/>
+      </c>
+      <c r="F35" s="20">
+        <f>IF(3&lt;=Setup!$C$9,3,"")</f>
+        <v/>
+      </c>
+      <c r="G35" s="20">
+        <f>IF(4&lt;=Setup!$C$9,4,"")</f>
+        <v/>
+      </c>
+      <c r="H35" s="21">
+        <f>IF(0&lt;=Setup!$D$9,0,"")</f>
+        <v/>
+      </c>
+      <c r="I35" s="20">
+        <f>IF(1&lt;=Setup!$D$9,1,"")</f>
+        <v/>
+      </c>
+      <c r="J35" s="20">
+        <f>IF(2&lt;=Setup!$D$9,2,"")</f>
+        <v/>
+      </c>
+      <c r="K35" s="20">
+        <f>IF(3&lt;=Setup!$D$9,3,"")</f>
+        <v/>
+      </c>
+      <c r="L35" s="20">
+        <f>IF(4&lt;=Setup!$D$9,4,"")</f>
+        <v/>
+      </c>
+      <c r="M35" s="20">
+        <f>IF(5&lt;=Setup!$D$9,5,"")</f>
+        <v/>
+      </c>
+      <c r="N35" s="20">
+        <f>IF(6&lt;=Setup!$D$9,6,"")</f>
+        <v/>
+      </c>
+      <c r="O35" s="7" t="n"/>
+      <c r="P35" s="22">
+        <f>"/ "&amp;Setup!$E$9</f>
+        <v/>
+      </c>
+      <c r="Q35" s="23" t="n"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="18" t="n"/>
+      <c r="B36" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" s="20">
+        <f>IF(0&lt;=Setup!$C$10,0,"")</f>
+        <v/>
+      </c>
+      <c r="D36" s="20">
+        <f>IF(1&lt;=Setup!$C$10,1,"")</f>
+        <v/>
+      </c>
+      <c r="E36" s="20">
+        <f>IF(2&lt;=Setup!$C$10,2,"")</f>
+        <v/>
+      </c>
+      <c r="F36" s="20">
+        <f>IF(3&lt;=Setup!$C$10,3,"")</f>
+        <v/>
+      </c>
+      <c r="G36" s="20">
+        <f>IF(4&lt;=Setup!$C$10,4,"")</f>
+        <v/>
+      </c>
+      <c r="H36" s="21">
+        <f>IF(0&lt;=Setup!$D$10,0,"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="20">
+        <f>IF(1&lt;=Setup!$D$10,1,"")</f>
+        <v/>
+      </c>
+      <c r="J36" s="20">
+        <f>IF(2&lt;=Setup!$D$10,2,"")</f>
+        <v/>
+      </c>
+      <c r="K36" s="20">
+        <f>IF(3&lt;=Setup!$D$10,3,"")</f>
+        <v/>
+      </c>
+      <c r="L36" s="20">
+        <f>IF(4&lt;=Setup!$D$10,4,"")</f>
+        <v/>
+      </c>
+      <c r="M36" s="20">
+        <f>IF(5&lt;=Setup!$D$10,5,"")</f>
+        <v/>
+      </c>
+      <c r="N36" s="20">
+        <f>IF(6&lt;=Setup!$D$10,6,"")</f>
+        <v/>
+      </c>
+      <c r="O36" s="7" t="n"/>
+      <c r="P36" s="22">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="Q36" s="23" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="18" t="n"/>
+      <c r="B37" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="C34" s="25">
+      <c r="C37" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="D34" s="25">
+      <c r="D37" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="E34" s="25">
+      <c r="E37" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="F34" s="25">
+      <c r="F37" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="G34" s="25">
+      <c r="G37" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="H34" s="26">
+      <c r="H37" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="I34" s="25">
+      <c r="I37" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="J34" s="25">
+      <c r="J37" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="K34" s="25">
+      <c r="K37" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="L34" s="25">
+      <c r="L37" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="M34" s="25">
+      <c r="M37" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="N34" s="25">
+      <c r="N37" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="O34" s="7" t="n"/>
-      <c r="P34" s="27">
+      <c r="O37" s="7" t="n"/>
+      <c r="P37" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="Q34" s="23" t="n"/>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="28" t="n"/>
-      <c r="B35" s="29" t="inlineStr">
+      <c r="Q37" s="23" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="28" t="n"/>
+      <c r="B38" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="C35" s="30" t="n"/>
-      <c r="D35" s="30" t="n"/>
-      <c r="E35" s="30" t="n"/>
-      <c r="F35" s="30" t="n"/>
-      <c r="G35" s="30" t="n"/>
-      <c r="H35" s="30" t="n"/>
-      <c r="I35" s="30" t="n"/>
-      <c r="J35" s="30" t="n"/>
-      <c r="K35" s="30" t="n"/>
-      <c r="L35" s="30" t="n"/>
-      <c r="M35" s="30" t="n"/>
-      <c r="N35" s="30" t="n"/>
-      <c r="O35" s="31" t="n"/>
-      <c r="P35" s="32">
+      <c r="C38" s="30" t="n"/>
+      <c r="D38" s="30" t="n"/>
+      <c r="E38" s="30" t="n"/>
+      <c r="F38" s="30" t="n"/>
+      <c r="G38" s="30" t="n"/>
+      <c r="H38" s="30" t="n"/>
+      <c r="I38" s="30" t="n"/>
+      <c r="J38" s="30" t="n"/>
+      <c r="K38" s="30" t="n"/>
+      <c r="L38" s="30" t="n"/>
+      <c r="M38" s="30" t="n"/>
+      <c r="N38" s="30" t="n"/>
+      <c r="O38" s="31" t="n"/>
+      <c r="P38" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="Q35" s="33" t="n"/>
-    </row>
-    <row r="36" ht="9" customHeight="1">
-      <c r="A36" s="34" t="n"/>
-      <c r="B36" s="34" t="n"/>
-      <c r="C36" s="34" t="n"/>
-      <c r="D36" s="34" t="n"/>
-      <c r="E36" s="34" t="n"/>
-      <c r="F36" s="34" t="n"/>
-      <c r="G36" s="34" t="n"/>
-      <c r="H36" s="34" t="n"/>
-      <c r="I36" s="34" t="n"/>
-      <c r="J36" s="34" t="n"/>
-      <c r="K36" s="34" t="n"/>
-      <c r="L36" s="34" t="n"/>
-      <c r="M36" s="34" t="n"/>
-      <c r="N36" s="34" t="n"/>
-      <c r="O36" s="34" t="n"/>
-      <c r="P36" s="34" t="n"/>
-      <c r="Q36" s="34" t="n"/>
-    </row>
-    <row r="37" ht="19" customHeight="1">
-      <c r="A37" s="10">
+      <c r="Q38" s="33" t="n"/>
+    </row>
+    <row r="39" ht="7" customHeight="1">
+      <c r="A39" s="34" t="n"/>
+      <c r="B39" s="34" t="n"/>
+      <c r="C39" s="34" t="n"/>
+      <c r="D39" s="34" t="n"/>
+      <c r="E39" s="34" t="n"/>
+      <c r="F39" s="34" t="n"/>
+      <c r="G39" s="34" t="n"/>
+      <c r="H39" s="34" t="n"/>
+      <c r="I39" s="34" t="n"/>
+      <c r="J39" s="34" t="n"/>
+      <c r="K39" s="34" t="n"/>
+      <c r="L39" s="34" t="n"/>
+      <c r="M39" s="34" t="n"/>
+      <c r="N39" s="34" t="n"/>
+      <c r="O39" s="34" t="n"/>
+      <c r="P39" s="34" t="n"/>
+      <c r="Q39" s="34" t="n"/>
+    </row>
+    <row r="40" ht="11" customHeight="1"/>
+    <row r="41" ht="19" customHeight="1">
+      <c r="A41" s="10">
         <f>Setup!$B$3&amp;"  •  Rubric: Problem Set "&amp;Setup!$B$4</f>
         <v/>
       </c>
-      <c r="B37" s="11" t="n"/>
-      <c r="C37" s="11" t="n"/>
-      <c r="D37" s="11" t="n"/>
-      <c r="E37" s="11" t="n"/>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
-      <c r="H37" s="11" t="n"/>
-      <c r="I37" s="11" t="n"/>
-      <c r="J37" s="11" t="n"/>
-      <c r="K37" s="11" t="n"/>
-      <c r="L37" s="11" t="n"/>
-      <c r="M37" s="11" t="n"/>
-      <c r="N37" s="11" t="n"/>
-      <c r="O37" s="11" t="n"/>
-      <c r="P37" s="11" t="n"/>
-      <c r="Q37" s="11" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="12" t="inlineStr">
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
+      <c r="H41" s="11" t="n"/>
+      <c r="I41" s="11" t="n"/>
+      <c r="J41" s="11" t="n"/>
+      <c r="K41" s="11" t="n"/>
+      <c r="L41" s="11" t="n"/>
+      <c r="M41" s="11" t="n"/>
+      <c r="N41" s="11" t="n"/>
+      <c r="O41" s="11" t="n"/>
+      <c r="P41" s="11" t="n"/>
+      <c r="Q41" s="11" t="n"/>
+    </row>
+    <row r="42" ht="15" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Name: _____________________________          Grade &amp; Section: __________________</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="C38" s="14" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="15" t="n"/>
-      <c r="F38" s="15" t="n"/>
-      <c r="G38" s="15" t="n"/>
-      <c r="H38" s="16" t="inlineStr">
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15" t="n"/>
+      <c r="G42" s="15" t="n"/>
+      <c r="H42" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="I38" s="15" t="n"/>
-      <c r="J38" s="15" t="n"/>
-      <c r="K38" s="15" t="n"/>
-      <c r="L38" s="15" t="n"/>
-      <c r="M38" s="15" t="n"/>
-      <c r="N38" s="15" t="n"/>
-      <c r="O38" s="14" t="inlineStr">
+      <c r="I42" s="15" t="n"/>
+      <c r="J42" s="15" t="n"/>
+      <c r="K42" s="15" t="n"/>
+      <c r="L42" s="15" t="n"/>
+      <c r="M42" s="15" t="n"/>
+      <c r="N42" s="15" t="n"/>
+      <c r="O42" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="P38" s="15" t="n"/>
-      <c r="Q38" s="17" t="inlineStr">
+      <c r="P42" s="15" t="n"/>
+      <c r="Q42" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Checked and verified by:
 ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
     </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="18" t="n"/>
-      <c r="B39" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="20">
-        <f>IF(0&lt;=Setup!$C$7,0,"")</f>
-        <v/>
-      </c>
-      <c r="D39" s="20">
-        <f>IF(1&lt;=Setup!$C$7,1,"")</f>
-        <v/>
-      </c>
-      <c r="E39" s="20">
-        <f>IF(2&lt;=Setup!$C$7,2,"")</f>
-        <v/>
-      </c>
-      <c r="F39" s="20">
-        <f>IF(3&lt;=Setup!$C$7,3,"")</f>
-        <v/>
-      </c>
-      <c r="G39" s="20">
-        <f>IF(4&lt;=Setup!$C$7,4,"")</f>
-        <v/>
-      </c>
-      <c r="H39" s="21">
-        <f>IF(0&lt;=Setup!$D$7,0,"")</f>
-        <v/>
-      </c>
-      <c r="I39" s="20">
-        <f>IF(1&lt;=Setup!$D$7,1,"")</f>
-        <v/>
-      </c>
-      <c r="J39" s="20">
-        <f>IF(2&lt;=Setup!$D$7,2,"")</f>
-        <v/>
-      </c>
-      <c r="K39" s="20">
-        <f>IF(3&lt;=Setup!$D$7,3,"")</f>
-        <v/>
-      </c>
-      <c r="L39" s="20">
-        <f>IF(4&lt;=Setup!$D$7,4,"")</f>
-        <v/>
-      </c>
-      <c r="M39" s="20">
-        <f>IF(5&lt;=Setup!$D$7,5,"")</f>
-        <v/>
-      </c>
-      <c r="N39" s="20">
-        <f>IF(6&lt;=Setup!$D$7,6,"")</f>
-        <v/>
-      </c>
-      <c r="O39" s="7" t="n"/>
-      <c r="P39" s="22">
-        <f>"/ "&amp;Setup!$E$7</f>
-        <v/>
-      </c>
-      <c r="Q39" s="23" t="n"/>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="18" t="n"/>
-      <c r="B40" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C40" s="20">
-        <f>IF(0&lt;=Setup!$C$8,0,"")</f>
-        <v/>
-      </c>
-      <c r="D40" s="20">
-        <f>IF(1&lt;=Setup!$C$8,1,"")</f>
-        <v/>
-      </c>
-      <c r="E40" s="20">
-        <f>IF(2&lt;=Setup!$C$8,2,"")</f>
-        <v/>
-      </c>
-      <c r="F40" s="20">
-        <f>IF(3&lt;=Setup!$C$8,3,"")</f>
-        <v/>
-      </c>
-      <c r="G40" s="20">
-        <f>IF(4&lt;=Setup!$C$8,4,"")</f>
-        <v/>
-      </c>
-      <c r="H40" s="21">
-        <f>IF(0&lt;=Setup!$D$8,0,"")</f>
-        <v/>
-      </c>
-      <c r="I40" s="20">
-        <f>IF(1&lt;=Setup!$D$8,1,"")</f>
-        <v/>
-      </c>
-      <c r="J40" s="20">
-        <f>IF(2&lt;=Setup!$D$8,2,"")</f>
-        <v/>
-      </c>
-      <c r="K40" s="20">
-        <f>IF(3&lt;=Setup!$D$8,3,"")</f>
-        <v/>
-      </c>
-      <c r="L40" s="20">
-        <f>IF(4&lt;=Setup!$D$8,4,"")</f>
-        <v/>
-      </c>
-      <c r="M40" s="20">
-        <f>IF(5&lt;=Setup!$D$8,5,"")</f>
-        <v/>
-      </c>
-      <c r="N40" s="20">
-        <f>IF(6&lt;=Setup!$D$8,6,"")</f>
-        <v/>
-      </c>
-      <c r="O40" s="7" t="n"/>
-      <c r="P40" s="22">
-        <f>"/ "&amp;Setup!$E$8</f>
-        <v/>
-      </c>
-      <c r="Q40" s="23" t="n"/>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="18" t="n"/>
-      <c r="B41" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="C41" s="20">
-        <f>IF(0&lt;=Setup!$C$9,0,"")</f>
-        <v/>
-      </c>
-      <c r="D41" s="20">
-        <f>IF(1&lt;=Setup!$C$9,1,"")</f>
-        <v/>
-      </c>
-      <c r="E41" s="20">
-        <f>IF(2&lt;=Setup!$C$9,2,"")</f>
-        <v/>
-      </c>
-      <c r="F41" s="20">
-        <f>IF(3&lt;=Setup!$C$9,3,"")</f>
-        <v/>
-      </c>
-      <c r="G41" s="20">
-        <f>IF(4&lt;=Setup!$C$9,4,"")</f>
-        <v/>
-      </c>
-      <c r="H41" s="21">
-        <f>IF(0&lt;=Setup!$D$9,0,"")</f>
-        <v/>
-      </c>
-      <c r="I41" s="20">
-        <f>IF(1&lt;=Setup!$D$9,1,"")</f>
-        <v/>
-      </c>
-      <c r="J41" s="20">
-        <f>IF(2&lt;=Setup!$D$9,2,"")</f>
-        <v/>
-      </c>
-      <c r="K41" s="20">
-        <f>IF(3&lt;=Setup!$D$9,3,"")</f>
-        <v/>
-      </c>
-      <c r="L41" s="20">
-        <f>IF(4&lt;=Setup!$D$9,4,"")</f>
-        <v/>
-      </c>
-      <c r="M41" s="20">
-        <f>IF(5&lt;=Setup!$D$9,5,"")</f>
-        <v/>
-      </c>
-      <c r="N41" s="20">
-        <f>IF(6&lt;=Setup!$D$9,6,"")</f>
-        <v/>
-      </c>
-      <c r="O41" s="7" t="n"/>
-      <c r="P41" s="22">
-        <f>"/ "&amp;Setup!$E$9</f>
-        <v/>
-      </c>
-      <c r="Q41" s="23" t="n"/>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="18" t="n"/>
-      <c r="B42" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="C42" s="20">
-        <f>IF(0&lt;=Setup!$C$10,0,"")</f>
-        <v/>
-      </c>
-      <c r="D42" s="20">
-        <f>IF(1&lt;=Setup!$C$10,1,"")</f>
-        <v/>
-      </c>
-      <c r="E42" s="20">
-        <f>IF(2&lt;=Setup!$C$10,2,"")</f>
-        <v/>
-      </c>
-      <c r="F42" s="20">
-        <f>IF(3&lt;=Setup!$C$10,3,"")</f>
-        <v/>
-      </c>
-      <c r="G42" s="20">
-        <f>IF(4&lt;=Setup!$C$10,4,"")</f>
-        <v/>
-      </c>
-      <c r="H42" s="21">
-        <f>IF(0&lt;=Setup!$D$10,0,"")</f>
-        <v/>
-      </c>
-      <c r="I42" s="20">
-        <f>IF(1&lt;=Setup!$D$10,1,"")</f>
-        <v/>
-      </c>
-      <c r="J42" s="20">
-        <f>IF(2&lt;=Setup!$D$10,2,"")</f>
-        <v/>
-      </c>
-      <c r="K42" s="20">
-        <f>IF(3&lt;=Setup!$D$10,3,"")</f>
-        <v/>
-      </c>
-      <c r="L42" s="20">
-        <f>IF(4&lt;=Setup!$D$10,4,"")</f>
-        <v/>
-      </c>
-      <c r="M42" s="20">
-        <f>IF(5&lt;=Setup!$D$10,5,"")</f>
-        <v/>
-      </c>
-      <c r="N42" s="20">
-        <f>IF(6&lt;=Setup!$D$10,6,"")</f>
-        <v/>
-      </c>
-      <c r="O42" s="7" t="n"/>
-      <c r="P42" s="22">
-        <f>"/ "&amp;Setup!$E$10</f>
-        <v/>
-      </c>
-      <c r="Q42" s="23" t="n"/>
-    </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="18" t="n"/>
-      <c r="B43" s="24" t="n">
+      <c r="B43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="20">
+        <f>IF(0&lt;=Setup!$C$7,0,"")</f>
+        <v/>
+      </c>
+      <c r="D43" s="20">
+        <f>IF(1&lt;=Setup!$C$7,1,"")</f>
+        <v/>
+      </c>
+      <c r="E43" s="20">
+        <f>IF(2&lt;=Setup!$C$7,2,"")</f>
+        <v/>
+      </c>
+      <c r="F43" s="20">
+        <f>IF(3&lt;=Setup!$C$7,3,"")</f>
+        <v/>
+      </c>
+      <c r="G43" s="20">
+        <f>IF(4&lt;=Setup!$C$7,4,"")</f>
+        <v/>
+      </c>
+      <c r="H43" s="21">
+        <f>IF(0&lt;=Setup!$D$7,0,"")</f>
+        <v/>
+      </c>
+      <c r="I43" s="20">
+        <f>IF(1&lt;=Setup!$D$7,1,"")</f>
+        <v/>
+      </c>
+      <c r="J43" s="20">
+        <f>IF(2&lt;=Setup!$D$7,2,"")</f>
+        <v/>
+      </c>
+      <c r="K43" s="20">
+        <f>IF(3&lt;=Setup!$D$7,3,"")</f>
+        <v/>
+      </c>
+      <c r="L43" s="20">
+        <f>IF(4&lt;=Setup!$D$7,4,"")</f>
+        <v/>
+      </c>
+      <c r="M43" s="20">
+        <f>IF(5&lt;=Setup!$D$7,5,"")</f>
+        <v/>
+      </c>
+      <c r="N43" s="20">
+        <f>IF(6&lt;=Setup!$D$7,6,"")</f>
+        <v/>
+      </c>
+      <c r="O43" s="7" t="n"/>
+      <c r="P43" s="22">
+        <f>"/ "&amp;Setup!$E$7</f>
+        <v/>
+      </c>
+      <c r="Q43" s="23" t="n"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="18" t="n"/>
+      <c r="B44" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" s="20">
+        <f>IF(0&lt;=Setup!$C$8,0,"")</f>
+        <v/>
+      </c>
+      <c r="D44" s="20">
+        <f>IF(1&lt;=Setup!$C$8,1,"")</f>
+        <v/>
+      </c>
+      <c r="E44" s="20">
+        <f>IF(2&lt;=Setup!$C$8,2,"")</f>
+        <v/>
+      </c>
+      <c r="F44" s="20">
+        <f>IF(3&lt;=Setup!$C$8,3,"")</f>
+        <v/>
+      </c>
+      <c r="G44" s="20">
+        <f>IF(4&lt;=Setup!$C$8,4,"")</f>
+        <v/>
+      </c>
+      <c r="H44" s="21">
+        <f>IF(0&lt;=Setup!$D$8,0,"")</f>
+        <v/>
+      </c>
+      <c r="I44" s="20">
+        <f>IF(1&lt;=Setup!$D$8,1,"")</f>
+        <v/>
+      </c>
+      <c r="J44" s="20">
+        <f>IF(2&lt;=Setup!$D$8,2,"")</f>
+        <v/>
+      </c>
+      <c r="K44" s="20">
+        <f>IF(3&lt;=Setup!$D$8,3,"")</f>
+        <v/>
+      </c>
+      <c r="L44" s="20">
+        <f>IF(4&lt;=Setup!$D$8,4,"")</f>
+        <v/>
+      </c>
+      <c r="M44" s="20">
+        <f>IF(5&lt;=Setup!$D$8,5,"")</f>
+        <v/>
+      </c>
+      <c r="N44" s="20">
+        <f>IF(6&lt;=Setup!$D$8,6,"")</f>
+        <v/>
+      </c>
+      <c r="O44" s="7" t="n"/>
+      <c r="P44" s="22">
+        <f>"/ "&amp;Setup!$E$8</f>
+        <v/>
+      </c>
+      <c r="Q44" s="23" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="18" t="n"/>
+      <c r="B45" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" s="20">
+        <f>IF(0&lt;=Setup!$C$9,0,"")</f>
+        <v/>
+      </c>
+      <c r="D45" s="20">
+        <f>IF(1&lt;=Setup!$C$9,1,"")</f>
+        <v/>
+      </c>
+      <c r="E45" s="20">
+        <f>IF(2&lt;=Setup!$C$9,2,"")</f>
+        <v/>
+      </c>
+      <c r="F45" s="20">
+        <f>IF(3&lt;=Setup!$C$9,3,"")</f>
+        <v/>
+      </c>
+      <c r="G45" s="20">
+        <f>IF(4&lt;=Setup!$C$9,4,"")</f>
+        <v/>
+      </c>
+      <c r="H45" s="21">
+        <f>IF(0&lt;=Setup!$D$9,0,"")</f>
+        <v/>
+      </c>
+      <c r="I45" s="20">
+        <f>IF(1&lt;=Setup!$D$9,1,"")</f>
+        <v/>
+      </c>
+      <c r="J45" s="20">
+        <f>IF(2&lt;=Setup!$D$9,2,"")</f>
+        <v/>
+      </c>
+      <c r="K45" s="20">
+        <f>IF(3&lt;=Setup!$D$9,3,"")</f>
+        <v/>
+      </c>
+      <c r="L45" s="20">
+        <f>IF(4&lt;=Setup!$D$9,4,"")</f>
+        <v/>
+      </c>
+      <c r="M45" s="20">
+        <f>IF(5&lt;=Setup!$D$9,5,"")</f>
+        <v/>
+      </c>
+      <c r="N45" s="20">
+        <f>IF(6&lt;=Setup!$D$9,6,"")</f>
+        <v/>
+      </c>
+      <c r="O45" s="7" t="n"/>
+      <c r="P45" s="22">
+        <f>"/ "&amp;Setup!$E$9</f>
+        <v/>
+      </c>
+      <c r="Q45" s="23" t="n"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="18" t="n"/>
+      <c r="B46" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C46" s="20">
+        <f>IF(0&lt;=Setup!$C$10,0,"")</f>
+        <v/>
+      </c>
+      <c r="D46" s="20">
+        <f>IF(1&lt;=Setup!$C$10,1,"")</f>
+        <v/>
+      </c>
+      <c r="E46" s="20">
+        <f>IF(2&lt;=Setup!$C$10,2,"")</f>
+        <v/>
+      </c>
+      <c r="F46" s="20">
+        <f>IF(3&lt;=Setup!$C$10,3,"")</f>
+        <v/>
+      </c>
+      <c r="G46" s="20">
+        <f>IF(4&lt;=Setup!$C$10,4,"")</f>
+        <v/>
+      </c>
+      <c r="H46" s="21">
+        <f>IF(0&lt;=Setup!$D$10,0,"")</f>
+        <v/>
+      </c>
+      <c r="I46" s="20">
+        <f>IF(1&lt;=Setup!$D$10,1,"")</f>
+        <v/>
+      </c>
+      <c r="J46" s="20">
+        <f>IF(2&lt;=Setup!$D$10,2,"")</f>
+        <v/>
+      </c>
+      <c r="K46" s="20">
+        <f>IF(3&lt;=Setup!$D$10,3,"")</f>
+        <v/>
+      </c>
+      <c r="L46" s="20">
+        <f>IF(4&lt;=Setup!$D$10,4,"")</f>
+        <v/>
+      </c>
+      <c r="M46" s="20">
+        <f>IF(5&lt;=Setup!$D$10,5,"")</f>
+        <v/>
+      </c>
+      <c r="N46" s="20">
+        <f>IF(6&lt;=Setup!$D$10,6,"")</f>
+        <v/>
+      </c>
+      <c r="O46" s="7" t="n"/>
+      <c r="P46" s="22">
+        <f>"/ "&amp;Setup!$E$10</f>
+        <v/>
+      </c>
+      <c r="Q46" s="23" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="18" t="n"/>
+      <c r="B47" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="C43" s="25">
+      <c r="C47" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="D43" s="25">
+      <c r="D47" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="E43" s="25">
+      <c r="E47" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="F43" s="25">
+      <c r="F47" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="G43" s="25">
+      <c r="G47" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="H43" s="26">
+      <c r="H47" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="I43" s="25">
+      <c r="I47" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="J43" s="25">
+      <c r="J47" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="K43" s="25">
+      <c r="K47" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="L43" s="25">
+      <c r="L47" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="M43" s="25">
+      <c r="M47" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="N43" s="25">
+      <c r="N47" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="O43" s="7" t="n"/>
-      <c r="P43" s="27">
+      <c r="O47" s="7" t="n"/>
+      <c r="P47" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="Q43" s="23" t="n"/>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="28" t="n"/>
-      <c r="B44" s="29" t="inlineStr">
+      <c r="Q47" s="23" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="28" t="n"/>
+      <c r="B48" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="C44" s="30" t="n"/>
-      <c r="D44" s="30" t="n"/>
-      <c r="E44" s="30" t="n"/>
-      <c r="F44" s="30" t="n"/>
-      <c r="G44" s="30" t="n"/>
-      <c r="H44" s="30" t="n"/>
-      <c r="I44" s="30" t="n"/>
-      <c r="J44" s="30" t="n"/>
-      <c r="K44" s="30" t="n"/>
-      <c r="L44" s="30" t="n"/>
-      <c r="M44" s="30" t="n"/>
-      <c r="N44" s="30" t="n"/>
-      <c r="O44" s="31" t="n"/>
-      <c r="P44" s="32">
+      <c r="C48" s="30" t="n"/>
+      <c r="D48" s="30" t="n"/>
+      <c r="E48" s="30" t="n"/>
+      <c r="F48" s="30" t="n"/>
+      <c r="G48" s="30" t="n"/>
+      <c r="H48" s="30" t="n"/>
+      <c r="I48" s="30" t="n"/>
+      <c r="J48" s="30" t="n"/>
+      <c r="K48" s="30" t="n"/>
+      <c r="L48" s="30" t="n"/>
+      <c r="M48" s="30" t="n"/>
+      <c r="N48" s="30" t="n"/>
+      <c r="O48" s="31" t="n"/>
+      <c r="P48" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="Q44" s="33" t="n"/>
-    </row>
-    <row r="45" ht="9" customHeight="1">
-      <c r="A45" s="34" t="n"/>
-      <c r="B45" s="34" t="n"/>
-      <c r="C45" s="34" t="n"/>
-      <c r="D45" s="34" t="n"/>
-      <c r="E45" s="34" t="n"/>
-      <c r="F45" s="34" t="n"/>
-      <c r="G45" s="34" t="n"/>
-      <c r="H45" s="34" t="n"/>
-      <c r="I45" s="34" t="n"/>
-      <c r="J45" s="34" t="n"/>
-      <c r="K45" s="34" t="n"/>
-      <c r="L45" s="34" t="n"/>
-      <c r="M45" s="34" t="n"/>
-      <c r="N45" s="34" t="n"/>
-      <c r="O45" s="34" t="n"/>
-      <c r="P45" s="34" t="n"/>
-      <c r="Q45" s="34" t="n"/>
-    </row>
-    <row r="46" ht="19" customHeight="1">
-      <c r="A46" s="10">
+      <c r="Q48" s="33" t="n"/>
+    </row>
+    <row r="49" ht="7" customHeight="1">
+      <c r="A49" s="34" t="n"/>
+      <c r="B49" s="34" t="n"/>
+      <c r="C49" s="34" t="n"/>
+      <c r="D49" s="34" t="n"/>
+      <c r="E49" s="34" t="n"/>
+      <c r="F49" s="34" t="n"/>
+      <c r="G49" s="34" t="n"/>
+      <c r="H49" s="34" t="n"/>
+      <c r="I49" s="34" t="n"/>
+      <c r="J49" s="34" t="n"/>
+      <c r="K49" s="34" t="n"/>
+      <c r="L49" s="34" t="n"/>
+      <c r="M49" s="34" t="n"/>
+      <c r="N49" s="34" t="n"/>
+      <c r="O49" s="34" t="n"/>
+      <c r="P49" s="34" t="n"/>
+      <c r="Q49" s="34" t="n"/>
+    </row>
+    <row r="50" ht="11" customHeight="1"/>
+    <row r="51" ht="19" customHeight="1">
+      <c r="A51" s="10">
         <f>Setup!$B$3&amp;"  •  Rubric: Problem Set "&amp;Setup!$B$4</f>
         <v/>
       </c>
-      <c r="B46" s="11" t="n"/>
-      <c r="C46" s="11" t="n"/>
-      <c r="D46" s="11" t="n"/>
-      <c r="E46" s="11" t="n"/>
-      <c r="F46" s="11" t="n"/>
-      <c r="G46" s="11" t="n"/>
-      <c r="H46" s="11" t="n"/>
-      <c r="I46" s="11" t="n"/>
-      <c r="J46" s="11" t="n"/>
-      <c r="K46" s="11" t="n"/>
-      <c r="L46" s="11" t="n"/>
-      <c r="M46" s="11" t="n"/>
-      <c r="N46" s="11" t="n"/>
-      <c r="O46" s="11" t="n"/>
-      <c r="P46" s="11" t="n"/>
-      <c r="Q46" s="11" t="n"/>
-    </row>
-    <row r="47" ht="15" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
+      <c r="B51" s="11" t="n"/>
+      <c r="C51" s="11" t="n"/>
+      <c r="D51" s="11" t="n"/>
+      <c r="E51" s="11" t="n"/>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="11" t="n"/>
+      <c r="H51" s="11" t="n"/>
+      <c r="I51" s="11" t="n"/>
+      <c r="J51" s="11" t="n"/>
+      <c r="K51" s="11" t="n"/>
+      <c r="L51" s="11" t="n"/>
+      <c r="M51" s="11" t="n"/>
+      <c r="N51" s="11" t="n"/>
+      <c r="O51" s="11" t="n"/>
+      <c r="P51" s="11" t="n"/>
+      <c r="Q51" s="11" t="n"/>
+    </row>
+    <row r="52" ht="15" customHeight="1">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t>Name: _____________________________          Grade &amp; Section: __________________</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr">
+      <c r="B52" s="13" t="inlineStr">
         <is>
           <t>Prob</t>
         </is>
       </c>
-      <c r="C47" s="14" t="inlineStr">
+      <c r="C52" s="14" t="inlineStr">
         <is>
           <t>Final Answer</t>
         </is>
       </c>
-      <c r="D47" s="15" t="n"/>
-      <c r="E47" s="15" t="n"/>
-      <c r="F47" s="15" t="n"/>
-      <c r="G47" s="15" t="n"/>
-      <c r="H47" s="16" t="inlineStr">
+      <c r="D52" s="15" t="n"/>
+      <c r="E52" s="15" t="n"/>
+      <c r="F52" s="15" t="n"/>
+      <c r="G52" s="15" t="n"/>
+      <c r="H52" s="16" t="inlineStr">
         <is>
           <t>Concept &amp; Execution</t>
         </is>
       </c>
-      <c r="I47" s="15" t="n"/>
-      <c r="J47" s="15" t="n"/>
-      <c r="K47" s="15" t="n"/>
-      <c r="L47" s="15" t="n"/>
-      <c r="M47" s="15" t="n"/>
-      <c r="N47" s="15" t="n"/>
-      <c r="O47" s="14" t="inlineStr">
+      <c r="I52" s="15" t="n"/>
+      <c r="J52" s="15" t="n"/>
+      <c r="K52" s="15" t="n"/>
+      <c r="L52" s="15" t="n"/>
+      <c r="M52" s="15" t="n"/>
+      <c r="N52" s="15" t="n"/>
+      <c r="O52" s="14" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="P47" s="15" t="n"/>
-      <c r="Q47" s="17" t="inlineStr">
+      <c r="P52" s="15" t="n"/>
+      <c r="Q52" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">Checked and verified by:
 ENGR. PHILIP JAYSON L. LESTOJAS </t>
         </is>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="18" t="n"/>
-      <c r="B48" s="19" t="n">
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="18" t="n"/>
+      <c r="B53" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="C48" s="20">
+      <c r="C53" s="20">
         <f>IF(0&lt;=Setup!$C$7,0,"")</f>
         <v/>
       </c>
-      <c r="D48" s="20">
+      <c r="D53" s="20">
         <f>IF(1&lt;=Setup!$C$7,1,"")</f>
         <v/>
       </c>
-      <c r="E48" s="20">
+      <c r="E53" s="20">
         <f>IF(2&lt;=Setup!$C$7,2,"")</f>
         <v/>
       </c>
-      <c r="F48" s="20">
+      <c r="F53" s="20">
         <f>IF(3&lt;=Setup!$C$7,3,"")</f>
         <v/>
       </c>
-      <c r="G48" s="20">
+      <c r="G53" s="20">
         <f>IF(4&lt;=Setup!$C$7,4,"")</f>
         <v/>
       </c>
-      <c r="H48" s="21">
+      <c r="H53" s="21">
         <f>IF(0&lt;=Setup!$D$7,0,"")</f>
         <v/>
       </c>
-      <c r="I48" s="20">
+      <c r="I53" s="20">
         <f>IF(1&lt;=Setup!$D$7,1,"")</f>
         <v/>
       </c>
-      <c r="J48" s="20">
+      <c r="J53" s="20">
         <f>IF(2&lt;=Setup!$D$7,2,"")</f>
         <v/>
       </c>
-      <c r="K48" s="20">
+      <c r="K53" s="20">
         <f>IF(3&lt;=Setup!$D$7,3,"")</f>
         <v/>
       </c>
-      <c r="L48" s="20">
+      <c r="L53" s="20">
         <f>IF(4&lt;=Setup!$D$7,4,"")</f>
         <v/>
       </c>
-      <c r="M48" s="20">
+      <c r="M53" s="20">
         <f>IF(5&lt;=Setup!$D$7,5,"")</f>
         <v/>
       </c>
-      <c r="N48" s="20">
+      <c r="N53" s="20">
         <f>IF(6&lt;=Setup!$D$7,6,"")</f>
         <v/>
       </c>
-      <c r="O48" s="7" t="n"/>
-      <c r="P48" s="22">
+      <c r="O53" s="7" t="n"/>
+      <c r="P53" s="22">
         <f>"/ "&amp;Setup!$E$7</f>
         <v/>
       </c>
-      <c r="Q48" s="23" t="n"/>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="18" t="n"/>
-      <c r="B49" s="19" t="n">
+      <c r="Q53" s="23" t="n"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="18" t="n"/>
+      <c r="B54" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="C49" s="20">
+      <c r="C54" s="20">
         <f>IF(0&lt;=Setup!$C$8,0,"")</f>
         <v/>
       </c>
-      <c r="D49" s="20">
+      <c r="D54" s="20">
         <f>IF(1&lt;=Setup!$C$8,1,"")</f>
         <v/>
       </c>
-      <c r="E49" s="20">
+      <c r="E54" s="20">
         <f>IF(2&lt;=Setup!$C$8,2,"")</f>
         <v/>
       </c>
-      <c r="F49" s="20">
+      <c r="F54" s="20">
         <f>IF(3&lt;=Setup!$C$8,3,"")</f>
         <v/>
       </c>
-      <c r="G49" s="20">
+      <c r="G54" s="20">
         <f>IF(4&lt;=Setup!$C$8,4,"")</f>
         <v/>
       </c>
-      <c r="H49" s="21">
+      <c r="H54" s="21">
         <f>IF(0&lt;=Setup!$D$8,0,"")</f>
         <v/>
       </c>
-      <c r="I49" s="20">
+      <c r="I54" s="20">
         <f>IF(1&lt;=Setup!$D$8,1,"")</f>
         <v/>
       </c>
-      <c r="J49" s="20">
+      <c r="J54" s="20">
         <f>IF(2&lt;=Setup!$D$8,2,"")</f>
         <v/>
       </c>
-      <c r="K49" s="20">
+      <c r="K54" s="20">
         <f>IF(3&lt;=Setup!$D$8,3,"")</f>
         <v/>
       </c>
-      <c r="L49" s="20">
+      <c r="L54" s="20">
         <f>IF(4&lt;=Setup!$D$8,4,"")</f>
         <v/>
       </c>
-      <c r="M49" s="20">
+      <c r="M54" s="20">
         <f>IF(5&lt;=Setup!$D$8,5,"")</f>
         <v/>
       </c>
-      <c r="N49" s="20">
+      <c r="N54" s="20">
         <f>IF(6&lt;=Setup!$D$8,6,"")</f>
         <v/>
       </c>
-      <c r="O49" s="7" t="n"/>
-      <c r="P49" s="22">
+      <c r="O54" s="7" t="n"/>
+      <c r="P54" s="22">
         <f>"/ "&amp;Setup!$E$8</f>
         <v/>
       </c>
-      <c r="Q49" s="23" t="n"/>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="18" t="n"/>
-      <c r="B50" s="19" t="n">
+      <c r="Q54" s="23" t="n"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="18" t="n"/>
+      <c r="B55" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="C50" s="20">
+      <c r="C55" s="20">
         <f>IF(0&lt;=Setup!$C$9,0,"")</f>
         <v/>
       </c>
-      <c r="D50" s="20">
+      <c r="D55" s="20">
         <f>IF(1&lt;=Setup!$C$9,1,"")</f>
         <v/>
       </c>
-      <c r="E50" s="20">
+      <c r="E55" s="20">
         <f>IF(2&lt;=Setup!$C$9,2,"")</f>
         <v/>
       </c>
-      <c r="F50" s="20">
+      <c r="F55" s="20">
         <f>IF(3&lt;=Setup!$C$9,3,"")</f>
         <v/>
       </c>
-      <c r="G50" s="20">
+      <c r="G55" s="20">
         <f>IF(4&lt;=Setup!$C$9,4,"")</f>
         <v/>
       </c>
-      <c r="H50" s="21">
+      <c r="H55" s="21">
         <f>IF(0&lt;=Setup!$D$9,0,"")</f>
         <v/>
       </c>
-      <c r="I50" s="20">
+      <c r="I55" s="20">
         <f>IF(1&lt;=Setup!$D$9,1,"")</f>
         <v/>
       </c>
-      <c r="J50" s="20">
+      <c r="J55" s="20">
         <f>IF(2&lt;=Setup!$D$9,2,"")</f>
         <v/>
       </c>
-      <c r="K50" s="20">
+      <c r="K55" s="20">
         <f>IF(3&lt;=Setup!$D$9,3,"")</f>
         <v/>
       </c>
-      <c r="L50" s="20">
+      <c r="L55" s="20">
         <f>IF(4&lt;=Setup!$D$9,4,"")</f>
         <v/>
       </c>
-      <c r="M50" s="20">
+      <c r="M55" s="20">
         <f>IF(5&lt;=Setup!$D$9,5,"")</f>
         <v/>
       </c>
-      <c r="N50" s="20">
+      <c r="N55" s="20">
         <f>IF(6&lt;=Setup!$D$9,6,"")</f>
         <v/>
       </c>
-      <c r="O50" s="7" t="n"/>
-      <c r="P50" s="22">
+      <c r="O55" s="7" t="n"/>
+      <c r="P55" s="22">
         <f>"/ "&amp;Setup!$E$9</f>
         <v/>
       </c>
-      <c r="Q50" s="23" t="n"/>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="18" t="n"/>
-      <c r="B51" s="19" t="n">
+      <c r="Q55" s="23" t="n"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="18" t="n"/>
+      <c r="B56" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="C51" s="20">
+      <c r="C56" s="20">
         <f>IF(0&lt;=Setup!$C$10,0,"")</f>
         <v/>
       </c>
-      <c r="D51" s="20">
+      <c r="D56" s="20">
         <f>IF(1&lt;=Setup!$C$10,1,"")</f>
         <v/>
       </c>
-      <c r="E51" s="20">
+      <c r="E56" s="20">
         <f>IF(2&lt;=Setup!$C$10,2,"")</f>
         <v/>
       </c>
-      <c r="F51" s="20">
+      <c r="F56" s="20">
         <f>IF(3&lt;=Setup!$C$10,3,"")</f>
         <v/>
       </c>
-      <c r="G51" s="20">
+      <c r="G56" s="20">
         <f>IF(4&lt;=Setup!$C$10,4,"")</f>
         <v/>
       </c>
-      <c r="H51" s="21">
+      <c r="H56" s="21">
         <f>IF(0&lt;=Setup!$D$10,0,"")</f>
         <v/>
       </c>
-      <c r="I51" s="20">
+      <c r="I56" s="20">
         <f>IF(1&lt;=Setup!$D$10,1,"")</f>
         <v/>
       </c>
-      <c r="J51" s="20">
+      <c r="J56" s="20">
         <f>IF(2&lt;=Setup!$D$10,2,"")</f>
         <v/>
       </c>
-      <c r="K51" s="20">
+      <c r="K56" s="20">
         <f>IF(3&lt;=Setup!$D$10,3,"")</f>
         <v/>
       </c>
-      <c r="L51" s="20">
+      <c r="L56" s="20">
         <f>IF(4&lt;=Setup!$D$10,4,"")</f>
         <v/>
       </c>
-      <c r="M51" s="20">
+      <c r="M56" s="20">
         <f>IF(5&lt;=Setup!$D$10,5,"")</f>
         <v/>
       </c>
-      <c r="N51" s="20">
+      <c r="N56" s="20">
         <f>IF(6&lt;=Setup!$D$10,6,"")</f>
         <v/>
       </c>
-      <c r="O51" s="7" t="n"/>
-      <c r="P51" s="22">
+      <c r="O56" s="7" t="n"/>
+      <c r="P56" s="22">
         <f>"/ "&amp;Setup!$E$10</f>
         <v/>
       </c>
-      <c r="Q51" s="23" t="n"/>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="18" t="n"/>
-      <c r="B52" s="24" t="n">
+      <c r="Q56" s="23" t="n"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="18" t="n"/>
+      <c r="B57" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="C52" s="25">
+      <c r="C57" s="25">
         <f>IF(0&lt;=Setup!$C$11,0,"")</f>
         <v/>
       </c>
-      <c r="D52" s="25">
+      <c r="D57" s="25">
         <f>IF(1&lt;=Setup!$C$11,1,"")</f>
         <v/>
       </c>
-      <c r="E52" s="25">
+      <c r="E57" s="25">
         <f>IF(2&lt;=Setup!$C$11,2,"")</f>
         <v/>
       </c>
-      <c r="F52" s="25">
+      <c r="F57" s="25">
         <f>IF(3&lt;=Setup!$C$11,3,"")</f>
         <v/>
       </c>
-      <c r="G52" s="25">
+      <c r="G57" s="25">
         <f>IF(4&lt;=Setup!$C$11,4,"")</f>
         <v/>
       </c>
-      <c r="H52" s="26">
+      <c r="H57" s="26">
         <f>IF(0&lt;=Setup!$D$11,0,"")</f>
         <v/>
       </c>
-      <c r="I52" s="25">
+      <c r="I57" s="25">
         <f>IF(1&lt;=Setup!$D$11,1,"")</f>
         <v/>
       </c>
-      <c r="J52" s="25">
+      <c r="J57" s="25">
         <f>IF(2&lt;=Setup!$D$11,2,"")</f>
         <v/>
       </c>
-      <c r="K52" s="25">
+      <c r="K57" s="25">
         <f>IF(3&lt;=Setup!$D$11,3,"")</f>
         <v/>
       </c>
-      <c r="L52" s="25">
+      <c r="L57" s="25">
         <f>IF(4&lt;=Setup!$D$11,4,"")</f>
         <v/>
       </c>
-      <c r="M52" s="25">
+      <c r="M57" s="25">
         <f>IF(5&lt;=Setup!$D$11,5,"")</f>
         <v/>
       </c>
-      <c r="N52" s="25">
+      <c r="N57" s="25">
         <f>IF(6&lt;=Setup!$D$11,6,"")</f>
         <v/>
       </c>
-      <c r="O52" s="7" t="n"/>
-      <c r="P52" s="27">
+      <c r="O57" s="7" t="n"/>
+      <c r="P57" s="27">
         <f>"/ "&amp;Setup!$E$11</f>
         <v/>
       </c>
-      <c r="Q52" s="23" t="n"/>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="28" t="n"/>
-      <c r="B53" s="29" t="inlineStr">
+      <c r="Q57" s="23" t="n"/>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="28" t="n"/>
+      <c r="B58" s="29" t="inlineStr">
         <is>
           <t>TOTAL SCORE  →</t>
         </is>
       </c>
-      <c r="C53" s="30" t="n"/>
-      <c r="D53" s="30" t="n"/>
-      <c r="E53" s="30" t="n"/>
-      <c r="F53" s="30" t="n"/>
-      <c r="G53" s="30" t="n"/>
-      <c r="H53" s="30" t="n"/>
-      <c r="I53" s="30" t="n"/>
-      <c r="J53" s="30" t="n"/>
-      <c r="K53" s="30" t="n"/>
-      <c r="L53" s="30" t="n"/>
-      <c r="M53" s="30" t="n"/>
-      <c r="N53" s="30" t="n"/>
-      <c r="O53" s="31" t="n"/>
-      <c r="P53" s="32">
+      <c r="C58" s="30" t="n"/>
+      <c r="D58" s="30" t="n"/>
+      <c r="E58" s="30" t="n"/>
+      <c r="F58" s="30" t="n"/>
+      <c r="G58" s="30" t="n"/>
+      <c r="H58" s="30" t="n"/>
+      <c r="I58" s="30" t="n"/>
+      <c r="J58" s="30" t="n"/>
+      <c r="K58" s="30" t="n"/>
+      <c r="L58" s="30" t="n"/>
+      <c r="M58" s="30" t="n"/>
+      <c r="N58" s="30" t="n"/>
+      <c r="O58" s="31" t="n"/>
+      <c r="P58" s="32">
         <f>"/ "&amp;SUM(Setup!$E$7:$E$11)</f>
         <v/>
       </c>
-      <c r="Q53" s="33" t="n"/>
+      <c r="Q58" s="33" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="H47:N47"/>
-    <mergeCell ref="Q38:Q44"/>
-    <mergeCell ref="Q29:Q35"/>
+    <mergeCell ref="A31:Q31"/>
+    <mergeCell ref="H22:N22"/>
+    <mergeCell ref="A12:A18"/>
+    <mergeCell ref="Q22:Q28"/>
+    <mergeCell ref="C42:G42"/>
+    <mergeCell ref="H12:N12"/>
     <mergeCell ref="A2:A8"/>
-    <mergeCell ref="A20:A26"/>
+    <mergeCell ref="A11:Q11"/>
+    <mergeCell ref="A51:Q51"/>
+    <mergeCell ref="H42:N42"/>
     <mergeCell ref="Q2:Q8"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="Q11:Q17"/>
-    <mergeCell ref="C29:G29"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="B35:N35"/>
-    <mergeCell ref="C47:G47"/>
-    <mergeCell ref="B26:N26"/>
-    <mergeCell ref="A29:A35"/>
-    <mergeCell ref="A47:A53"/>
-    <mergeCell ref="H29:N29"/>
-    <mergeCell ref="A38:A44"/>
-    <mergeCell ref="H20:N20"/>
-    <mergeCell ref="H38:N38"/>
-    <mergeCell ref="A37:Q37"/>
-    <mergeCell ref="A46:Q46"/>
+    <mergeCell ref="A32:A38"/>
+    <mergeCell ref="A22:A28"/>
+    <mergeCell ref="A42:A48"/>
+    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="A41:Q41"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="A52:A58"/>
+    <mergeCell ref="A21:Q21"/>
     <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="Q47:Q53"/>
-    <mergeCell ref="O47:P47"/>
-    <mergeCell ref="A11:A17"/>
+    <mergeCell ref="B18:N18"/>
+    <mergeCell ref="B58:N58"/>
+    <mergeCell ref="Q32:Q38"/>
+    <mergeCell ref="Q12:Q18"/>
+    <mergeCell ref="O42:P42"/>
+    <mergeCell ref="B48:N48"/>
+    <mergeCell ref="C52:G52"/>
+    <mergeCell ref="O12:P12"/>
+    <mergeCell ref="O52:P52"/>
     <mergeCell ref="O2:P2"/>
-    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="Q52:Q58"/>
+    <mergeCell ref="C32:G32"/>
     <mergeCell ref="B8:N8"/>
-    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="H52:N52"/>
     <mergeCell ref="H2:N2"/>
-    <mergeCell ref="B17:N17"/>
-    <mergeCell ref="O38:P38"/>
-    <mergeCell ref="H11:N11"/>
-    <mergeCell ref="B44:N44"/>
-    <mergeCell ref="A10:Q10"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="Q20:Q26"/>
-    <mergeCell ref="B53:N53"/>
-    <mergeCell ref="A19:Q19"/>
+    <mergeCell ref="Q42:Q48"/>
+    <mergeCell ref="H32:N32"/>
+    <mergeCell ref="B38:N38"/>
+    <mergeCell ref="B28:N28"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>

</xml_diff>